<commit_message>
chrna1 chrne data entries
</commit_message>
<xml_diff>
--- a/HK Zeiterfassung 2026.xlsx
+++ b/HK Zeiterfassung 2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harik\Downloads\Computational Chemistry\Variant-Effect-Predictor-for-nAChRs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71516F91-5112-481D-B195-F5DE457932EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{129C1F3E-4864-4E53-98AE-F7F02CFF60FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2295" yWindow="2295" windowWidth="26850" windowHeight="13530" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Januar " sheetId="26" r:id="rId1"/>
@@ -2489,6 +2489,46 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="17" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="17" fontId="0" fillId="3" borderId="17" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -2551,61 +2591,6 @@
       <alignment horizontal="right"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="3" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="17" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="17" fontId="0" fillId="3" borderId="17" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2628,6 +2613,21 @@
     <xf numFmtId="166" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2923,98 +2923,98 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="60" t="s">
+      <c r="A1" s="70" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="62"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="72"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="65" t="s">
+      <c r="A2" s="73" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="74"/>
+      <c r="C2" s="75" t="s">
         <v>408</v>
       </c>
-      <c r="D2" s="65"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="67" t="s">
+      <c r="D2" s="75"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="64"/>
+      <c r="G2" s="74"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="68" t="s">
+      <c r="I2" s="78" t="s">
         <v>407</v>
       </c>
-      <c r="J2" s="69"/>
+      <c r="J2" s="79"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="54" t="s">
+      <c r="B3" s="63"/>
+      <c r="C3" s="64" t="s">
         <v>408</v>
       </c>
-      <c r="D3" s="54"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="56" t="s">
+      <c r="D3" s="64"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="57"/>
+      <c r="G3" s="67"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="58">
+      <c r="I3" s="68">
         <v>2026</v>
       </c>
-      <c r="J3" s="59"/>
+      <c r="J3" s="69"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="70" t="s">
+      <c r="C4" s="52" t="s">
         <v>408</v>
       </c>
-      <c r="D4" s="70"/>
-      <c r="E4" s="71"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="53"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="72" t="s">
+      <c r="I4" s="54" t="s">
         <v>408</v>
       </c>
-      <c r="J4" s="73"/>
+      <c r="J4" s="55"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="74" t="s">
+      <c r="C5" s="56" t="s">
         <v>408</v>
       </c>
-      <c r="D5" s="74"/>
-      <c r="E5" s="75"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="57"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="76" t="s">
+      <c r="I5" s="58" t="s">
         <v>409</v>
       </c>
-      <c r="J5" s="77"/>
+      <c r="J5" s="59"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -3027,10 +3027,10 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="78" t="s">
+      <c r="I6" s="60" t="s">
         <v>409</v>
       </c>
-      <c r="J6" s="79"/>
+      <c r="J6" s="61"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -3819,11 +3819,6 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -3833,6 +3828,11 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -3863,104 +3863,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="60" t="s">
+      <c r="A1" s="70" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="62"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="72"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="65" t="str">
+      <c r="A2" s="73" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="74"/>
+      <c r="C2" s="75" t="str">
         <f>September!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="65"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="67" t="s">
+      <c r="D2" s="75"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="64"/>
+      <c r="G2" s="74"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="68" t="s">
+      <c r="I2" s="78" t="s">
         <v>311</v>
       </c>
-      <c r="J2" s="69"/>
+      <c r="J2" s="79"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="54" t="str">
+      <c r="B3" s="63"/>
+      <c r="C3" s="64" t="str">
         <f>September!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="54"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="56" t="s">
+      <c r="D3" s="64"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="57"/>
+      <c r="G3" s="67"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="58">
+      <c r="I3" s="68">
         <v>2026</v>
       </c>
-      <c r="J3" s="59"/>
+      <c r="J3" s="69"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="70" t="str">
+      <c r="C4" s="52" t="str">
         <f>September!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="70"/>
-      <c r="E4" s="71"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="53"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="72" t="str">
+      <c r="I4" s="54" t="str">
         <f>September!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="73"/>
+      <c r="J4" s="55"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="74" t="str">
+      <c r="C5" s="56" t="str">
         <f>September!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="74"/>
-      <c r="E5" s="75"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="57"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="76">
+      <c r="I5" s="58">
         <f>September!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="77"/>
+      <c r="J5" s="59"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -3973,11 +3973,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="78" t="str">
+      <c r="I6" s="60" t="str">
         <f>September!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="79"/>
+      <c r="J6" s="61"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -4734,7 +4734,7 @@
       <c r="F43" s="1"/>
       <c r="H43" s="34">
         <f>September!H43</f>
-        <v>0.68750000000000011</v>
+        <v>0.82638888888888895</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -4749,7 +4749,7 @@
       <c r="G44" s="15"/>
       <c r="H44" s="38">
         <f>H42-H41+H43</f>
-        <v>0.68750000000000011</v>
+        <v>0.82638888888888895</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
@@ -4767,11 +4767,6 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -4781,6 +4776,11 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -4811,104 +4811,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="60" t="s">
+      <c r="A1" s="70" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="62"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="72"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="65" t="str">
+      <c r="A2" s="73" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="74"/>
+      <c r="C2" s="75" t="str">
         <f>'Oktober '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="65"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="67" t="s">
+      <c r="D2" s="75"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="64"/>
+      <c r="G2" s="74"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="68" t="s">
+      <c r="I2" s="78" t="s">
         <v>343</v>
       </c>
-      <c r="J2" s="69"/>
+      <c r="J2" s="79"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="54" t="str">
+      <c r="B3" s="63"/>
+      <c r="C3" s="64" t="str">
         <f>'Oktober '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="54"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="56" t="s">
+      <c r="D3" s="64"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="57"/>
+      <c r="G3" s="67"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="58">
+      <c r="I3" s="68">
         <v>2026</v>
       </c>
-      <c r="J3" s="59"/>
+      <c r="J3" s="69"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="70" t="str">
+      <c r="C4" s="52" t="str">
         <f>'Oktober '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="70"/>
-      <c r="E4" s="71"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="53"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="72" t="str">
+      <c r="I4" s="54" t="str">
         <f>'Oktober '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="73"/>
+      <c r="J4" s="55"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="74" t="str">
+      <c r="C5" s="56" t="str">
         <f>'Oktober '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="74"/>
-      <c r="E5" s="75"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="57"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="76">
+      <c r="I5" s="58">
         <f>'Oktober '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="77"/>
+      <c r="J5" s="59"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -4921,11 +4921,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="78" t="str">
+      <c r="I6" s="60" t="str">
         <f>'Oktober '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="79"/>
+      <c r="J6" s="61"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -5661,7 +5661,7 @@
       <c r="F42" s="1"/>
       <c r="H42" s="34">
         <f>'Oktober '!H44</f>
-        <v>0.68750000000000011</v>
+        <v>0.82638888888888895</v>
       </c>
     </row>
     <row r="43" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -5676,7 +5676,7 @@
       <c r="G43" s="15"/>
       <c r="H43" s="38">
         <f>H41-H40+H42</f>
-        <v>0.68750000000000011</v>
+        <v>0.82638888888888895</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
@@ -5694,11 +5694,6 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -5708,6 +5703,11 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -5738,104 +5738,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="60" t="s">
+      <c r="A1" s="70" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="62"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="72"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="65" t="str">
+      <c r="A2" s="73" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="74"/>
+      <c r="C2" s="75" t="str">
         <f>'November '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="65"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="67" t="s">
+      <c r="D2" s="75"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="64"/>
+      <c r="G2" s="74"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="68" t="s">
+      <c r="I2" s="78" t="s">
         <v>374</v>
       </c>
-      <c r="J2" s="69"/>
+      <c r="J2" s="79"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="54" t="str">
+      <c r="B3" s="63"/>
+      <c r="C3" s="64" t="str">
         <f>'November '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="54"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="56" t="s">
+      <c r="D3" s="64"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="57"/>
+      <c r="G3" s="67"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="58">
+      <c r="I3" s="68">
         <v>2026</v>
       </c>
-      <c r="J3" s="59"/>
+      <c r="J3" s="69"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="70" t="str">
+      <c r="C4" s="52" t="str">
         <f>'November '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="70"/>
-      <c r="E4" s="71"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="53"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="72" t="str">
+      <c r="I4" s="54" t="str">
         <f>'November '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="73"/>
+      <c r="J4" s="55"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="74" t="str">
+      <c r="C5" s="56" t="str">
         <f>'November '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="74"/>
-      <c r="E5" s="75"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="57"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="76">
+      <c r="I5" s="58">
         <f>'November '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="77"/>
+      <c r="J5" s="59"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -5848,11 +5848,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="78" t="str">
+      <c r="I6" s="60" t="str">
         <f>'November '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="79"/>
+      <c r="J6" s="61"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -6609,7 +6609,7 @@
       <c r="F43" s="1"/>
       <c r="H43" s="34">
         <f>'November '!H43</f>
-        <v>0.68750000000000011</v>
+        <v>0.82638888888888895</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -6624,7 +6624,7 @@
       <c r="G44" s="15"/>
       <c r="H44" s="38">
         <f>H42-H41+H43</f>
-        <v>0.68750000000000011</v>
+        <v>0.82638888888888895</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
@@ -6642,11 +6642,6 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -6656,6 +6651,11 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -6687,22 +6687,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="85" t="s">
+      <c r="A1" s="80" t="s">
         <v>416</v>
       </c>
-      <c r="B1" s="86"/>
-      <c r="C1" s="86"/>
-      <c r="D1" s="86"/>
-      <c r="E1" s="86"/>
-      <c r="F1" s="86"/>
-      <c r="G1" s="86"/>
-      <c r="H1" s="87"/>
+      <c r="B1" s="81"/>
+      <c r="C1" s="81"/>
+      <c r="D1" s="81"/>
+      <c r="E1" s="81"/>
+      <c r="F1" s="81"/>
+      <c r="G1" s="81"/>
+      <c r="H1" s="82"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="52" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="53"/>
+      <c r="A2" s="62" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="63"/>
       <c r="C2" s="47" t="str">
         <f>'November '!C2:E2</f>
         <v>Hari Krishna</v>
@@ -6711,15 +6711,15 @@
       <c r="E2" s="22" t="s">
         <v>418</v>
       </c>
-      <c r="F2" s="91"/>
-      <c r="G2" s="91"/>
+      <c r="F2" s="86"/>
+      <c r="G2" s="86"/>
       <c r="H2" s="48"/>
     </row>
     <row r="3" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="82" t="s">
+      <c r="A3" s="89" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="57"/>
+      <c r="B3" s="67"/>
       <c r="C3" s="49" t="str">
         <f>'November '!C3:E3</f>
         <v>Mohan Raj</v>
@@ -6728,8 +6728,8 @@
       <c r="E3" s="18" t="s">
         <v>122</v>
       </c>
-      <c r="F3" s="58"/>
-      <c r="G3" s="58"/>
+      <c r="F3" s="68"/>
+      <c r="G3" s="68"/>
       <c r="H3" s="50"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
@@ -6743,17 +6743,17 @@
       </c>
     </row>
     <row r="6" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="89" t="s">
+      <c r="A6" s="84" t="s">
         <v>417</v>
       </c>
-      <c r="B6" s="90"/>
-      <c r="C6" s="88" t="s">
+      <c r="B6" s="85"/>
+      <c r="C6" s="83" t="s">
         <v>419</v>
       </c>
-      <c r="D6" s="88"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="88"/>
-      <c r="G6" s="88"/>
+      <c r="D6" s="83"/>
+      <c r="E6" s="83"/>
+      <c r="F6" s="83"/>
+      <c r="G6" s="83"/>
       <c r="H6" s="51"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
@@ -6765,10 +6765,10 @@
       <c r="D8" s="3"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A9" s="80" t="s">
+      <c r="A9" s="87" t="s">
         <v>410</v>
       </c>
-      <c r="B9" s="81"/>
+      <c r="B9" s="88"/>
       <c r="C9" s="44" t="s">
         <v>411</v>
       </c>
@@ -6784,10 +6784,10 @@
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A10" s="83" t="s">
+      <c r="A10" s="90" t="s">
         <v>407</v>
       </c>
-      <c r="B10" s="84"/>
+      <c r="B10" s="91"/>
       <c r="C10" s="46">
         <f>'Januar '!H41</f>
         <v>0</v>
@@ -6806,10 +6806,10 @@
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A11" s="83" t="s">
+      <c r="A11" s="90" t="s">
         <v>406</v>
       </c>
-      <c r="B11" s="84"/>
+      <c r="B11" s="91"/>
       <c r="C11" s="46">
         <f>'Februar '!H39</f>
         <v>0</v>
@@ -6829,17 +6829,17 @@
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A12" s="83" t="s">
+      <c r="A12" s="90" t="s">
         <v>89</v>
       </c>
-      <c r="B12" s="84"/>
+      <c r="B12" s="91"/>
       <c r="C12" s="46">
         <f>'März '!H41</f>
         <v>0</v>
       </c>
       <c r="D12" s="46">
         <f>'März '!H42</f>
-        <v>0.68750000000000011</v>
+        <v>0.82638888888888895</v>
       </c>
       <c r="E12" s="46">
         <f>'März '!H43</f>
@@ -6848,15 +6848,15 @@
       <c r="F12" s="46"/>
       <c r="G12" s="46">
         <f>'März '!H44</f>
-        <v>0.68750000000000011</v>
+        <v>0.82638888888888895</v>
       </c>
       <c r="M12" s="28"/>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A13" s="83" t="s">
+      <c r="A13" s="90" t="s">
         <v>121</v>
       </c>
-      <c r="B13" s="84"/>
+      <c r="B13" s="91"/>
       <c r="C13" s="46">
         <f>'April '!H40</f>
         <v>0</v>
@@ -6867,19 +6867,19 @@
       </c>
       <c r="E13" s="46">
         <f>'April '!H42</f>
-        <v>0.68750000000000011</v>
+        <v>0.82638888888888895</v>
       </c>
       <c r="F13" s="46"/>
       <c r="G13" s="46">
         <f>'April '!H43</f>
-        <v>0.68750000000000011</v>
+        <v>0.82638888888888895</v>
       </c>
     </row>
     <row r="14" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="83" t="s">
+      <c r="A14" s="90" t="s">
         <v>185</v>
       </c>
-      <c r="B14" s="84"/>
+      <c r="B14" s="91"/>
       <c r="C14" s="46">
         <f>'Mai '!H41</f>
         <v>0</v>
@@ -6890,19 +6890,19 @@
       </c>
       <c r="E14" s="46">
         <f>'Mai '!H43</f>
-        <v>0.68750000000000011</v>
+        <v>0.82638888888888895</v>
       </c>
       <c r="F14" s="46"/>
       <c r="G14" s="46">
         <f>'Mai '!H44</f>
-        <v>0.68750000000000011</v>
+        <v>0.82638888888888895</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A15" s="83" t="s">
+      <c r="A15" s="90" t="s">
         <v>184</v>
       </c>
-      <c r="B15" s="84"/>
+      <c r="B15" s="91"/>
       <c r="C15" s="46">
         <f>'Juni '!H40</f>
         <v>0</v>
@@ -6913,19 +6913,19 @@
       </c>
       <c r="E15" s="46">
         <f>'Juni '!H42</f>
-        <v>0.68750000000000011</v>
+        <v>0.82638888888888895</v>
       </c>
       <c r="F15" s="46"/>
       <c r="G15" s="46">
         <f>'Juni '!H43</f>
-        <v>0.68750000000000011</v>
+        <v>0.82638888888888895</v>
       </c>
     </row>
     <row r="16" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="83" t="s">
+      <c r="A16" s="90" t="s">
         <v>247</v>
       </c>
-      <c r="B16" s="84"/>
+      <c r="B16" s="91"/>
       <c r="C16" s="46">
         <f>'Juli '!H41</f>
         <v>0</v>
@@ -6936,19 +6936,19 @@
       </c>
       <c r="E16" s="46">
         <f>'Juli '!H43</f>
-        <v>0.68750000000000011</v>
+        <v>0.82638888888888895</v>
       </c>
       <c r="F16" s="46"/>
       <c r="G16" s="46">
         <f>'Juli '!H44</f>
-        <v>0.68750000000000011</v>
+        <v>0.82638888888888895</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="83" t="s">
+      <c r="A17" s="90" t="s">
         <v>248</v>
       </c>
-      <c r="B17" s="84"/>
+      <c r="B17" s="91"/>
       <c r="C17" s="46">
         <f>'August '!H41</f>
         <v>0</v>
@@ -6959,19 +6959,19 @@
       </c>
       <c r="E17" s="46">
         <f>'August '!H43</f>
-        <v>0.68750000000000011</v>
+        <v>0.82638888888888895</v>
       </c>
       <c r="F17" s="46"/>
       <c r="G17" s="46">
         <f>'August '!H44</f>
-        <v>0.68750000000000011</v>
+        <v>0.82638888888888895</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="83" t="s">
+      <c r="A18" s="90" t="s">
         <v>280</v>
       </c>
-      <c r="B18" s="84"/>
+      <c r="B18" s="91"/>
       <c r="C18" s="46">
         <f>September!H40</f>
         <v>0</v>
@@ -6982,19 +6982,19 @@
       </c>
       <c r="E18" s="46">
         <f>September!H42</f>
-        <v>0.68750000000000011</v>
+        <v>0.82638888888888895</v>
       </c>
       <c r="F18" s="46"/>
       <c r="G18" s="46">
         <f>September!H43</f>
-        <v>0.68750000000000011</v>
+        <v>0.82638888888888895</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="83" t="s">
+      <c r="A19" s="90" t="s">
         <v>311</v>
       </c>
-      <c r="B19" s="84"/>
+      <c r="B19" s="91"/>
       <c r="C19" s="46">
         <f>'Oktober '!H41</f>
         <v>0</v>
@@ -7005,19 +7005,19 @@
       </c>
       <c r="E19" s="46">
         <f>'Oktober '!H43</f>
-        <v>0.68750000000000011</v>
+        <v>0.82638888888888895</v>
       </c>
       <c r="F19" s="46"/>
       <c r="G19" s="46">
         <f>'Oktober '!H44</f>
-        <v>0.68750000000000011</v>
+        <v>0.82638888888888895</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="83" t="s">
+      <c r="A20" s="90" t="s">
         <v>343</v>
       </c>
-      <c r="B20" s="84"/>
+      <c r="B20" s="91"/>
       <c r="C20" s="46">
         <f>'November '!H40</f>
         <v>0</v>
@@ -7028,19 +7028,19 @@
       </c>
       <c r="E20" s="46">
         <f>'November '!H42</f>
-        <v>0.68750000000000011</v>
+        <v>0.82638888888888895</v>
       </c>
       <c r="F20" s="46"/>
       <c r="G20" s="46">
         <f>'November '!H43</f>
-        <v>0.68750000000000011</v>
+        <v>0.82638888888888895</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="83" t="s">
+      <c r="A21" s="90" t="s">
         <v>374</v>
       </c>
-      <c r="B21" s="84"/>
+      <c r="B21" s="91"/>
       <c r="C21" s="46">
         <f>'Dezember '!H41</f>
         <v>0</v>
@@ -7051,12 +7051,12 @@
       </c>
       <c r="E21" s="46">
         <f>'Dezember '!H43</f>
-        <v>0.68750000000000011</v>
+        <v>0.82638888888888895</v>
       </c>
       <c r="F21" s="46"/>
       <c r="G21" s="46">
         <f>'Dezember '!H44</f>
-        <v>0.68750000000000011</v>
+        <v>0.82638888888888895</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
@@ -7093,11 +7093,6 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="20">
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="C6:G6"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="F3:G3"/>
     <mergeCell ref="A9:B9"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A3:B3"/>
@@ -7113,6 +7108,11 @@
     <mergeCell ref="A17:B17"/>
     <mergeCell ref="A18:B18"/>
     <mergeCell ref="A19:B19"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="C6:G6"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="F3:G3"/>
   </mergeCells>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.39370078740157483" bottom="0.39370078740157483" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -7135,104 +7135,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="60" t="s">
+      <c r="A1" s="70" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="62"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="72"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="65" t="str">
+      <c r="A2" s="73" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="74"/>
+      <c r="C2" s="75" t="str">
         <f>'Januar '!C2:E2</f>
         <v>XXX</v>
       </c>
-      <c r="D2" s="65"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="67" t="s">
+      <c r="D2" s="75"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="64"/>
+      <c r="G2" s="74"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="68" t="s">
+      <c r="I2" s="78" t="s">
         <v>406</v>
       </c>
-      <c r="J2" s="69"/>
+      <c r="J2" s="79"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="54" t="str">
+      <c r="B3" s="63"/>
+      <c r="C3" s="64" t="str">
         <f>'Januar '!C3:E3</f>
         <v>XXX</v>
       </c>
-      <c r="D3" s="54"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="56" t="s">
+      <c r="D3" s="64"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="57"/>
+      <c r="G3" s="67"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="58">
+      <c r="I3" s="68">
         <v>2026</v>
       </c>
-      <c r="J3" s="59"/>
+      <c r="J3" s="69"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="70" t="str">
+      <c r="C4" s="52" t="str">
         <f>'Januar '!C4:E4</f>
         <v>XXX</v>
       </c>
-      <c r="D4" s="70"/>
-      <c r="E4" s="71"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="53"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="72" t="str">
+      <c r="I4" s="54" t="str">
         <f>'Januar '!I4:J4</f>
         <v>XXX</v>
       </c>
-      <c r="J4" s="73"/>
+      <c r="J4" s="55"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="74" t="str">
+      <c r="C5" s="56" t="str">
         <f>'Januar '!C5:E5</f>
         <v>XXX</v>
       </c>
-      <c r="D5" s="74"/>
-      <c r="E5" s="75"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="57"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="76" t="str">
+      <c r="I5" s="58" t="str">
         <f>'Januar '!I5:J5</f>
         <v>XX</v>
       </c>
-      <c r="J5" s="77"/>
+      <c r="J5" s="59"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -7245,11 +7245,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="78" t="str">
+      <c r="I6" s="60" t="str">
         <f>'Januar '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="79"/>
+      <c r="J6" s="61"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -7985,11 +7985,6 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -7999,6 +7994,11 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -8029,98 +8029,98 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="60" t="s">
+      <c r="A1" s="70" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="62"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="72"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="65" t="s">
+      <c r="A2" s="73" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="74"/>
+      <c r="C2" s="75" t="s">
         <v>420</v>
       </c>
-      <c r="D2" s="65"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="67" t="s">
+      <c r="D2" s="75"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="64"/>
+      <c r="G2" s="74"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="68" t="s">
+      <c r="I2" s="78" t="s">
         <v>89</v>
       </c>
-      <c r="J2" s="69"/>
+      <c r="J2" s="79"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="54" t="s">
+      <c r="B3" s="63"/>
+      <c r="C3" s="64" t="s">
         <v>421</v>
       </c>
-      <c r="D3" s="54"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="56" t="s">
+      <c r="D3" s="64"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="57"/>
+      <c r="G3" s="67"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="58">
+      <c r="I3" s="68">
         <v>2026</v>
       </c>
-      <c r="J3" s="59"/>
+      <c r="J3" s="69"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="70" t="s">
+      <c r="C4" s="52" t="s">
         <v>422</v>
       </c>
-      <c r="D4" s="70"/>
-      <c r="E4" s="71"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="53"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="72" t="s">
+      <c r="I4" s="54" t="s">
         <v>424</v>
       </c>
-      <c r="J4" s="73"/>
+      <c r="J4" s="55"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="74" t="s">
+      <c r="C5" s="56" t="s">
         <v>423</v>
       </c>
-      <c r="D5" s="74"/>
-      <c r="E5" s="75"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="57"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="76">
+      <c r="I5" s="58">
         <v>8</v>
       </c>
-      <c r="J5" s="77"/>
+      <c r="J5" s="59"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -8133,11 +8133,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="78" t="str">
+      <c r="I6" s="60" t="str">
         <f>'Februar '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="79"/>
+      <c r="J6" s="61"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -8587,16 +8587,22 @@
         <v>14</v>
       </c>
       <c r="C26" s="32"/>
-      <c r="D26" s="29"/>
-      <c r="E26" s="29"/>
-      <c r="F26" s="29"/>
+      <c r="D26" s="29">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="E26" s="29">
+        <v>0.75</v>
+      </c>
+      <c r="F26" s="29">
+        <v>2.7777777777777776E-2</v>
+      </c>
       <c r="G26" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.13888888888888884</v>
       </c>
       <c r="H26" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.13888888888888884</v>
       </c>
       <c r="I26" s="30"/>
       <c r="J26" s="31"/>
@@ -8913,7 +8919,7 @@
       <c r="F42" s="1"/>
       <c r="H42" s="34">
         <f>SUM(H9:H39)</f>
-        <v>0.68750000000000011</v>
+        <v>0.82638888888888895</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
@@ -8939,7 +8945,7 @@
       <c r="G44" s="15"/>
       <c r="H44" s="38">
         <f>H42-H41+H43</f>
-        <v>0.68750000000000011</v>
+        <v>0.82638888888888895</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
@@ -8952,11 +8958,6 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -8966,6 +8967,11 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -8996,104 +9002,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="60" t="s">
+      <c r="A1" s="70" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="62"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="72"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="65" t="str">
+      <c r="A2" s="73" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="74"/>
+      <c r="C2" s="75" t="str">
         <f>'März '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="65"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="67" t="s">
+      <c r="D2" s="75"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="64"/>
+      <c r="G2" s="74"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="68" t="s">
+      <c r="I2" s="78" t="s">
         <v>121</v>
       </c>
-      <c r="J2" s="69"/>
+      <c r="J2" s="79"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="54" t="str">
+      <c r="B3" s="63"/>
+      <c r="C3" s="64" t="str">
         <f>'März '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="54"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="56" t="s">
+      <c r="D3" s="64"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="57"/>
+      <c r="G3" s="67"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="58">
+      <c r="I3" s="68">
         <v>2026</v>
       </c>
-      <c r="J3" s="59"/>
+      <c r="J3" s="69"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="70" t="str">
+      <c r="C4" s="52" t="str">
         <f>'März '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="70"/>
-      <c r="E4" s="71"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="53"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="72" t="str">
+      <c r="I4" s="54" t="str">
         <f>'März '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="73"/>
+      <c r="J4" s="55"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="74" t="str">
+      <c r="C5" s="56" t="str">
         <f>'März '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="74"/>
-      <c r="E5" s="75"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="57"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="76">
+      <c r="I5" s="58">
         <f>'März '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="77"/>
+      <c r="J5" s="59"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -9106,11 +9112,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="78" t="str">
+      <c r="I6" s="60" t="str">
         <f>'März '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="79"/>
+      <c r="J6" s="61"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -9845,7 +9851,7 @@
       <c r="F42" s="1"/>
       <c r="H42" s="34">
         <f>'März '!H44</f>
-        <v>0.68750000000000011</v>
+        <v>0.82638888888888895</v>
       </c>
     </row>
     <row r="43" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -9860,7 +9866,7 @@
       <c r="G43" s="15"/>
       <c r="H43" s="38">
         <f>H41-H40+H42</f>
-        <v>0.68750000000000011</v>
+        <v>0.82638888888888895</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
@@ -9878,11 +9884,6 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -9892,6 +9893,11 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -9922,104 +9928,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="60" t="s">
+      <c r="A1" s="70" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="62"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="72"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="65" t="str">
+      <c r="A2" s="73" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="74"/>
+      <c r="C2" s="75" t="str">
         <f>'April '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="65"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="67" t="s">
+      <c r="D2" s="75"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="64"/>
+      <c r="G2" s="74"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="68" t="s">
+      <c r="I2" s="78" t="s">
         <v>185</v>
       </c>
-      <c r="J2" s="69"/>
+      <c r="J2" s="79"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="54" t="str">
+      <c r="B3" s="63"/>
+      <c r="C3" s="64" t="str">
         <f>'April '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="54"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="56" t="s">
+      <c r="D3" s="64"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="57"/>
+      <c r="G3" s="67"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="58">
+      <c r="I3" s="68">
         <v>2026</v>
       </c>
-      <c r="J3" s="59"/>
+      <c r="J3" s="69"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="70" t="str">
+      <c r="C4" s="52" t="str">
         <f>'April '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="70"/>
-      <c r="E4" s="71"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="53"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="72" t="str">
+      <c r="I4" s="54" t="str">
         <f>'April '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="73"/>
+      <c r="J4" s="55"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="74" t="str">
+      <c r="C5" s="56" t="str">
         <f>'April '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="74"/>
-      <c r="E5" s="75"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="57"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="76">
+      <c r="I5" s="58">
         <f>'April '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="77"/>
+      <c r="J5" s="59"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -10032,11 +10038,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="78" t="str">
+      <c r="I6" s="60" t="str">
         <f>'April '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="79"/>
+      <c r="J6" s="61"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -10793,7 +10799,7 @@
       <c r="F43" s="1"/>
       <c r="H43" s="34">
         <f>'April '!H43</f>
-        <v>0.68750000000000011</v>
+        <v>0.82638888888888895</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -10808,7 +10814,7 @@
       <c r="G44" s="15"/>
       <c r="H44" s="38">
         <f>H42-H41+H43</f>
-        <v>0.68750000000000011</v>
+        <v>0.82638888888888895</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
@@ -10826,11 +10832,6 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -10840,6 +10841,11 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -10870,104 +10876,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="60" t="s">
+      <c r="A1" s="70" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="62"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="72"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="65" t="str">
+      <c r="A2" s="73" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="74"/>
+      <c r="C2" s="75" t="str">
         <f>'Mai '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="65"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="67" t="s">
+      <c r="D2" s="75"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="64"/>
+      <c r="G2" s="74"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="68" t="s">
+      <c r="I2" s="78" t="s">
         <v>184</v>
       </c>
-      <c r="J2" s="69"/>
+      <c r="J2" s="79"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="54" t="str">
+      <c r="B3" s="63"/>
+      <c r="C3" s="64" t="str">
         <f>'Mai '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="54"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="56" t="s">
+      <c r="D3" s="64"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="57"/>
+      <c r="G3" s="67"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="58">
+      <c r="I3" s="68">
         <v>2026</v>
       </c>
-      <c r="J3" s="59"/>
+      <c r="J3" s="69"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="70" t="str">
+      <c r="C4" s="52" t="str">
         <f>'Mai '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="70"/>
-      <c r="E4" s="71"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="53"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="72" t="str">
+      <c r="I4" s="54" t="str">
         <f>'Mai '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="73"/>
+      <c r="J4" s="55"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="74" t="str">
+      <c r="C5" s="56" t="str">
         <f>'Mai '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="74"/>
-      <c r="E5" s="75"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="57"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="76">
+      <c r="I5" s="58">
         <f>'Mai '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="77"/>
+      <c r="J5" s="59"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -10980,11 +10986,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="78" t="str">
+      <c r="I6" s="60" t="str">
         <f>'Mai '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="79"/>
+      <c r="J6" s="61"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -11719,7 +11725,7 @@
       <c r="F42" s="1"/>
       <c r="H42" s="34">
         <f>'Mai '!H44</f>
-        <v>0.68750000000000011</v>
+        <v>0.82638888888888895</v>
       </c>
     </row>
     <row r="43" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -11734,7 +11740,7 @@
       <c r="G43" s="15"/>
       <c r="H43" s="38">
         <f>H41-H40+H42</f>
-        <v>0.68750000000000011</v>
+        <v>0.82638888888888895</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
@@ -11752,11 +11758,6 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -11766,6 +11767,11 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -11796,104 +11802,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="60" t="s">
+      <c r="A1" s="70" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="62"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="72"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="65" t="str">
+      <c r="A2" s="73" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="74"/>
+      <c r="C2" s="75" t="str">
         <f>'Juni '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="65"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="67" t="s">
+      <c r="D2" s="75"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="64"/>
+      <c r="G2" s="74"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="68" t="s">
+      <c r="I2" s="78" t="s">
         <v>247</v>
       </c>
-      <c r="J2" s="69"/>
+      <c r="J2" s="79"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="54" t="str">
+      <c r="B3" s="63"/>
+      <c r="C3" s="64" t="str">
         <f>'Juni '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="54"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="56" t="s">
+      <c r="D3" s="64"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="57"/>
+      <c r="G3" s="67"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="58">
+      <c r="I3" s="68">
         <v>2026</v>
       </c>
-      <c r="J3" s="59"/>
+      <c r="J3" s="69"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="70" t="str">
+      <c r="C4" s="52" t="str">
         <f>'Juni '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="70"/>
-      <c r="E4" s="71"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="53"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="72" t="str">
+      <c r="I4" s="54" t="str">
         <f>'Juni '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="73"/>
+      <c r="J4" s="55"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="74" t="str">
+      <c r="C5" s="56" t="str">
         <f>'Juni '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="74"/>
-      <c r="E5" s="75"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="57"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="76">
+      <c r="I5" s="58">
         <f>'Juni '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="77"/>
+      <c r="J5" s="59"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -11906,11 +11912,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="78" t="str">
+      <c r="I6" s="60" t="str">
         <f>'Juni '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="79"/>
+      <c r="J6" s="61"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -12667,7 +12673,7 @@
       <c r="F43" s="1"/>
       <c r="H43" s="34">
         <f>'Juni '!H43</f>
-        <v>0.68750000000000011</v>
+        <v>0.82638888888888895</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -12682,7 +12688,7 @@
       <c r="G44" s="15"/>
       <c r="H44" s="38">
         <f>H42-H41+H43</f>
-        <v>0.68750000000000011</v>
+        <v>0.82638888888888895</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
@@ -12700,11 +12706,6 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -12714,6 +12715,11 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -12744,104 +12750,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="60" t="s">
+      <c r="A1" s="70" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="62"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="72"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="65" t="str">
+      <c r="A2" s="73" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="74"/>
+      <c r="C2" s="75" t="str">
         <f>'Juli '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="65"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="67" t="s">
+      <c r="D2" s="75"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="64"/>
+      <c r="G2" s="74"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="68" t="s">
+      <c r="I2" s="78" t="s">
         <v>248</v>
       </c>
-      <c r="J2" s="69"/>
+      <c r="J2" s="79"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="54" t="str">
+      <c r="B3" s="63"/>
+      <c r="C3" s="64" t="str">
         <f>'Juli '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="54"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="56" t="s">
+      <c r="D3" s="64"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="57"/>
+      <c r="G3" s="67"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="58">
+      <c r="I3" s="68">
         <v>2026</v>
       </c>
-      <c r="J3" s="59"/>
+      <c r="J3" s="69"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="70" t="str">
+      <c r="C4" s="52" t="str">
         <f>'Juli '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="70"/>
-      <c r="E4" s="71"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="53"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="72" t="str">
+      <c r="I4" s="54" t="str">
         <f>'Juli '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="73"/>
+      <c r="J4" s="55"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="74" t="str">
+      <c r="C5" s="56" t="str">
         <f>'Juli '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="74"/>
-      <c r="E5" s="75"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="57"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="76">
+      <c r="I5" s="58">
         <f>'Juli '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="77"/>
+      <c r="J5" s="59"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -12854,11 +12860,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="78" t="str">
+      <c r="I6" s="60" t="str">
         <f>'Juli '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="79"/>
+      <c r="J6" s="61"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -13615,7 +13621,7 @@
       <c r="F43" s="1"/>
       <c r="H43" s="34">
         <f>'Juli '!H44</f>
-        <v>0.68750000000000011</v>
+        <v>0.82638888888888895</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -13630,7 +13636,7 @@
       <c r="G44" s="15"/>
       <c r="H44" s="38">
         <f>H42-H41+H43</f>
-        <v>0.68750000000000011</v>
+        <v>0.82638888888888895</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
@@ -13648,11 +13654,6 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -13662,6 +13663,11 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -13692,104 +13698,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="60" t="s">
+      <c r="A1" s="70" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="62"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="72"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="65" t="str">
+      <c r="A2" s="73" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="74"/>
+      <c r="C2" s="75" t="str">
         <f>'August '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="65"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="67" t="s">
+      <c r="D2" s="75"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="64"/>
+      <c r="G2" s="74"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="68" t="s">
+      <c r="I2" s="78" t="s">
         <v>280</v>
       </c>
-      <c r="J2" s="69"/>
+      <c r="J2" s="79"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="54" t="str">
+      <c r="B3" s="63"/>
+      <c r="C3" s="64" t="str">
         <f>'August '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="54"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="56" t="s">
+      <c r="D3" s="64"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="57"/>
+      <c r="G3" s="67"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="58">
+      <c r="I3" s="68">
         <v>2026</v>
       </c>
-      <c r="J3" s="59"/>
+      <c r="J3" s="69"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="70" t="str">
+      <c r="C4" s="52" t="str">
         <f>'August '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="70"/>
-      <c r="E4" s="71"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="53"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="72" t="str">
+      <c r="I4" s="54" t="str">
         <f>'August '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="73"/>
+      <c r="J4" s="55"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="74" t="str">
+      <c r="C5" s="56" t="str">
         <f>'August '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="74"/>
-      <c r="E5" s="75"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="57"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="76">
+      <c r="I5" s="58">
         <f>'August '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="77"/>
+      <c r="J5" s="59"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -13802,11 +13808,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="78" t="str">
+      <c r="I6" s="60" t="str">
         <f>'August '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="79"/>
+      <c r="J6" s="61"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -14541,7 +14547,7 @@
       <c r="F42" s="1"/>
       <c r="H42" s="34">
         <f>'August '!H44</f>
-        <v>0.68750000000000011</v>
+        <v>0.82638888888888895</v>
       </c>
     </row>
     <row r="43" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -14556,7 +14562,7 @@
       <c r="G43" s="15"/>
       <c r="H43" s="38">
         <f>H41-H40+H42</f>
-        <v>0.68750000000000011</v>
+        <v>0.82638888888888895</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
@@ -14574,11 +14580,6 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -14588,6 +14589,11 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">

</xml_diff>

<commit_message>
chrna2 chrna1 charna7 complete
</commit_message>
<xml_diff>
--- a/HK Zeiterfassung 2026.xlsx
+++ b/HK Zeiterfassung 2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harik\Downloads\Computational Chemistry\Variant-Effect-Predictor-for-nAChRs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{129C1F3E-4864-4E53-98AE-F7F02CFF60FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA5A6D29-0D38-4000-8834-6F10F64FDD1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3510" yWindow="3030" windowWidth="20295" windowHeight="10845" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Januar " sheetId="26" r:id="rId1"/>
@@ -4734,7 +4734,7 @@
       <c r="F43" s="1"/>
       <c r="H43" s="34">
         <f>September!H43</f>
-        <v>0.82638888888888895</v>
+        <v>1.125</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -4749,7 +4749,7 @@
       <c r="G44" s="15"/>
       <c r="H44" s="38">
         <f>H42-H41+H43</f>
-        <v>0.82638888888888895</v>
+        <v>1.125</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
@@ -5661,7 +5661,7 @@
       <c r="F42" s="1"/>
       <c r="H42" s="34">
         <f>'Oktober '!H44</f>
-        <v>0.82638888888888895</v>
+        <v>1.125</v>
       </c>
     </row>
     <row r="43" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -5676,7 +5676,7 @@
       <c r="G43" s="15"/>
       <c r="H43" s="38">
         <f>H41-H40+H42</f>
-        <v>0.82638888888888895</v>
+        <v>1.125</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
@@ -6609,7 +6609,7 @@
       <c r="F43" s="1"/>
       <c r="H43" s="34">
         <f>'November '!H43</f>
-        <v>0.82638888888888895</v>
+        <v>1.125</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -6624,7 +6624,7 @@
       <c r="G44" s="15"/>
       <c r="H44" s="38">
         <f>H42-H41+H43</f>
-        <v>0.82638888888888895</v>
+        <v>1.125</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
@@ -6839,7 +6839,7 @@
       </c>
       <c r="D12" s="46">
         <f>'März '!H42</f>
-        <v>0.82638888888888895</v>
+        <v>1.125</v>
       </c>
       <c r="E12" s="46">
         <f>'März '!H43</f>
@@ -6848,7 +6848,7 @@
       <c r="F12" s="46"/>
       <c r="G12" s="46">
         <f>'März '!H44</f>
-        <v>0.82638888888888895</v>
+        <v>1.125</v>
       </c>
       <c r="M12" s="28"/>
     </row>
@@ -6867,12 +6867,12 @@
       </c>
       <c r="E13" s="46">
         <f>'April '!H42</f>
-        <v>0.82638888888888895</v>
+        <v>1.125</v>
       </c>
       <c r="F13" s="46"/>
       <c r="G13" s="46">
         <f>'April '!H43</f>
-        <v>0.82638888888888895</v>
+        <v>1.125</v>
       </c>
     </row>
     <row r="14" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -6890,12 +6890,12 @@
       </c>
       <c r="E14" s="46">
         <f>'Mai '!H43</f>
-        <v>0.82638888888888895</v>
+        <v>1.125</v>
       </c>
       <c r="F14" s="46"/>
       <c r="G14" s="46">
         <f>'Mai '!H44</f>
-        <v>0.82638888888888895</v>
+        <v>1.125</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
@@ -6913,12 +6913,12 @@
       </c>
       <c r="E15" s="46">
         <f>'Juni '!H42</f>
-        <v>0.82638888888888895</v>
+        <v>1.125</v>
       </c>
       <c r="F15" s="46"/>
       <c r="G15" s="46">
         <f>'Juni '!H43</f>
-        <v>0.82638888888888895</v>
+        <v>1.125</v>
       </c>
     </row>
     <row r="16" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -6936,12 +6936,12 @@
       </c>
       <c r="E16" s="46">
         <f>'Juli '!H43</f>
-        <v>0.82638888888888895</v>
+        <v>1.125</v>
       </c>
       <c r="F16" s="46"/>
       <c r="G16" s="46">
         <f>'Juli '!H44</f>
-        <v>0.82638888888888895</v>
+        <v>1.125</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
@@ -6959,12 +6959,12 @@
       </c>
       <c r="E17" s="46">
         <f>'August '!H43</f>
-        <v>0.82638888888888895</v>
+        <v>1.125</v>
       </c>
       <c r="F17" s="46"/>
       <c r="G17" s="46">
         <f>'August '!H44</f>
-        <v>0.82638888888888895</v>
+        <v>1.125</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
@@ -6982,12 +6982,12 @@
       </c>
       <c r="E18" s="46">
         <f>September!H42</f>
-        <v>0.82638888888888895</v>
+        <v>1.125</v>
       </c>
       <c r="F18" s="46"/>
       <c r="G18" s="46">
         <f>September!H43</f>
-        <v>0.82638888888888895</v>
+        <v>1.125</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
@@ -7005,12 +7005,12 @@
       </c>
       <c r="E19" s="46">
         <f>'Oktober '!H43</f>
-        <v>0.82638888888888895</v>
+        <v>1.125</v>
       </c>
       <c r="F19" s="46"/>
       <c r="G19" s="46">
         <f>'Oktober '!H44</f>
-        <v>0.82638888888888895</v>
+        <v>1.125</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
@@ -7028,12 +7028,12 @@
       </c>
       <c r="E20" s="46">
         <f>'November '!H42</f>
-        <v>0.82638888888888895</v>
+        <v>1.125</v>
       </c>
       <c r="F20" s="46"/>
       <c r="G20" s="46">
         <f>'November '!H43</f>
-        <v>0.82638888888888895</v>
+        <v>1.125</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
@@ -7051,12 +7051,12 @@
       </c>
       <c r="E21" s="46">
         <f>'Dezember '!H43</f>
-        <v>0.82638888888888895</v>
+        <v>1.125</v>
       </c>
       <c r="F21" s="46"/>
       <c r="G21" s="46">
         <f>'Dezember '!H44</f>
-        <v>0.82638888888888895</v>
+        <v>1.125</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
@@ -8594,15 +8594,15 @@
         <v>0.75</v>
       </c>
       <c r="F26" s="29">
-        <v>2.7777777777777776E-2</v>
+        <v>3.125E-2</v>
       </c>
       <c r="G26" s="6">
         <f t="shared" si="0"/>
-        <v>0.13888888888888884</v>
+        <v>0.13541666666666663</v>
       </c>
       <c r="H26" s="26">
         <f t="shared" si="1"/>
-        <v>0.13888888888888884</v>
+        <v>0.13541666666666663</v>
       </c>
       <c r="I26" s="30"/>
       <c r="J26" s="31"/>
@@ -8615,16 +8615,20 @@
         <v>15</v>
       </c>
       <c r="C27" s="32"/>
-      <c r="D27" s="29"/>
-      <c r="E27" s="29"/>
+      <c r="D27" s="29">
+        <v>0.625</v>
+      </c>
+      <c r="E27" s="29">
+        <v>0.71875</v>
+      </c>
       <c r="F27" s="29"/>
       <c r="G27" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>9.375E-2</v>
       </c>
       <c r="H27" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>9.375E-2</v>
       </c>
       <c r="I27" s="30"/>
       <c r="J27" s="31"/>
@@ -8703,16 +8707,22 @@
         <v>12</v>
       </c>
       <c r="C31" s="32"/>
-      <c r="D31" s="29"/>
-      <c r="E31" s="29"/>
-      <c r="F31" s="29"/>
+      <c r="D31" s="29">
+        <v>0.59722222222222221</v>
+      </c>
+      <c r="E31" s="29">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="F31" s="29">
+        <v>2.7777777777777776E-2</v>
+      </c>
       <c r="G31" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.20833333333333337</v>
       </c>
       <c r="H31" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.20833333333333337</v>
       </c>
       <c r="I31" s="30"/>
       <c r="J31" s="31"/>
@@ -8919,7 +8929,7 @@
       <c r="F42" s="1"/>
       <c r="H42" s="34">
         <f>SUM(H9:H39)</f>
-        <v>0.82638888888888895</v>
+        <v>1.125</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
@@ -8945,7 +8955,7 @@
       <c r="G44" s="15"/>
       <c r="H44" s="38">
         <f>H42-H41+H43</f>
-        <v>0.82638888888888895</v>
+        <v>1.125</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
@@ -9851,7 +9861,7 @@
       <c r="F42" s="1"/>
       <c r="H42" s="34">
         <f>'März '!H44</f>
-        <v>0.82638888888888895</v>
+        <v>1.125</v>
       </c>
     </row>
     <row r="43" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -9866,7 +9876,7 @@
       <c r="G43" s="15"/>
       <c r="H43" s="38">
         <f>H41-H40+H42</f>
-        <v>0.82638888888888895</v>
+        <v>1.125</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
@@ -10799,7 +10809,7 @@
       <c r="F43" s="1"/>
       <c r="H43" s="34">
         <f>'April '!H43</f>
-        <v>0.82638888888888895</v>
+        <v>1.125</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -10814,7 +10824,7 @@
       <c r="G44" s="15"/>
       <c r="H44" s="38">
         <f>H42-H41+H43</f>
-        <v>0.82638888888888895</v>
+        <v>1.125</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
@@ -11725,7 +11735,7 @@
       <c r="F42" s="1"/>
       <c r="H42" s="34">
         <f>'Mai '!H44</f>
-        <v>0.82638888888888895</v>
+        <v>1.125</v>
       </c>
     </row>
     <row r="43" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -11740,7 +11750,7 @@
       <c r="G43" s="15"/>
       <c r="H43" s="38">
         <f>H41-H40+H42</f>
-        <v>0.82638888888888895</v>
+        <v>1.125</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
@@ -12673,7 +12683,7 @@
       <c r="F43" s="1"/>
       <c r="H43" s="34">
         <f>'Juni '!H43</f>
-        <v>0.82638888888888895</v>
+        <v>1.125</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -12688,7 +12698,7 @@
       <c r="G44" s="15"/>
       <c r="H44" s="38">
         <f>H42-H41+H43</f>
-        <v>0.82638888888888895</v>
+        <v>1.125</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
@@ -13621,7 +13631,7 @@
       <c r="F43" s="1"/>
       <c r="H43" s="34">
         <f>'Juli '!H44</f>
-        <v>0.82638888888888895</v>
+        <v>1.125</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -13636,7 +13646,7 @@
       <c r="G44" s="15"/>
       <c r="H44" s="38">
         <f>H42-H41+H43</f>
-        <v>0.82638888888888895</v>
+        <v>1.125</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
@@ -14547,7 +14557,7 @@
       <c r="F42" s="1"/>
       <c r="H42" s="34">
         <f>'August '!H44</f>
-        <v>0.82638888888888895</v>
+        <v>1.125</v>
       </c>
     </row>
     <row r="43" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -14562,7 +14572,7 @@
       <c r="G43" s="15"/>
       <c r="H43" s="38">
         <f>H41-H40+H42</f>
-        <v>0.82638888888888895</v>
+        <v>1.125</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
new database from crocodb found and added more data points into the database
</commit_message>
<xml_diff>
--- a/HK Zeiterfassung 2026.xlsx
+++ b/HK Zeiterfassung 2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr date1904="1" codeName="DieseArbeitsmappe"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harik\Downloads\Computational Chemistry\Variant-Effect-Predictor-for-nAChRs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B543937-8274-4B78-AA37-7748540B5379}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59407B70-B356-4B82-BB6E-DCEF2913814D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12105" yWindow="4170" windowWidth="17085" windowHeight="10425" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7440" yWindow="5265" windowWidth="19755" windowHeight="12330" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Januar " sheetId="26" r:id="rId1"/>
@@ -4734,7 +4734,7 @@
       <c r="F43" s="1"/>
       <c r="H43" s="34">
         <f>September!H43</f>
-        <v>2.083333333333333</v>
+        <v>2.6666666666666661</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -4749,7 +4749,7 @@
       <c r="G44" s="15"/>
       <c r="H44" s="38">
         <f>H42-H41+H43</f>
-        <v>2.083333333333333</v>
+        <v>2.6666666666666661</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
@@ -5661,7 +5661,7 @@
       <c r="F42" s="1"/>
       <c r="H42" s="34">
         <f>'Oktober '!H44</f>
-        <v>2.083333333333333</v>
+        <v>2.6666666666666661</v>
       </c>
     </row>
     <row r="43" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -5676,7 +5676,7 @@
       <c r="G43" s="15"/>
       <c r="H43" s="38">
         <f>H41-H40+H42</f>
-        <v>2.083333333333333</v>
+        <v>2.6666666666666661</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
@@ -6609,7 +6609,7 @@
       <c r="F43" s="1"/>
       <c r="H43" s="34">
         <f>'November '!H43</f>
-        <v>2.083333333333333</v>
+        <v>2.6666666666666661</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -6624,7 +6624,7 @@
       <c r="G44" s="15"/>
       <c r="H44" s="38">
         <f>H42-H41+H43</f>
-        <v>2.083333333333333</v>
+        <v>2.6666666666666661</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
@@ -6863,7 +6863,7 @@
       </c>
       <c r="D13" s="46">
         <f>'April '!H41</f>
-        <v>0.74999999999999978</v>
+        <v>1.333333333333333</v>
       </c>
       <c r="E13" s="46">
         <f>'April '!H42</f>
@@ -6872,7 +6872,7 @@
       <c r="F13" s="46"/>
       <c r="G13" s="46">
         <f>'April '!H43</f>
-        <v>2.083333333333333</v>
+        <v>2.6666666666666661</v>
       </c>
     </row>
     <row r="14" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -6890,12 +6890,12 @@
       </c>
       <c r="E14" s="46">
         <f>'Mai '!H43</f>
-        <v>2.083333333333333</v>
+        <v>2.6666666666666661</v>
       </c>
       <c r="F14" s="46"/>
       <c r="G14" s="46">
         <f>'Mai '!H44</f>
-        <v>2.083333333333333</v>
+        <v>2.6666666666666661</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
@@ -6913,12 +6913,12 @@
       </c>
       <c r="E15" s="46">
         <f>'Juni '!H42</f>
-        <v>2.083333333333333</v>
+        <v>2.6666666666666661</v>
       </c>
       <c r="F15" s="46"/>
       <c r="G15" s="46">
         <f>'Juni '!H43</f>
-        <v>2.083333333333333</v>
+        <v>2.6666666666666661</v>
       </c>
     </row>
     <row r="16" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -6936,12 +6936,12 @@
       </c>
       <c r="E16" s="46">
         <f>'Juli '!H43</f>
-        <v>2.083333333333333</v>
+        <v>2.6666666666666661</v>
       </c>
       <c r="F16" s="46"/>
       <c r="G16" s="46">
         <f>'Juli '!H44</f>
-        <v>2.083333333333333</v>
+        <v>2.6666666666666661</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
@@ -6959,12 +6959,12 @@
       </c>
       <c r="E17" s="46">
         <f>'August '!H43</f>
-        <v>2.083333333333333</v>
+        <v>2.6666666666666661</v>
       </c>
       <c r="F17" s="46"/>
       <c r="G17" s="46">
         <f>'August '!H44</f>
-        <v>2.083333333333333</v>
+        <v>2.6666666666666661</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
@@ -6982,12 +6982,12 @@
       </c>
       <c r="E18" s="46">
         <f>September!H42</f>
-        <v>2.083333333333333</v>
+        <v>2.6666666666666661</v>
       </c>
       <c r="F18" s="46"/>
       <c r="G18" s="46">
         <f>September!H43</f>
-        <v>2.083333333333333</v>
+        <v>2.6666666666666661</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
@@ -7005,12 +7005,12 @@
       </c>
       <c r="E19" s="46">
         <f>'Oktober '!H43</f>
-        <v>2.083333333333333</v>
+        <v>2.6666666666666661</v>
       </c>
       <c r="F19" s="46"/>
       <c r="G19" s="46">
         <f>'Oktober '!H44</f>
-        <v>2.083333333333333</v>
+        <v>2.6666666666666661</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
@@ -7028,12 +7028,12 @@
       </c>
       <c r="E20" s="46">
         <f>'November '!H42</f>
-        <v>2.083333333333333</v>
+        <v>2.6666666666666661</v>
       </c>
       <c r="F20" s="46"/>
       <c r="G20" s="46">
         <f>'November '!H43</f>
-        <v>2.083333333333333</v>
+        <v>2.6666666666666661</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
@@ -7051,12 +7051,12 @@
       </c>
       <c r="E21" s="46">
         <f>'Dezember '!H43</f>
-        <v>2.083333333333333</v>
+        <v>2.6666666666666661</v>
       </c>
       <c r="F21" s="46"/>
       <c r="G21" s="46">
         <f>'Dezember '!H44</f>
-        <v>2.083333333333333</v>
+        <v>2.6666666666666661</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
@@ -9392,16 +9392,20 @@
         <v>16</v>
       </c>
       <c r="C18" s="32"/>
-      <c r="D18" s="29"/>
-      <c r="E18" s="29"/>
+      <c r="D18" s="29">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="E18" s="29">
+        <v>0.5</v>
+      </c>
       <c r="F18" s="29"/>
       <c r="G18" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>8.3333333333333315E-2</v>
       </c>
       <c r="H18" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>8.3333333333333315E-2</v>
       </c>
       <c r="I18" s="30"/>
       <c r="J18" s="31"/>
@@ -9690,16 +9694,20 @@
         <v>15</v>
       </c>
       <c r="C31" s="32"/>
-      <c r="D31" s="29"/>
-      <c r="E31" s="29"/>
+      <c r="D31" s="29">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="E31" s="29">
+        <v>0.6875</v>
+      </c>
       <c r="F31" s="29"/>
       <c r="G31" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.10416666666666663</v>
       </c>
       <c r="H31" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.10416666666666663</v>
       </c>
       <c r="I31" s="30"/>
       <c r="J31" s="31"/>
@@ -9800,16 +9808,20 @@
         <v>13</v>
       </c>
       <c r="C36" s="32"/>
-      <c r="D36" s="29"/>
-      <c r="E36" s="29"/>
+      <c r="D36" s="29">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="E36" s="29">
+        <v>0.77083333333333337</v>
+      </c>
       <c r="F36" s="29"/>
       <c r="G36" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.1875</v>
       </c>
       <c r="H36" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.1875</v>
       </c>
       <c r="I36" s="30"/>
       <c r="J36" s="31"/>
@@ -9844,16 +9856,20 @@
         <v>15</v>
       </c>
       <c r="C38" s="32"/>
-      <c r="D38" s="29"/>
-      <c r="E38" s="29"/>
+      <c r="D38" s="29">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="E38" s="29">
+        <v>0.75</v>
+      </c>
       <c r="F38" s="29"/>
       <c r="G38" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.20833333333333337</v>
       </c>
       <c r="H38" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.20833333333333337</v>
       </c>
       <c r="I38" s="30"/>
       <c r="J38" s="31"/>
@@ -9884,7 +9900,7 @@
       <c r="F41" s="1"/>
       <c r="H41" s="34">
         <f>SUM(H9:H38)</f>
-        <v>0.74999999999999978</v>
+        <v>1.333333333333333</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
@@ -9910,7 +9926,7 @@
       <c r="G43" s="15"/>
       <c r="H43" s="38">
         <f>H41-H40+H42</f>
-        <v>2.083333333333333</v>
+        <v>2.6666666666666661</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
@@ -10843,7 +10859,7 @@
       <c r="F43" s="1"/>
       <c r="H43" s="34">
         <f>'April '!H43</f>
-        <v>2.083333333333333</v>
+        <v>2.6666666666666661</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -10858,7 +10874,7 @@
       <c r="G44" s="15"/>
       <c r="H44" s="38">
         <f>H42-H41+H43</f>
-        <v>2.083333333333333</v>
+        <v>2.6666666666666661</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
@@ -11769,7 +11785,7 @@
       <c r="F42" s="1"/>
       <c r="H42" s="34">
         <f>'Mai '!H44</f>
-        <v>2.083333333333333</v>
+        <v>2.6666666666666661</v>
       </c>
     </row>
     <row r="43" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -11784,7 +11800,7 @@
       <c r="G43" s="15"/>
       <c r="H43" s="38">
         <f>H41-H40+H42</f>
-        <v>2.083333333333333</v>
+        <v>2.6666666666666661</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
@@ -12717,7 +12733,7 @@
       <c r="F43" s="1"/>
       <c r="H43" s="34">
         <f>'Juni '!H43</f>
-        <v>2.083333333333333</v>
+        <v>2.6666666666666661</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -12732,7 +12748,7 @@
       <c r="G44" s="15"/>
       <c r="H44" s="38">
         <f>H42-H41+H43</f>
-        <v>2.083333333333333</v>
+        <v>2.6666666666666661</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
@@ -13665,7 +13681,7 @@
       <c r="F43" s="1"/>
       <c r="H43" s="34">
         <f>'Juli '!H44</f>
-        <v>2.083333333333333</v>
+        <v>2.6666666666666661</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -13680,7 +13696,7 @@
       <c r="G44" s="15"/>
       <c r="H44" s="38">
         <f>H42-H41+H43</f>
-        <v>2.083333333333333</v>
+        <v>2.6666666666666661</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
@@ -14591,7 +14607,7 @@
       <c r="F42" s="1"/>
       <c r="H42" s="34">
         <f>'August '!H44</f>
-        <v>2.083333333333333</v>
+        <v>2.6666666666666661</v>
       </c>
     </row>
     <row r="43" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -14606,7 +14622,7 @@
       <c r="G43" s="15"/>
       <c r="H43" s="38">
         <f>H41-H40+H42</f>
-        <v>2.083333333333333</v>
+        <v>2.6666666666666661</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
new data and references of all previous data in jabref
</commit_message>
<xml_diff>
--- a/HK Zeiterfassung 2026.xlsx
+++ b/HK Zeiterfassung 2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harik\Downloads\Computational Chemistry\Variant-Effect-Predictor-for-nAChRs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59407B70-B356-4B82-BB6E-DCEF2913814D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3E06CD9-E32B-497B-9BCB-63B620049B11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7440" yWindow="5265" windowWidth="19755" windowHeight="12330" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10665" yWindow="5700" windowWidth="17280" windowHeight="9885" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Januar " sheetId="26" r:id="rId1"/>
@@ -2489,46 +2489,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="3" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="17" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="17" fontId="0" fillId="3" borderId="17" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -2591,6 +2551,61 @@
       <alignment horizontal="right"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="17" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="17" fontId="0" fillId="3" borderId="17" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2613,21 +2628,6 @@
     <xf numFmtId="166" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2923,98 +2923,98 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="72"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="62"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="73" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="74"/>
-      <c r="C2" s="75" t="s">
+      <c r="A2" s="63" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="64"/>
+      <c r="C2" s="65" t="s">
         <v>408</v>
       </c>
-      <c r="D2" s="75"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="77" t="s">
+      <c r="D2" s="65"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="74"/>
+      <c r="G2" s="64"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="78" t="s">
+      <c r="I2" s="68" t="s">
         <v>407</v>
       </c>
-      <c r="J2" s="79"/>
+      <c r="J2" s="69"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="64" t="s">
+      <c r="B3" s="53"/>
+      <c r="C3" s="54" t="s">
         <v>408</v>
       </c>
-      <c r="D3" s="64"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="66" t="s">
+      <c r="D3" s="54"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="67"/>
+      <c r="G3" s="57"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="68">
+      <c r="I3" s="58">
         <v>2026</v>
       </c>
-      <c r="J3" s="69"/>
+      <c r="J3" s="59"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="52" t="s">
+      <c r="C4" s="70" t="s">
         <v>408</v>
       </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="53"/>
+      <c r="D4" s="70"/>
+      <c r="E4" s="71"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="54" t="s">
+      <c r="I4" s="72" t="s">
         <v>408</v>
       </c>
-      <c r="J4" s="55"/>
+      <c r="J4" s="73"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="56" t="s">
+      <c r="C5" s="74" t="s">
         <v>408</v>
       </c>
-      <c r="D5" s="56"/>
-      <c r="E5" s="57"/>
+      <c r="D5" s="74"/>
+      <c r="E5" s="75"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="58" t="s">
+      <c r="I5" s="76" t="s">
         <v>409</v>
       </c>
-      <c r="J5" s="59"/>
+      <c r="J5" s="77"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -3027,10 +3027,10 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="60" t="s">
+      <c r="I6" s="78" t="s">
         <v>409</v>
       </c>
-      <c r="J6" s="61"/>
+      <c r="J6" s="79"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -3819,6 +3819,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -3828,11 +3833,6 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -3863,104 +3863,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="72"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="62"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="73" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="74"/>
-      <c r="C2" s="75" t="str">
+      <c r="A2" s="63" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="64"/>
+      <c r="C2" s="65" t="str">
         <f>September!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="75"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="77" t="s">
+      <c r="D2" s="65"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="74"/>
+      <c r="G2" s="64"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="78" t="s">
+      <c r="I2" s="68" t="s">
         <v>311</v>
       </c>
-      <c r="J2" s="79"/>
+      <c r="J2" s="69"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="64" t="str">
+      <c r="B3" s="53"/>
+      <c r="C3" s="54" t="str">
         <f>September!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="64"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="66" t="s">
+      <c r="D3" s="54"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="67"/>
+      <c r="G3" s="57"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="68">
+      <c r="I3" s="58">
         <v>2026</v>
       </c>
-      <c r="J3" s="69"/>
+      <c r="J3" s="59"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="52" t="str">
+      <c r="C4" s="70" t="str">
         <f>September!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="53"/>
+      <c r="D4" s="70"/>
+      <c r="E4" s="71"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="54" t="str">
+      <c r="I4" s="72" t="str">
         <f>September!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="55"/>
+      <c r="J4" s="73"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="56" t="str">
+      <c r="C5" s="74" t="str">
         <f>September!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="56"/>
-      <c r="E5" s="57"/>
+      <c r="D5" s="74"/>
+      <c r="E5" s="75"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="58">
+      <c r="I5" s="76">
         <f>September!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="59"/>
+      <c r="J5" s="77"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -3973,11 +3973,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="60" t="str">
+      <c r="I6" s="78" t="str">
         <f>September!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="61"/>
+      <c r="J6" s="79"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -4734,7 +4734,7 @@
       <c r="F43" s="1"/>
       <c r="H43" s="34">
         <f>September!H43</f>
-        <v>2.6666666666666661</v>
+        <v>2.8749999999999996</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -4749,7 +4749,7 @@
       <c r="G44" s="15"/>
       <c r="H44" s="38">
         <f>H42-H41+H43</f>
-        <v>2.6666666666666661</v>
+        <v>2.8749999999999996</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
@@ -4767,6 +4767,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -4776,11 +4781,6 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -4811,104 +4811,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="72"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="62"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="73" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="74"/>
-      <c r="C2" s="75" t="str">
+      <c r="A2" s="63" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="64"/>
+      <c r="C2" s="65" t="str">
         <f>'Oktober '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="75"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="77" t="s">
+      <c r="D2" s="65"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="74"/>
+      <c r="G2" s="64"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="78" t="s">
+      <c r="I2" s="68" t="s">
         <v>343</v>
       </c>
-      <c r="J2" s="79"/>
+      <c r="J2" s="69"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="64" t="str">
+      <c r="B3" s="53"/>
+      <c r="C3" s="54" t="str">
         <f>'Oktober '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="64"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="66" t="s">
+      <c r="D3" s="54"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="67"/>
+      <c r="G3" s="57"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="68">
+      <c r="I3" s="58">
         <v>2026</v>
       </c>
-      <c r="J3" s="69"/>
+      <c r="J3" s="59"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="52" t="str">
+      <c r="C4" s="70" t="str">
         <f>'Oktober '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="53"/>
+      <c r="D4" s="70"/>
+      <c r="E4" s="71"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="54" t="str">
+      <c r="I4" s="72" t="str">
         <f>'Oktober '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="55"/>
+      <c r="J4" s="73"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="56" t="str">
+      <c r="C5" s="74" t="str">
         <f>'Oktober '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="56"/>
-      <c r="E5" s="57"/>
+      <c r="D5" s="74"/>
+      <c r="E5" s="75"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="58">
+      <c r="I5" s="76">
         <f>'Oktober '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="59"/>
+      <c r="J5" s="77"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -4921,11 +4921,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="60" t="str">
+      <c r="I6" s="78" t="str">
         <f>'Oktober '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="61"/>
+      <c r="J6" s="79"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -5661,7 +5661,7 @@
       <c r="F42" s="1"/>
       <c r="H42" s="34">
         <f>'Oktober '!H44</f>
-        <v>2.6666666666666661</v>
+        <v>2.8749999999999996</v>
       </c>
     </row>
     <row r="43" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -5676,7 +5676,7 @@
       <c r="G43" s="15"/>
       <c r="H43" s="38">
         <f>H41-H40+H42</f>
-        <v>2.6666666666666661</v>
+        <v>2.8749999999999996</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
@@ -5694,6 +5694,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -5703,11 +5708,6 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -5738,104 +5738,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="72"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="62"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="73" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="74"/>
-      <c r="C2" s="75" t="str">
+      <c r="A2" s="63" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="64"/>
+      <c r="C2" s="65" t="str">
         <f>'November '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="75"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="77" t="s">
+      <c r="D2" s="65"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="74"/>
+      <c r="G2" s="64"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="78" t="s">
+      <c r="I2" s="68" t="s">
         <v>374</v>
       </c>
-      <c r="J2" s="79"/>
+      <c r="J2" s="69"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="64" t="str">
+      <c r="B3" s="53"/>
+      <c r="C3" s="54" t="str">
         <f>'November '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="64"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="66" t="s">
+      <c r="D3" s="54"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="67"/>
+      <c r="G3" s="57"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="68">
+      <c r="I3" s="58">
         <v>2026</v>
       </c>
-      <c r="J3" s="69"/>
+      <c r="J3" s="59"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="52" t="str">
+      <c r="C4" s="70" t="str">
         <f>'November '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="53"/>
+      <c r="D4" s="70"/>
+      <c r="E4" s="71"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="54" t="str">
+      <c r="I4" s="72" t="str">
         <f>'November '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="55"/>
+      <c r="J4" s="73"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="56" t="str">
+      <c r="C5" s="74" t="str">
         <f>'November '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="56"/>
-      <c r="E5" s="57"/>
+      <c r="D5" s="74"/>
+      <c r="E5" s="75"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="58">
+      <c r="I5" s="76">
         <f>'November '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="59"/>
+      <c r="J5" s="77"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -5848,11 +5848,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="60" t="str">
+      <c r="I6" s="78" t="str">
         <f>'November '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="61"/>
+      <c r="J6" s="79"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -6609,7 +6609,7 @@
       <c r="F43" s="1"/>
       <c r="H43" s="34">
         <f>'November '!H43</f>
-        <v>2.6666666666666661</v>
+        <v>2.8749999999999996</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -6624,7 +6624,7 @@
       <c r="G44" s="15"/>
       <c r="H44" s="38">
         <f>H42-H41+H43</f>
-        <v>2.6666666666666661</v>
+        <v>2.8749999999999996</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
@@ -6642,6 +6642,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -6651,11 +6656,6 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -6687,22 +6687,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="80" t="s">
+      <c r="A1" s="85" t="s">
         <v>416</v>
       </c>
-      <c r="B1" s="81"/>
-      <c r="C1" s="81"/>
-      <c r="D1" s="81"/>
-      <c r="E1" s="81"/>
-      <c r="F1" s="81"/>
-      <c r="G1" s="81"/>
-      <c r="H1" s="82"/>
+      <c r="B1" s="86"/>
+      <c r="C1" s="86"/>
+      <c r="D1" s="86"/>
+      <c r="E1" s="86"/>
+      <c r="F1" s="86"/>
+      <c r="G1" s="86"/>
+      <c r="H1" s="87"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="62" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="63"/>
+      <c r="A2" s="52" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="53"/>
       <c r="C2" s="47" t="str">
         <f>'November '!C2:E2</f>
         <v>Hari Krishna</v>
@@ -6711,15 +6711,15 @@
       <c r="E2" s="22" t="s">
         <v>418</v>
       </c>
-      <c r="F2" s="86"/>
-      <c r="G2" s="86"/>
+      <c r="F2" s="91"/>
+      <c r="G2" s="91"/>
       <c r="H2" s="48"/>
     </row>
     <row r="3" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="89" t="s">
+      <c r="A3" s="82" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="67"/>
+      <c r="B3" s="57"/>
       <c r="C3" s="49" t="str">
         <f>'November '!C3:E3</f>
         <v>Mohan Raj</v>
@@ -6728,8 +6728,8 @@
       <c r="E3" s="18" t="s">
         <v>122</v>
       </c>
-      <c r="F3" s="68"/>
-      <c r="G3" s="68"/>
+      <c r="F3" s="58"/>
+      <c r="G3" s="58"/>
       <c r="H3" s="50"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
@@ -6743,17 +6743,17 @@
       </c>
     </row>
     <row r="6" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="84" t="s">
+      <c r="A6" s="89" t="s">
         <v>417</v>
       </c>
-      <c r="B6" s="85"/>
-      <c r="C6" s="83" t="s">
+      <c r="B6" s="90"/>
+      <c r="C6" s="88" t="s">
         <v>419</v>
       </c>
-      <c r="D6" s="83"/>
-      <c r="E6" s="83"/>
-      <c r="F6" s="83"/>
-      <c r="G6" s="83"/>
+      <c r="D6" s="88"/>
+      <c r="E6" s="88"/>
+      <c r="F6" s="88"/>
+      <c r="G6" s="88"/>
       <c r="H6" s="51"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
@@ -6765,10 +6765,10 @@
       <c r="D8" s="3"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A9" s="87" t="s">
+      <c r="A9" s="80" t="s">
         <v>410</v>
       </c>
-      <c r="B9" s="88"/>
+      <c r="B9" s="81"/>
       <c r="C9" s="44" t="s">
         <v>411</v>
       </c>
@@ -6784,10 +6784,10 @@
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A10" s="90" t="s">
+      <c r="A10" s="83" t="s">
         <v>407</v>
       </c>
-      <c r="B10" s="91"/>
+      <c r="B10" s="84"/>
       <c r="C10" s="46">
         <f>'Januar '!H41</f>
         <v>0</v>
@@ -6806,10 +6806,10 @@
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A11" s="90" t="s">
+      <c r="A11" s="83" t="s">
         <v>406</v>
       </c>
-      <c r="B11" s="91"/>
+      <c r="B11" s="84"/>
       <c r="C11" s="46">
         <f>'Februar '!H39</f>
         <v>0</v>
@@ -6829,10 +6829,10 @@
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A12" s="90" t="s">
+      <c r="A12" s="83" t="s">
         <v>89</v>
       </c>
-      <c r="B12" s="91"/>
+      <c r="B12" s="84"/>
       <c r="C12" s="46">
         <f>'März '!H41</f>
         <v>0</v>
@@ -6853,10 +6853,10 @@
       <c r="M12" s="28"/>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A13" s="90" t="s">
+      <c r="A13" s="83" t="s">
         <v>121</v>
       </c>
-      <c r="B13" s="91"/>
+      <c r="B13" s="84"/>
       <c r="C13" s="46">
         <f>'April '!H40</f>
         <v>0</v>
@@ -6876,17 +6876,17 @@
       </c>
     </row>
     <row r="14" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="90" t="s">
+      <c r="A14" s="83" t="s">
         <v>185</v>
       </c>
-      <c r="B14" s="91"/>
+      <c r="B14" s="84"/>
       <c r="C14" s="46">
         <f>'Mai '!H41</f>
         <v>0</v>
       </c>
       <c r="D14" s="46">
         <f>'Mai '!H42</f>
-        <v>0</v>
+        <v>0.20833333333333329</v>
       </c>
       <c r="E14" s="46">
         <f>'Mai '!H43</f>
@@ -6895,14 +6895,14 @@
       <c r="F14" s="46"/>
       <c r="G14" s="46">
         <f>'Mai '!H44</f>
-        <v>2.6666666666666661</v>
+        <v>2.8749999999999996</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A15" s="90" t="s">
+      <c r="A15" s="83" t="s">
         <v>184</v>
       </c>
-      <c r="B15" s="91"/>
+      <c r="B15" s="84"/>
       <c r="C15" s="46">
         <f>'Juni '!H40</f>
         <v>0</v>
@@ -6913,19 +6913,19 @@
       </c>
       <c r="E15" s="46">
         <f>'Juni '!H42</f>
-        <v>2.6666666666666661</v>
+        <v>2.8749999999999996</v>
       </c>
       <c r="F15" s="46"/>
       <c r="G15" s="46">
         <f>'Juni '!H43</f>
-        <v>2.6666666666666661</v>
+        <v>2.8749999999999996</v>
       </c>
     </row>
     <row r="16" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="90" t="s">
+      <c r="A16" s="83" t="s">
         <v>247</v>
       </c>
-      <c r="B16" s="91"/>
+      <c r="B16" s="84"/>
       <c r="C16" s="46">
         <f>'Juli '!H41</f>
         <v>0</v>
@@ -6936,19 +6936,19 @@
       </c>
       <c r="E16" s="46">
         <f>'Juli '!H43</f>
-        <v>2.6666666666666661</v>
+        <v>2.8749999999999996</v>
       </c>
       <c r="F16" s="46"/>
       <c r="G16" s="46">
         <f>'Juli '!H44</f>
-        <v>2.6666666666666661</v>
+        <v>2.8749999999999996</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="90" t="s">
+      <c r="A17" s="83" t="s">
         <v>248</v>
       </c>
-      <c r="B17" s="91"/>
+      <c r="B17" s="84"/>
       <c r="C17" s="46">
         <f>'August '!H41</f>
         <v>0</v>
@@ -6959,19 +6959,19 @@
       </c>
       <c r="E17" s="46">
         <f>'August '!H43</f>
-        <v>2.6666666666666661</v>
+        <v>2.8749999999999996</v>
       </c>
       <c r="F17" s="46"/>
       <c r="G17" s="46">
         <f>'August '!H44</f>
-        <v>2.6666666666666661</v>
+        <v>2.8749999999999996</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="90" t="s">
+      <c r="A18" s="83" t="s">
         <v>280</v>
       </c>
-      <c r="B18" s="91"/>
+      <c r="B18" s="84"/>
       <c r="C18" s="46">
         <f>September!H40</f>
         <v>0</v>
@@ -6982,19 +6982,19 @@
       </c>
       <c r="E18" s="46">
         <f>September!H42</f>
-        <v>2.6666666666666661</v>
+        <v>2.8749999999999996</v>
       </c>
       <c r="F18" s="46"/>
       <c r="G18" s="46">
         <f>September!H43</f>
-        <v>2.6666666666666661</v>
+        <v>2.8749999999999996</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="90" t="s">
+      <c r="A19" s="83" t="s">
         <v>311</v>
       </c>
-      <c r="B19" s="91"/>
+      <c r="B19" s="84"/>
       <c r="C19" s="46">
         <f>'Oktober '!H41</f>
         <v>0</v>
@@ -7005,19 +7005,19 @@
       </c>
       <c r="E19" s="46">
         <f>'Oktober '!H43</f>
-        <v>2.6666666666666661</v>
+        <v>2.8749999999999996</v>
       </c>
       <c r="F19" s="46"/>
       <c r="G19" s="46">
         <f>'Oktober '!H44</f>
-        <v>2.6666666666666661</v>
+        <v>2.8749999999999996</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="90" t="s">
+      <c r="A20" s="83" t="s">
         <v>343</v>
       </c>
-      <c r="B20" s="91"/>
+      <c r="B20" s="84"/>
       <c r="C20" s="46">
         <f>'November '!H40</f>
         <v>0</v>
@@ -7028,19 +7028,19 @@
       </c>
       <c r="E20" s="46">
         <f>'November '!H42</f>
-        <v>2.6666666666666661</v>
+        <v>2.8749999999999996</v>
       </c>
       <c r="F20" s="46"/>
       <c r="G20" s="46">
         <f>'November '!H43</f>
-        <v>2.6666666666666661</v>
+        <v>2.8749999999999996</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="90" t="s">
+      <c r="A21" s="83" t="s">
         <v>374</v>
       </c>
-      <c r="B21" s="91"/>
+      <c r="B21" s="84"/>
       <c r="C21" s="46">
         <f>'Dezember '!H41</f>
         <v>0</v>
@@ -7051,12 +7051,12 @@
       </c>
       <c r="E21" s="46">
         <f>'Dezember '!H43</f>
-        <v>2.6666666666666661</v>
+        <v>2.8749999999999996</v>
       </c>
       <c r="F21" s="46"/>
       <c r="G21" s="46">
         <f>'Dezember '!H44</f>
-        <v>2.6666666666666661</v>
+        <v>2.8749999999999996</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
@@ -7093,6 +7093,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="20">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="C6:G6"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="F3:G3"/>
     <mergeCell ref="A9:B9"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A3:B3"/>
@@ -7108,11 +7113,6 @@
     <mergeCell ref="A17:B17"/>
     <mergeCell ref="A18:B18"/>
     <mergeCell ref="A19:B19"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="C6:G6"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="F3:G3"/>
   </mergeCells>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.39370078740157483" bottom="0.39370078740157483" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -7135,104 +7135,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="72"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="62"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="73" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="74"/>
-      <c r="C2" s="75" t="str">
+      <c r="A2" s="63" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="64"/>
+      <c r="C2" s="65" t="str">
         <f>'Januar '!C2:E2</f>
         <v>XXX</v>
       </c>
-      <c r="D2" s="75"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="77" t="s">
+      <c r="D2" s="65"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="74"/>
+      <c r="G2" s="64"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="78" t="s">
+      <c r="I2" s="68" t="s">
         <v>406</v>
       </c>
-      <c r="J2" s="79"/>
+      <c r="J2" s="69"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="64" t="str">
+      <c r="B3" s="53"/>
+      <c r="C3" s="54" t="str">
         <f>'Januar '!C3:E3</f>
         <v>XXX</v>
       </c>
-      <c r="D3" s="64"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="66" t="s">
+      <c r="D3" s="54"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="67"/>
+      <c r="G3" s="57"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="68">
+      <c r="I3" s="58">
         <v>2026</v>
       </c>
-      <c r="J3" s="69"/>
+      <c r="J3" s="59"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="52" t="str">
+      <c r="C4" s="70" t="str">
         <f>'Januar '!C4:E4</f>
         <v>XXX</v>
       </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="53"/>
+      <c r="D4" s="70"/>
+      <c r="E4" s="71"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="54" t="str">
+      <c r="I4" s="72" t="str">
         <f>'Januar '!I4:J4</f>
         <v>XXX</v>
       </c>
-      <c r="J4" s="55"/>
+      <c r="J4" s="73"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="56" t="str">
+      <c r="C5" s="74" t="str">
         <f>'Januar '!C5:E5</f>
         <v>XXX</v>
       </c>
-      <c r="D5" s="56"/>
-      <c r="E5" s="57"/>
+      <c r="D5" s="74"/>
+      <c r="E5" s="75"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="58" t="str">
+      <c r="I5" s="76" t="str">
         <f>'Januar '!I5:J5</f>
         <v>XX</v>
       </c>
-      <c r="J5" s="59"/>
+      <c r="J5" s="77"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -7245,11 +7245,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="60" t="str">
+      <c r="I6" s="78" t="str">
         <f>'Januar '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="61"/>
+      <c r="J6" s="79"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -7985,6 +7985,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -7994,11 +7999,6 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -8029,98 +8029,98 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="72"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="62"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="73" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="74"/>
-      <c r="C2" s="75" t="s">
+      <c r="A2" s="63" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="64"/>
+      <c r="C2" s="65" t="s">
         <v>420</v>
       </c>
-      <c r="D2" s="75"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="77" t="s">
+      <c r="D2" s="65"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="74"/>
+      <c r="G2" s="64"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="78" t="s">
+      <c r="I2" s="68" t="s">
         <v>89</v>
       </c>
-      <c r="J2" s="79"/>
+      <c r="J2" s="69"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="64" t="s">
+      <c r="B3" s="53"/>
+      <c r="C3" s="54" t="s">
         <v>421</v>
       </c>
-      <c r="D3" s="64"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="66" t="s">
+      <c r="D3" s="54"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="67"/>
+      <c r="G3" s="57"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="68">
+      <c r="I3" s="58">
         <v>2026</v>
       </c>
-      <c r="J3" s="69"/>
+      <c r="J3" s="59"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="52" t="s">
+      <c r="C4" s="70" t="s">
         <v>422</v>
       </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="53"/>
+      <c r="D4" s="70"/>
+      <c r="E4" s="71"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="54" t="s">
+      <c r="I4" s="72" t="s">
         <v>424</v>
       </c>
-      <c r="J4" s="55"/>
+      <c r="J4" s="73"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="56" t="s">
+      <c r="C5" s="74" t="s">
         <v>423</v>
       </c>
-      <c r="D5" s="56"/>
-      <c r="E5" s="57"/>
+      <c r="D5" s="74"/>
+      <c r="E5" s="75"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="58">
+      <c r="I5" s="76">
         <v>8</v>
       </c>
-      <c r="J5" s="59"/>
+      <c r="J5" s="77"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -8133,11 +8133,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="60" t="str">
+      <c r="I6" s="78" t="str">
         <f>'Februar '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="61"/>
+      <c r="J6" s="79"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -8976,6 +8976,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -8985,11 +8990,6 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -9020,104 +9020,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="72"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="62"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="73" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="74"/>
-      <c r="C2" s="75" t="str">
+      <c r="A2" s="63" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="64"/>
+      <c r="C2" s="65" t="str">
         <f>'März '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="75"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="77" t="s">
+      <c r="D2" s="65"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="74"/>
+      <c r="G2" s="64"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="78" t="s">
+      <c r="I2" s="68" t="s">
         <v>121</v>
       </c>
-      <c r="J2" s="79"/>
+      <c r="J2" s="69"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="64" t="str">
+      <c r="B3" s="53"/>
+      <c r="C3" s="54" t="str">
         <f>'März '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="64"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="66" t="s">
+      <c r="D3" s="54"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="67"/>
+      <c r="G3" s="57"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="68">
+      <c r="I3" s="58">
         <v>2026</v>
       </c>
-      <c r="J3" s="69"/>
+      <c r="J3" s="59"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="52" t="str">
+      <c r="C4" s="70" t="str">
         <f>'März '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="53"/>
+      <c r="D4" s="70"/>
+      <c r="E4" s="71"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="54" t="str">
+      <c r="I4" s="72" t="str">
         <f>'März '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="55"/>
+      <c r="J4" s="73"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="56" t="str">
+      <c r="C5" s="74" t="str">
         <f>'März '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="56"/>
-      <c r="E5" s="57"/>
+      <c r="D5" s="74"/>
+      <c r="E5" s="75"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="58">
+      <c r="I5" s="76">
         <f>'März '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="59"/>
+      <c r="J5" s="77"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -9130,11 +9130,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="60" t="str">
+      <c r="I6" s="78" t="str">
         <f>'März '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="61"/>
+      <c r="J6" s="79"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -9944,6 +9944,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -9953,11 +9958,6 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -9988,104 +9988,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="72"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="62"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="73" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="74"/>
-      <c r="C2" s="75" t="str">
+      <c r="A2" s="63" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="64"/>
+      <c r="C2" s="65" t="str">
         <f>'April '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="75"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="77" t="s">
+      <c r="D2" s="65"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="74"/>
+      <c r="G2" s="64"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="78" t="s">
+      <c r="I2" s="68" t="s">
         <v>185</v>
       </c>
-      <c r="J2" s="79"/>
+      <c r="J2" s="69"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="64" t="str">
+      <c r="B3" s="53"/>
+      <c r="C3" s="54" t="str">
         <f>'April '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="64"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="66" t="s">
+      <c r="D3" s="54"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="67"/>
+      <c r="G3" s="57"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="68">
+      <c r="I3" s="58">
         <v>2026</v>
       </c>
-      <c r="J3" s="69"/>
+      <c r="J3" s="59"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="52" t="str">
+      <c r="C4" s="70" t="str">
         <f>'April '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="53"/>
+      <c r="D4" s="70"/>
+      <c r="E4" s="71"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="54" t="str">
+      <c r="I4" s="72" t="str">
         <f>'April '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="55"/>
+      <c r="J4" s="73"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="56" t="str">
+      <c r="C5" s="74" t="str">
         <f>'April '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="56"/>
-      <c r="E5" s="57"/>
+      <c r="D5" s="74"/>
+      <c r="E5" s="75"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="58">
+      <c r="I5" s="76">
         <f>'April '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="59"/>
+      <c r="J5" s="77"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -10098,11 +10098,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="60" t="str">
+      <c r="I6" s="78" t="str">
         <f>'April '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="61"/>
+      <c r="J6" s="79"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -10280,16 +10280,22 @@
         <v>15</v>
       </c>
       <c r="C15" s="32"/>
-      <c r="D15" s="29"/>
-      <c r="E15" s="29"/>
-      <c r="F15" s="29"/>
+      <c r="D15" s="29">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="E15" s="29">
+        <v>0.8125</v>
+      </c>
+      <c r="F15" s="29">
+        <v>2.0833333333333332E-2</v>
+      </c>
       <c r="G15" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.20833333333333329</v>
       </c>
       <c r="H15" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.20833333333333329</v>
       </c>
       <c r="I15" s="30"/>
       <c r="J15" s="31"/>
@@ -10848,7 +10854,7 @@
       <c r="F42" s="1"/>
       <c r="H42" s="34">
         <f>SUM(H9:H39)</f>
-        <v>0</v>
+        <v>0.20833333333333329</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
@@ -10874,7 +10880,7 @@
       <c r="G44" s="15"/>
       <c r="H44" s="38">
         <f>H42-H41+H43</f>
-        <v>2.6666666666666661</v>
+        <v>2.8749999999999996</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
@@ -10892,6 +10898,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -10901,11 +10912,6 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -10936,104 +10942,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="72"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="62"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="73" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="74"/>
-      <c r="C2" s="75" t="str">
+      <c r="A2" s="63" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="64"/>
+      <c r="C2" s="65" t="str">
         <f>'Mai '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="75"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="77" t="s">
+      <c r="D2" s="65"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="74"/>
+      <c r="G2" s="64"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="78" t="s">
+      <c r="I2" s="68" t="s">
         <v>184</v>
       </c>
-      <c r="J2" s="79"/>
+      <c r="J2" s="69"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="64" t="str">
+      <c r="B3" s="53"/>
+      <c r="C3" s="54" t="str">
         <f>'Mai '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="64"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="66" t="s">
+      <c r="D3" s="54"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="67"/>
+      <c r="G3" s="57"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="68">
+      <c r="I3" s="58">
         <v>2026</v>
       </c>
-      <c r="J3" s="69"/>
+      <c r="J3" s="59"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="52" t="str">
+      <c r="C4" s="70" t="str">
         <f>'Mai '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="53"/>
+      <c r="D4" s="70"/>
+      <c r="E4" s="71"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="54" t="str">
+      <c r="I4" s="72" t="str">
         <f>'Mai '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="55"/>
+      <c r="J4" s="73"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="56" t="str">
+      <c r="C5" s="74" t="str">
         <f>'Mai '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="56"/>
-      <c r="E5" s="57"/>
+      <c r="D5" s="74"/>
+      <c r="E5" s="75"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="58">
+      <c r="I5" s="76">
         <f>'Mai '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="59"/>
+      <c r="J5" s="77"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -11046,11 +11052,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="60" t="str">
+      <c r="I6" s="78" t="str">
         <f>'Mai '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="61"/>
+      <c r="J6" s="79"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -11785,7 +11791,7 @@
       <c r="F42" s="1"/>
       <c r="H42" s="34">
         <f>'Mai '!H44</f>
-        <v>2.6666666666666661</v>
+        <v>2.8749999999999996</v>
       </c>
     </row>
     <row r="43" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -11800,7 +11806,7 @@
       <c r="G43" s="15"/>
       <c r="H43" s="38">
         <f>H41-H40+H42</f>
-        <v>2.6666666666666661</v>
+        <v>2.8749999999999996</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
@@ -11818,6 +11824,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -11827,11 +11838,6 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -11862,104 +11868,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="72"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="62"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="73" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="74"/>
-      <c r="C2" s="75" t="str">
+      <c r="A2" s="63" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="64"/>
+      <c r="C2" s="65" t="str">
         <f>'Juni '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="75"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="77" t="s">
+      <c r="D2" s="65"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="74"/>
+      <c r="G2" s="64"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="78" t="s">
+      <c r="I2" s="68" t="s">
         <v>247</v>
       </c>
-      <c r="J2" s="79"/>
+      <c r="J2" s="69"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="64" t="str">
+      <c r="B3" s="53"/>
+      <c r="C3" s="54" t="str">
         <f>'Juni '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="64"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="66" t="s">
+      <c r="D3" s="54"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="67"/>
+      <c r="G3" s="57"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="68">
+      <c r="I3" s="58">
         <v>2026</v>
       </c>
-      <c r="J3" s="69"/>
+      <c r="J3" s="59"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="52" t="str">
+      <c r="C4" s="70" t="str">
         <f>'Juni '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="53"/>
+      <c r="D4" s="70"/>
+      <c r="E4" s="71"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="54" t="str">
+      <c r="I4" s="72" t="str">
         <f>'Juni '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="55"/>
+      <c r="J4" s="73"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="56" t="str">
+      <c r="C5" s="74" t="str">
         <f>'Juni '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="56"/>
-      <c r="E5" s="57"/>
+      <c r="D5" s="74"/>
+      <c r="E5" s="75"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="58">
+      <c r="I5" s="76">
         <f>'Juni '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="59"/>
+      <c r="J5" s="77"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -11972,11 +11978,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="60" t="str">
+      <c r="I6" s="78" t="str">
         <f>'Juni '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="61"/>
+      <c r="J6" s="79"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -12733,7 +12739,7 @@
       <c r="F43" s="1"/>
       <c r="H43" s="34">
         <f>'Juni '!H43</f>
-        <v>2.6666666666666661</v>
+        <v>2.8749999999999996</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -12748,7 +12754,7 @@
       <c r="G44" s="15"/>
       <c r="H44" s="38">
         <f>H42-H41+H43</f>
-        <v>2.6666666666666661</v>
+        <v>2.8749999999999996</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
@@ -12766,6 +12772,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -12775,11 +12786,6 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -12810,104 +12816,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="72"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="62"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="73" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="74"/>
-      <c r="C2" s="75" t="str">
+      <c r="A2" s="63" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="64"/>
+      <c r="C2" s="65" t="str">
         <f>'Juli '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="75"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="77" t="s">
+      <c r="D2" s="65"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="74"/>
+      <c r="G2" s="64"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="78" t="s">
+      <c r="I2" s="68" t="s">
         <v>248</v>
       </c>
-      <c r="J2" s="79"/>
+      <c r="J2" s="69"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="64" t="str">
+      <c r="B3" s="53"/>
+      <c r="C3" s="54" t="str">
         <f>'Juli '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="64"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="66" t="s">
+      <c r="D3" s="54"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="67"/>
+      <c r="G3" s="57"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="68">
+      <c r="I3" s="58">
         <v>2026</v>
       </c>
-      <c r="J3" s="69"/>
+      <c r="J3" s="59"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="52" t="str">
+      <c r="C4" s="70" t="str">
         <f>'Juli '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="53"/>
+      <c r="D4" s="70"/>
+      <c r="E4" s="71"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="54" t="str">
+      <c r="I4" s="72" t="str">
         <f>'Juli '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="55"/>
+      <c r="J4" s="73"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="56" t="str">
+      <c r="C5" s="74" t="str">
         <f>'Juli '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="56"/>
-      <c r="E5" s="57"/>
+      <c r="D5" s="74"/>
+      <c r="E5" s="75"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="58">
+      <c r="I5" s="76">
         <f>'Juli '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="59"/>
+      <c r="J5" s="77"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -12920,11 +12926,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="60" t="str">
+      <c r="I6" s="78" t="str">
         <f>'Juli '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="61"/>
+      <c r="J6" s="79"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -13681,7 +13687,7 @@
       <c r="F43" s="1"/>
       <c r="H43" s="34">
         <f>'Juli '!H44</f>
-        <v>2.6666666666666661</v>
+        <v>2.8749999999999996</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -13696,7 +13702,7 @@
       <c r="G44" s="15"/>
       <c r="H44" s="38">
         <f>H42-H41+H43</f>
-        <v>2.6666666666666661</v>
+        <v>2.8749999999999996</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
@@ -13714,6 +13720,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -13723,11 +13734,6 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -13758,104 +13764,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="72"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="62"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="73" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="74"/>
-      <c r="C2" s="75" t="str">
+      <c r="A2" s="63" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="64"/>
+      <c r="C2" s="65" t="str">
         <f>'August '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="75"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="77" t="s">
+      <c r="D2" s="65"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="74"/>
+      <c r="G2" s="64"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="78" t="s">
+      <c r="I2" s="68" t="s">
         <v>280</v>
       </c>
-      <c r="J2" s="79"/>
+      <c r="J2" s="69"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="64" t="str">
+      <c r="B3" s="53"/>
+      <c r="C3" s="54" t="str">
         <f>'August '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="64"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="66" t="s">
+      <c r="D3" s="54"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="67"/>
+      <c r="G3" s="57"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="68">
+      <c r="I3" s="58">
         <v>2026</v>
       </c>
-      <c r="J3" s="69"/>
+      <c r="J3" s="59"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="52" t="str">
+      <c r="C4" s="70" t="str">
         <f>'August '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="53"/>
+      <c r="D4" s="70"/>
+      <c r="E4" s="71"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="54" t="str">
+      <c r="I4" s="72" t="str">
         <f>'August '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="55"/>
+      <c r="J4" s="73"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="56" t="str">
+      <c r="C5" s="74" t="str">
         <f>'August '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="56"/>
-      <c r="E5" s="57"/>
+      <c r="D5" s="74"/>
+      <c r="E5" s="75"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="58">
+      <c r="I5" s="76">
         <f>'August '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="59"/>
+      <c r="J5" s="77"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -13868,11 +13874,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="60" t="str">
+      <c r="I6" s="78" t="str">
         <f>'August '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="61"/>
+      <c r="J6" s="79"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -14607,7 +14613,7 @@
       <c r="F42" s="1"/>
       <c r="H42" s="34">
         <f>'August '!H44</f>
-        <v>2.6666666666666661</v>
+        <v>2.8749999999999996</v>
       </c>
     </row>
     <row r="43" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -14622,7 +14628,7 @@
       <c r="G43" s="15"/>
       <c r="H43" s="38">
         <f>H41-H40+H42</f>
-        <v>2.6666666666666661</v>
+        <v>2.8749999999999996</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
@@ -14640,6 +14646,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -14649,11 +14660,6 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">

</xml_diff>

<commit_message>
cleaning and organizing the data
</commit_message>
<xml_diff>
--- a/HK Zeiterfassung 2026.xlsx
+++ b/HK Zeiterfassung 2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr date1904="1" codeName="DieseArbeitsmappe"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harik\Downloads\Computational Chemistry\Variant-Effect-Predictor-for-nAChRs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7416644-C04C-4EE9-83FD-0350D2C8DDB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CA6153E-716B-457E-8D92-20952AC793AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28980" yWindow="2220" windowWidth="18165" windowHeight="10290" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Januar " sheetId="26" r:id="rId1"/>
@@ -31,15 +31,6 @@
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -2489,46 +2480,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="3" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="17" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="17" fontId="0" fillId="3" borderId="17" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -2591,6 +2542,61 @@
       <alignment horizontal="right"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="17" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="17" fontId="0" fillId="3" borderId="17" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2613,21 +2619,6 @@
     <xf numFmtId="166" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2923,98 +2914,98 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="72"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="62"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="73" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="74"/>
-      <c r="C2" s="75" t="s">
+      <c r="A2" s="63" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="64"/>
+      <c r="C2" s="65" t="s">
         <v>408</v>
       </c>
-      <c r="D2" s="75"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="77" t="s">
+      <c r="D2" s="65"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="74"/>
+      <c r="G2" s="64"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="78" t="s">
+      <c r="I2" s="68" t="s">
         <v>407</v>
       </c>
-      <c r="J2" s="79"/>
+      <c r="J2" s="69"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="64" t="s">
+      <c r="B3" s="53"/>
+      <c r="C3" s="54" t="s">
         <v>408</v>
       </c>
-      <c r="D3" s="64"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="66" t="s">
+      <c r="D3" s="54"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="67"/>
+      <c r="G3" s="57"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="68">
+      <c r="I3" s="58">
         <v>2026</v>
       </c>
-      <c r="J3" s="69"/>
+      <c r="J3" s="59"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="52" t="s">
+      <c r="C4" s="70" t="s">
         <v>408</v>
       </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="53"/>
+      <c r="D4" s="70"/>
+      <c r="E4" s="71"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="54" t="s">
+      <c r="I4" s="72" t="s">
         <v>408</v>
       </c>
-      <c r="J4" s="55"/>
+      <c r="J4" s="73"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="56" t="s">
+      <c r="C5" s="74" t="s">
         <v>408</v>
       </c>
-      <c r="D5" s="56"/>
-      <c r="E5" s="57"/>
+      <c r="D5" s="74"/>
+      <c r="E5" s="75"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="58" t="s">
+      <c r="I5" s="76" t="s">
         <v>409</v>
       </c>
-      <c r="J5" s="59"/>
+      <c r="J5" s="77"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -3027,10 +3018,10 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="60" t="s">
+      <c r="I6" s="78" t="s">
         <v>409</v>
       </c>
-      <c r="J6" s="61"/>
+      <c r="J6" s="79"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -3819,6 +3810,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -3828,11 +3824,6 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -3863,104 +3854,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="72"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="62"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="73" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="74"/>
-      <c r="C2" s="75" t="str">
+      <c r="A2" s="63" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="64"/>
+      <c r="C2" s="65" t="str">
         <f>September!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="75"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="77" t="s">
+      <c r="D2" s="65"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="74"/>
+      <c r="G2" s="64"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="78" t="s">
+      <c r="I2" s="68" t="s">
         <v>311</v>
       </c>
-      <c r="J2" s="79"/>
+      <c r="J2" s="69"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="64" t="str">
+      <c r="B3" s="53"/>
+      <c r="C3" s="54" t="str">
         <f>September!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="64"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="66" t="s">
+      <c r="D3" s="54"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="67"/>
+      <c r="G3" s="57"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="68">
+      <c r="I3" s="58">
         <v>2026</v>
       </c>
-      <c r="J3" s="69"/>
+      <c r="J3" s="59"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="52" t="str">
+      <c r="C4" s="70" t="str">
         <f>September!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="53"/>
+      <c r="D4" s="70"/>
+      <c r="E4" s="71"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="54" t="str">
+      <c r="I4" s="72" t="str">
         <f>September!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="55"/>
+      <c r="J4" s="73"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="56" t="str">
+      <c r="C5" s="74" t="str">
         <f>September!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="56"/>
-      <c r="E5" s="57"/>
+      <c r="D5" s="74"/>
+      <c r="E5" s="75"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="58">
+      <c r="I5" s="76">
         <f>September!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="59"/>
+      <c r="J5" s="77"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -3973,11 +3964,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="60" t="str">
+      <c r="I6" s="78" t="str">
         <f>September!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="61"/>
+      <c r="J6" s="79"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -4734,7 +4725,7 @@
       <c r="F43" s="1"/>
       <c r="H43" s="34">
         <f>September!H43</f>
-        <v>3.1458333333333326</v>
+        <v>3.4374999999999991</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -4749,7 +4740,7 @@
       <c r="G44" s="15"/>
       <c r="H44" s="38">
         <f>H42-H41+H43</f>
-        <v>3.1458333333333326</v>
+        <v>3.4374999999999991</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
@@ -4767,6 +4758,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -4776,11 +4772,6 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -4811,104 +4802,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="72"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="62"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="73" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="74"/>
-      <c r="C2" s="75" t="str">
+      <c r="A2" s="63" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="64"/>
+      <c r="C2" s="65" t="str">
         <f>'Oktober '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="75"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="77" t="s">
+      <c r="D2" s="65"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="74"/>
+      <c r="G2" s="64"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="78" t="s">
+      <c r="I2" s="68" t="s">
         <v>343</v>
       </c>
-      <c r="J2" s="79"/>
+      <c r="J2" s="69"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="64" t="str">
+      <c r="B3" s="53"/>
+      <c r="C3" s="54" t="str">
         <f>'Oktober '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="64"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="66" t="s">
+      <c r="D3" s="54"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="67"/>
+      <c r="G3" s="57"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="68">
+      <c r="I3" s="58">
         <v>2026</v>
       </c>
-      <c r="J3" s="69"/>
+      <c r="J3" s="59"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="52" t="str">
+      <c r="C4" s="70" t="str">
         <f>'Oktober '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="53"/>
+      <c r="D4" s="70"/>
+      <c r="E4" s="71"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="54" t="str">
+      <c r="I4" s="72" t="str">
         <f>'Oktober '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="55"/>
+      <c r="J4" s="73"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="56" t="str">
+      <c r="C5" s="74" t="str">
         <f>'Oktober '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="56"/>
-      <c r="E5" s="57"/>
+      <c r="D5" s="74"/>
+      <c r="E5" s="75"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="58">
+      <c r="I5" s="76">
         <f>'Oktober '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="59"/>
+      <c r="J5" s="77"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -4921,11 +4912,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="60" t="str">
+      <c r="I6" s="78" t="str">
         <f>'Oktober '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="61"/>
+      <c r="J6" s="79"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -5661,7 +5652,7 @@
       <c r="F42" s="1"/>
       <c r="H42" s="34">
         <f>'Oktober '!H44</f>
-        <v>3.1458333333333326</v>
+        <v>3.4374999999999991</v>
       </c>
     </row>
     <row r="43" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -5676,7 +5667,7 @@
       <c r="G43" s="15"/>
       <c r="H43" s="38">
         <f>H41-H40+H42</f>
-        <v>3.1458333333333326</v>
+        <v>3.4374999999999991</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
@@ -5694,6 +5685,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -5703,11 +5699,6 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -5738,104 +5729,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="72"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="62"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="73" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="74"/>
-      <c r="C2" s="75" t="str">
+      <c r="A2" s="63" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="64"/>
+      <c r="C2" s="65" t="str">
         <f>'November '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="75"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="77" t="s">
+      <c r="D2" s="65"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="74"/>
+      <c r="G2" s="64"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="78" t="s">
+      <c r="I2" s="68" t="s">
         <v>374</v>
       </c>
-      <c r="J2" s="79"/>
+      <c r="J2" s="69"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="64" t="str">
+      <c r="B3" s="53"/>
+      <c r="C3" s="54" t="str">
         <f>'November '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="64"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="66" t="s">
+      <c r="D3" s="54"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="67"/>
+      <c r="G3" s="57"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="68">
+      <c r="I3" s="58">
         <v>2026</v>
       </c>
-      <c r="J3" s="69"/>
+      <c r="J3" s="59"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="52" t="str">
+      <c r="C4" s="70" t="str">
         <f>'November '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="53"/>
+      <c r="D4" s="70"/>
+      <c r="E4" s="71"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="54" t="str">
+      <c r="I4" s="72" t="str">
         <f>'November '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="55"/>
+      <c r="J4" s="73"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="56" t="str">
+      <c r="C5" s="74" t="str">
         <f>'November '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="56"/>
-      <c r="E5" s="57"/>
+      <c r="D5" s="74"/>
+      <c r="E5" s="75"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="58">
+      <c r="I5" s="76">
         <f>'November '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="59"/>
+      <c r="J5" s="77"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -5848,11 +5839,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="60" t="str">
+      <c r="I6" s="78" t="str">
         <f>'November '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="61"/>
+      <c r="J6" s="79"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -6609,7 +6600,7 @@
       <c r="F43" s="1"/>
       <c r="H43" s="34">
         <f>'November '!H43</f>
-        <v>3.1458333333333326</v>
+        <v>3.4374999999999991</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -6624,7 +6615,7 @@
       <c r="G44" s="15"/>
       <c r="H44" s="38">
         <f>H42-H41+H43</f>
-        <v>3.1458333333333326</v>
+        <v>3.4374999999999991</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
@@ -6642,6 +6633,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -6651,11 +6647,6 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -6687,22 +6678,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="80" t="s">
+      <c r="A1" s="85" t="s">
         <v>416</v>
       </c>
-      <c r="B1" s="81"/>
-      <c r="C1" s="81"/>
-      <c r="D1" s="81"/>
-      <c r="E1" s="81"/>
-      <c r="F1" s="81"/>
-      <c r="G1" s="81"/>
-      <c r="H1" s="82"/>
+      <c r="B1" s="86"/>
+      <c r="C1" s="86"/>
+      <c r="D1" s="86"/>
+      <c r="E1" s="86"/>
+      <c r="F1" s="86"/>
+      <c r="G1" s="86"/>
+      <c r="H1" s="87"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="62" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="63"/>
+      <c r="A2" s="52" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="53"/>
       <c r="C2" s="47" t="str">
         <f>'November '!C2:E2</f>
         <v>Hari Krishna</v>
@@ -6711,15 +6702,15 @@
       <c r="E2" s="22" t="s">
         <v>418</v>
       </c>
-      <c r="F2" s="86"/>
-      <c r="G2" s="86"/>
+      <c r="F2" s="91"/>
+      <c r="G2" s="91"/>
       <c r="H2" s="48"/>
     </row>
     <row r="3" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="89" t="s">
+      <c r="A3" s="82" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="67"/>
+      <c r="B3" s="57"/>
       <c r="C3" s="49" t="str">
         <f>'November '!C3:E3</f>
         <v>Mohan Raj</v>
@@ -6728,8 +6719,8 @@
       <c r="E3" s="18" t="s">
         <v>122</v>
       </c>
-      <c r="F3" s="68"/>
-      <c r="G3" s="68"/>
+      <c r="F3" s="58"/>
+      <c r="G3" s="58"/>
       <c r="H3" s="50"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
@@ -6743,17 +6734,17 @@
       </c>
     </row>
     <row r="6" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="84" t="s">
+      <c r="A6" s="89" t="s">
         <v>417</v>
       </c>
-      <c r="B6" s="85"/>
-      <c r="C6" s="83" t="s">
+      <c r="B6" s="90"/>
+      <c r="C6" s="88" t="s">
         <v>419</v>
       </c>
-      <c r="D6" s="83"/>
-      <c r="E6" s="83"/>
-      <c r="F6" s="83"/>
-      <c r="G6" s="83"/>
+      <c r="D6" s="88"/>
+      <c r="E6" s="88"/>
+      <c r="F6" s="88"/>
+      <c r="G6" s="88"/>
       <c r="H6" s="51"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
@@ -6765,10 +6756,10 @@
       <c r="D8" s="3"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A9" s="87" t="s">
+      <c r="A9" s="80" t="s">
         <v>410</v>
       </c>
-      <c r="B9" s="88"/>
+      <c r="B9" s="81"/>
       <c r="C9" s="44" t="s">
         <v>411</v>
       </c>
@@ -6784,10 +6775,10 @@
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A10" s="90" t="s">
+      <c r="A10" s="83" t="s">
         <v>407</v>
       </c>
-      <c r="B10" s="91"/>
+      <c r="B10" s="84"/>
       <c r="C10" s="46">
         <f>'Januar '!H41</f>
         <v>0</v>
@@ -6806,10 +6797,10 @@
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A11" s="90" t="s">
+      <c r="A11" s="83" t="s">
         <v>406</v>
       </c>
-      <c r="B11" s="91"/>
+      <c r="B11" s="84"/>
       <c r="C11" s="46">
         <f>'Februar '!H39</f>
         <v>0</v>
@@ -6829,10 +6820,10 @@
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A12" s="90" t="s">
+      <c r="A12" s="83" t="s">
         <v>89</v>
       </c>
-      <c r="B12" s="91"/>
+      <c r="B12" s="84"/>
       <c r="C12" s="46">
         <f>'März '!H41</f>
         <v>0</v>
@@ -6853,10 +6844,10 @@
       <c r="M12" s="28"/>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A13" s="90" t="s">
+      <c r="A13" s="83" t="s">
         <v>121</v>
       </c>
-      <c r="B13" s="91"/>
+      <c r="B13" s="84"/>
       <c r="C13" s="46">
         <f>'April '!H40</f>
         <v>0</v>
@@ -6876,17 +6867,17 @@
       </c>
     </row>
     <row r="14" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="90" t="s">
+      <c r="A14" s="83" t="s">
         <v>185</v>
       </c>
-      <c r="B14" s="91"/>
+      <c r="B14" s="84"/>
       <c r="C14" s="46">
         <f>'Mai '!H41</f>
         <v>0</v>
       </c>
       <c r="D14" s="46">
         <f>'Mai '!H42</f>
-        <v>0.47916666666666652</v>
+        <v>0.77083333333333326</v>
       </c>
       <c r="E14" s="46">
         <f>'Mai '!H43</f>
@@ -6895,14 +6886,14 @@
       <c r="F14" s="46"/>
       <c r="G14" s="46">
         <f>'Mai '!H44</f>
-        <v>3.1458333333333326</v>
+        <v>3.4374999999999991</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A15" s="90" t="s">
+      <c r="A15" s="83" t="s">
         <v>184</v>
       </c>
-      <c r="B15" s="91"/>
+      <c r="B15" s="84"/>
       <c r="C15" s="46">
         <f>'Juni '!H40</f>
         <v>0</v>
@@ -6913,19 +6904,19 @@
       </c>
       <c r="E15" s="46">
         <f>'Juni '!H42</f>
-        <v>3.1458333333333326</v>
+        <v>3.4374999999999991</v>
       </c>
       <c r="F15" s="46"/>
       <c r="G15" s="46">
         <f>'Juni '!H43</f>
-        <v>3.1458333333333326</v>
+        <v>3.4374999999999991</v>
       </c>
     </row>
     <row r="16" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="90" t="s">
+      <c r="A16" s="83" t="s">
         <v>247</v>
       </c>
-      <c r="B16" s="91"/>
+      <c r="B16" s="84"/>
       <c r="C16" s="46">
         <f>'Juli '!H41</f>
         <v>0</v>
@@ -6936,19 +6927,19 @@
       </c>
       <c r="E16" s="46">
         <f>'Juli '!H43</f>
-        <v>3.1458333333333326</v>
+        <v>3.4374999999999991</v>
       </c>
       <c r="F16" s="46"/>
       <c r="G16" s="46">
         <f>'Juli '!H44</f>
-        <v>3.1458333333333326</v>
+        <v>3.4374999999999991</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="90" t="s">
+      <c r="A17" s="83" t="s">
         <v>248</v>
       </c>
-      <c r="B17" s="91"/>
+      <c r="B17" s="84"/>
       <c r="C17" s="46">
         <f>'August '!H41</f>
         <v>0</v>
@@ -6959,19 +6950,19 @@
       </c>
       <c r="E17" s="46">
         <f>'August '!H43</f>
-        <v>3.1458333333333326</v>
+        <v>3.4374999999999991</v>
       </c>
       <c r="F17" s="46"/>
       <c r="G17" s="46">
         <f>'August '!H44</f>
-        <v>3.1458333333333326</v>
+        <v>3.4374999999999991</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="90" t="s">
+      <c r="A18" s="83" t="s">
         <v>280</v>
       </c>
-      <c r="B18" s="91"/>
+      <c r="B18" s="84"/>
       <c r="C18" s="46">
         <f>September!H40</f>
         <v>0</v>
@@ -6982,19 +6973,19 @@
       </c>
       <c r="E18" s="46">
         <f>September!H42</f>
-        <v>3.1458333333333326</v>
+        <v>3.4374999999999991</v>
       </c>
       <c r="F18" s="46"/>
       <c r="G18" s="46">
         <f>September!H43</f>
-        <v>3.1458333333333326</v>
+        <v>3.4374999999999991</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="90" t="s">
+      <c r="A19" s="83" t="s">
         <v>311</v>
       </c>
-      <c r="B19" s="91"/>
+      <c r="B19" s="84"/>
       <c r="C19" s="46">
         <f>'Oktober '!H41</f>
         <v>0</v>
@@ -7005,19 +6996,19 @@
       </c>
       <c r="E19" s="46">
         <f>'Oktober '!H43</f>
-        <v>3.1458333333333326</v>
+        <v>3.4374999999999991</v>
       </c>
       <c r="F19" s="46"/>
       <c r="G19" s="46">
         <f>'Oktober '!H44</f>
-        <v>3.1458333333333326</v>
+        <v>3.4374999999999991</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="90" t="s">
+      <c r="A20" s="83" t="s">
         <v>343</v>
       </c>
-      <c r="B20" s="91"/>
+      <c r="B20" s="84"/>
       <c r="C20" s="46">
         <f>'November '!H40</f>
         <v>0</v>
@@ -7028,19 +7019,19 @@
       </c>
       <c r="E20" s="46">
         <f>'November '!H42</f>
-        <v>3.1458333333333326</v>
+        <v>3.4374999999999991</v>
       </c>
       <c r="F20" s="46"/>
       <c r="G20" s="46">
         <f>'November '!H43</f>
-        <v>3.1458333333333326</v>
+        <v>3.4374999999999991</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="90" t="s">
+      <c r="A21" s="83" t="s">
         <v>374</v>
       </c>
-      <c r="B21" s="91"/>
+      <c r="B21" s="84"/>
       <c r="C21" s="46">
         <f>'Dezember '!H41</f>
         <v>0</v>
@@ -7051,12 +7042,12 @@
       </c>
       <c r="E21" s="46">
         <f>'Dezember '!H43</f>
-        <v>3.1458333333333326</v>
+        <v>3.4374999999999991</v>
       </c>
       <c r="F21" s="46"/>
       <c r="G21" s="46">
         <f>'Dezember '!H44</f>
-        <v>3.1458333333333326</v>
+        <v>3.4374999999999991</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
@@ -7093,6 +7084,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="20">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="C6:G6"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="F3:G3"/>
     <mergeCell ref="A9:B9"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A3:B3"/>
@@ -7108,11 +7104,6 @@
     <mergeCell ref="A17:B17"/>
     <mergeCell ref="A18:B18"/>
     <mergeCell ref="A19:B19"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="C6:G6"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="F3:G3"/>
   </mergeCells>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.39370078740157483" bottom="0.39370078740157483" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -7135,104 +7126,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="72"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="62"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="73" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="74"/>
-      <c r="C2" s="75" t="str">
+      <c r="A2" s="63" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="64"/>
+      <c r="C2" s="65" t="str">
         <f>'Januar '!C2:E2</f>
         <v>XXX</v>
       </c>
-      <c r="D2" s="75"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="77" t="s">
+      <c r="D2" s="65"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="74"/>
+      <c r="G2" s="64"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="78" t="s">
+      <c r="I2" s="68" t="s">
         <v>406</v>
       </c>
-      <c r="J2" s="79"/>
+      <c r="J2" s="69"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="64" t="str">
+      <c r="B3" s="53"/>
+      <c r="C3" s="54" t="str">
         <f>'Januar '!C3:E3</f>
         <v>XXX</v>
       </c>
-      <c r="D3" s="64"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="66" t="s">
+      <c r="D3" s="54"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="67"/>
+      <c r="G3" s="57"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="68">
+      <c r="I3" s="58">
         <v>2026</v>
       </c>
-      <c r="J3" s="69"/>
+      <c r="J3" s="59"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="52" t="str">
+      <c r="C4" s="70" t="str">
         <f>'Januar '!C4:E4</f>
         <v>XXX</v>
       </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="53"/>
+      <c r="D4" s="70"/>
+      <c r="E4" s="71"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="54" t="str">
+      <c r="I4" s="72" t="str">
         <f>'Januar '!I4:J4</f>
         <v>XXX</v>
       </c>
-      <c r="J4" s="55"/>
+      <c r="J4" s="73"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="56" t="str">
+      <c r="C5" s="74" t="str">
         <f>'Januar '!C5:E5</f>
         <v>XXX</v>
       </c>
-      <c r="D5" s="56"/>
-      <c r="E5" s="57"/>
+      <c r="D5" s="74"/>
+      <c r="E5" s="75"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="58" t="str">
+      <c r="I5" s="76" t="str">
         <f>'Januar '!I5:J5</f>
         <v>XX</v>
       </c>
-      <c r="J5" s="59"/>
+      <c r="J5" s="77"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -7245,11 +7236,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="60" t="str">
+      <c r="I6" s="78" t="str">
         <f>'Januar '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="61"/>
+      <c r="J6" s="79"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -7985,6 +7976,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -7994,11 +7990,6 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -8029,98 +8020,98 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="72"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="62"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="73" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="74"/>
-      <c r="C2" s="75" t="s">
+      <c r="A2" s="63" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="64"/>
+      <c r="C2" s="65" t="s">
         <v>420</v>
       </c>
-      <c r="D2" s="75"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="77" t="s">
+      <c r="D2" s="65"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="74"/>
+      <c r="G2" s="64"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="78" t="s">
+      <c r="I2" s="68" t="s">
         <v>89</v>
       </c>
-      <c r="J2" s="79"/>
+      <c r="J2" s="69"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="64" t="s">
+      <c r="B3" s="53"/>
+      <c r="C3" s="54" t="s">
         <v>421</v>
       </c>
-      <c r="D3" s="64"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="66" t="s">
+      <c r="D3" s="54"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="67"/>
+      <c r="G3" s="57"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="68">
+      <c r="I3" s="58">
         <v>2026</v>
       </c>
-      <c r="J3" s="69"/>
+      <c r="J3" s="59"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="52" t="s">
+      <c r="C4" s="70" t="s">
         <v>422</v>
       </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="53"/>
+      <c r="D4" s="70"/>
+      <c r="E4" s="71"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="54" t="s">
+      <c r="I4" s="72" t="s">
         <v>424</v>
       </c>
-      <c r="J4" s="55"/>
+      <c r="J4" s="73"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="56" t="s">
+      <c r="C5" s="74" t="s">
         <v>423</v>
       </c>
-      <c r="D5" s="56"/>
-      <c r="E5" s="57"/>
+      <c r="D5" s="74"/>
+      <c r="E5" s="75"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="58">
+      <c r="I5" s="76">
         <v>8</v>
       </c>
-      <c r="J5" s="59"/>
+      <c r="J5" s="77"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -8133,11 +8124,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="60" t="str">
+      <c r="I6" s="78" t="str">
         <f>'Februar '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="61"/>
+      <c r="J6" s="79"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -8976,6 +8967,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -8985,11 +8981,6 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -9020,104 +9011,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="72"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="62"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="73" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="74"/>
-      <c r="C2" s="75" t="str">
+      <c r="A2" s="63" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="64"/>
+      <c r="C2" s="65" t="str">
         <f>'März '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="75"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="77" t="s">
+      <c r="D2" s="65"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="74"/>
+      <c r="G2" s="64"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="78" t="s">
+      <c r="I2" s="68" t="s">
         <v>121</v>
       </c>
-      <c r="J2" s="79"/>
+      <c r="J2" s="69"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="64" t="str">
+      <c r="B3" s="53"/>
+      <c r="C3" s="54" t="str">
         <f>'März '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="64"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="66" t="s">
+      <c r="D3" s="54"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="67"/>
+      <c r="G3" s="57"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="68">
+      <c r="I3" s="58">
         <v>2026</v>
       </c>
-      <c r="J3" s="69"/>
+      <c r="J3" s="59"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="52" t="str">
+      <c r="C4" s="70" t="str">
         <f>'März '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="53"/>
+      <c r="D4" s="70"/>
+      <c r="E4" s="71"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="54" t="str">
+      <c r="I4" s="72" t="str">
         <f>'März '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="55"/>
+      <c r="J4" s="73"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="56" t="str">
+      <c r="C5" s="74" t="str">
         <f>'März '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="56"/>
-      <c r="E5" s="57"/>
+      <c r="D5" s="74"/>
+      <c r="E5" s="75"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="58">
+      <c r="I5" s="76">
         <f>'März '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="59"/>
+      <c r="J5" s="77"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -9130,11 +9121,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="60" t="str">
+      <c r="I6" s="78" t="str">
         <f>'März '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="61"/>
+      <c r="J6" s="79"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -9944,6 +9935,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -9953,11 +9949,6 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -9988,104 +9979,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="72"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="62"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="73" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="74"/>
-      <c r="C2" s="75" t="str">
+      <c r="A2" s="63" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="64"/>
+      <c r="C2" s="65" t="str">
         <f>'April '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="75"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="77" t="s">
+      <c r="D2" s="65"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="74"/>
+      <c r="G2" s="64"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="78" t="s">
+      <c r="I2" s="68" t="s">
         <v>185</v>
       </c>
-      <c r="J2" s="79"/>
+      <c r="J2" s="69"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="64" t="str">
+      <c r="B3" s="53"/>
+      <c r="C3" s="54" t="str">
         <f>'April '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="64"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="66" t="s">
+      <c r="D3" s="54"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="67"/>
+      <c r="G3" s="57"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="68">
+      <c r="I3" s="58">
         <v>2026</v>
       </c>
-      <c r="J3" s="69"/>
+      <c r="J3" s="59"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="52" t="str">
+      <c r="C4" s="70" t="str">
         <f>'April '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="53"/>
+      <c r="D4" s="70"/>
+      <c r="E4" s="71"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="54" t="str">
+      <c r="I4" s="72" t="str">
         <f>'April '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="55"/>
+      <c r="J4" s="73"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="56" t="str">
+      <c r="C5" s="74" t="str">
         <f>'April '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="56"/>
-      <c r="E5" s="57"/>
+      <c r="D5" s="74"/>
+      <c r="E5" s="75"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="58">
+      <c r="I5" s="76">
         <f>'April '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="59"/>
+      <c r="J5" s="77"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -10098,11 +10089,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="60" t="str">
+      <c r="I6" s="78" t="str">
         <f>'April '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="61"/>
+      <c r="J6" s="79"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -10236,16 +10227,20 @@
         <v>13</v>
       </c>
       <c r="C13" s="32"/>
-      <c r="D13" s="29"/>
-      <c r="E13" s="29"/>
+      <c r="D13" s="29">
+        <v>0.625</v>
+      </c>
+      <c r="E13" s="29">
+        <v>0.75</v>
+      </c>
       <c r="F13" s="29"/>
       <c r="G13" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="H13" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="I13" s="30"/>
       <c r="J13" s="31"/>
@@ -10624,16 +10619,20 @@
         <v>16</v>
       </c>
       <c r="C30" s="32"/>
-      <c r="D30" s="29"/>
-      <c r="E30" s="29"/>
+      <c r="D30" s="29">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="E30" s="29">
+        <v>0.70833333333333337</v>
+      </c>
       <c r="F30" s="29"/>
       <c r="G30" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.16666666666666674</v>
       </c>
       <c r="H30" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.16666666666666674</v>
       </c>
       <c r="I30" s="30"/>
       <c r="J30" s="31"/>
@@ -10862,7 +10861,7 @@
       <c r="F42" s="1"/>
       <c r="H42" s="34">
         <f>SUM(H9:H39)</f>
-        <v>0.47916666666666652</v>
+        <v>0.77083333333333326</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
@@ -10888,7 +10887,7 @@
       <c r="G44" s="15"/>
       <c r="H44" s="38">
         <f>H42-H41+H43</f>
-        <v>3.1458333333333326</v>
+        <v>3.4374999999999991</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
@@ -10906,6 +10905,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -10915,11 +10919,6 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -10950,104 +10949,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="72"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="62"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="73" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="74"/>
-      <c r="C2" s="75" t="str">
+      <c r="A2" s="63" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="64"/>
+      <c r="C2" s="65" t="str">
         <f>'Mai '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="75"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="77" t="s">
+      <c r="D2" s="65"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="74"/>
+      <c r="G2" s="64"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="78" t="s">
+      <c r="I2" s="68" t="s">
         <v>184</v>
       </c>
-      <c r="J2" s="79"/>
+      <c r="J2" s="69"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="64" t="str">
+      <c r="B3" s="53"/>
+      <c r="C3" s="54" t="str">
         <f>'Mai '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="64"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="66" t="s">
+      <c r="D3" s="54"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="67"/>
+      <c r="G3" s="57"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="68">
+      <c r="I3" s="58">
         <v>2026</v>
       </c>
-      <c r="J3" s="69"/>
+      <c r="J3" s="59"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="52" t="str">
+      <c r="C4" s="70" t="str">
         <f>'Mai '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="53"/>
+      <c r="D4" s="70"/>
+      <c r="E4" s="71"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="54" t="str">
+      <c r="I4" s="72" t="str">
         <f>'Mai '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="55"/>
+      <c r="J4" s="73"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="56" t="str">
+      <c r="C5" s="74" t="str">
         <f>'Mai '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="56"/>
-      <c r="E5" s="57"/>
+      <c r="D5" s="74"/>
+      <c r="E5" s="75"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="58">
+      <c r="I5" s="76">
         <f>'Mai '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="59"/>
+      <c r="J5" s="77"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -11060,11 +11059,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="60" t="str">
+      <c r="I6" s="78" t="str">
         <f>'Mai '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="61"/>
+      <c r="J6" s="79"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -11799,7 +11798,7 @@
       <c r="F42" s="1"/>
       <c r="H42" s="34">
         <f>'Mai '!H44</f>
-        <v>3.1458333333333326</v>
+        <v>3.4374999999999991</v>
       </c>
     </row>
     <row r="43" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -11814,7 +11813,7 @@
       <c r="G43" s="15"/>
       <c r="H43" s="38">
         <f>H41-H40+H42</f>
-        <v>3.1458333333333326</v>
+        <v>3.4374999999999991</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
@@ -11832,6 +11831,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -11841,11 +11845,6 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -11876,104 +11875,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="72"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="62"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="73" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="74"/>
-      <c r="C2" s="75" t="str">
+      <c r="A2" s="63" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="64"/>
+      <c r="C2" s="65" t="str">
         <f>'Juni '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="75"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="77" t="s">
+      <c r="D2" s="65"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="74"/>
+      <c r="G2" s="64"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="78" t="s">
+      <c r="I2" s="68" t="s">
         <v>247</v>
       </c>
-      <c r="J2" s="79"/>
+      <c r="J2" s="69"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="64" t="str">
+      <c r="B3" s="53"/>
+      <c r="C3" s="54" t="str">
         <f>'Juni '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="64"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="66" t="s">
+      <c r="D3" s="54"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="67"/>
+      <c r="G3" s="57"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="68">
+      <c r="I3" s="58">
         <v>2026</v>
       </c>
-      <c r="J3" s="69"/>
+      <c r="J3" s="59"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="52" t="str">
+      <c r="C4" s="70" t="str">
         <f>'Juni '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="53"/>
+      <c r="D4" s="70"/>
+      <c r="E4" s="71"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="54" t="str">
+      <c r="I4" s="72" t="str">
         <f>'Juni '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="55"/>
+      <c r="J4" s="73"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="56" t="str">
+      <c r="C5" s="74" t="str">
         <f>'Juni '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="56"/>
-      <c r="E5" s="57"/>
+      <c r="D5" s="74"/>
+      <c r="E5" s="75"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="58">
+      <c r="I5" s="76">
         <f>'Juni '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="59"/>
+      <c r="J5" s="77"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -11986,11 +11985,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="60" t="str">
+      <c r="I6" s="78" t="str">
         <f>'Juni '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="61"/>
+      <c r="J6" s="79"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -12747,7 +12746,7 @@
       <c r="F43" s="1"/>
       <c r="H43" s="34">
         <f>'Juni '!H43</f>
-        <v>3.1458333333333326</v>
+        <v>3.4374999999999991</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -12762,7 +12761,7 @@
       <c r="G44" s="15"/>
       <c r="H44" s="38">
         <f>H42-H41+H43</f>
-        <v>3.1458333333333326</v>
+        <v>3.4374999999999991</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
@@ -12780,6 +12779,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -12789,11 +12793,6 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -12824,104 +12823,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="72"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="62"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="73" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="74"/>
-      <c r="C2" s="75" t="str">
+      <c r="A2" s="63" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="64"/>
+      <c r="C2" s="65" t="str">
         <f>'Juli '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="75"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="77" t="s">
+      <c r="D2" s="65"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="74"/>
+      <c r="G2" s="64"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="78" t="s">
+      <c r="I2" s="68" t="s">
         <v>248</v>
       </c>
-      <c r="J2" s="79"/>
+      <c r="J2" s="69"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="64" t="str">
+      <c r="B3" s="53"/>
+      <c r="C3" s="54" t="str">
         <f>'Juli '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="64"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="66" t="s">
+      <c r="D3" s="54"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="67"/>
+      <c r="G3" s="57"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="68">
+      <c r="I3" s="58">
         <v>2026</v>
       </c>
-      <c r="J3" s="69"/>
+      <c r="J3" s="59"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="52" t="str">
+      <c r="C4" s="70" t="str">
         <f>'Juli '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="53"/>
+      <c r="D4" s="70"/>
+      <c r="E4" s="71"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="54" t="str">
+      <c r="I4" s="72" t="str">
         <f>'Juli '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="55"/>
+      <c r="J4" s="73"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="56" t="str">
+      <c r="C5" s="74" t="str">
         <f>'Juli '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="56"/>
-      <c r="E5" s="57"/>
+      <c r="D5" s="74"/>
+      <c r="E5" s="75"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="58">
+      <c r="I5" s="76">
         <f>'Juli '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="59"/>
+      <c r="J5" s="77"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -12934,11 +12933,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="60" t="str">
+      <c r="I6" s="78" t="str">
         <f>'Juli '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="61"/>
+      <c r="J6" s="79"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -13695,7 +13694,7 @@
       <c r="F43" s="1"/>
       <c r="H43" s="34">
         <f>'Juli '!H44</f>
-        <v>3.1458333333333326</v>
+        <v>3.4374999999999991</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -13710,7 +13709,7 @@
       <c r="G44" s="15"/>
       <c r="H44" s="38">
         <f>H42-H41+H43</f>
-        <v>3.1458333333333326</v>
+        <v>3.4374999999999991</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
@@ -13728,6 +13727,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -13737,11 +13741,6 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -13772,104 +13771,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="72"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="62"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="73" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="74"/>
-      <c r="C2" s="75" t="str">
+      <c r="A2" s="63" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="64"/>
+      <c r="C2" s="65" t="str">
         <f>'August '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="75"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="77" t="s">
+      <c r="D2" s="65"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="74"/>
+      <c r="G2" s="64"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="78" t="s">
+      <c r="I2" s="68" t="s">
         <v>280</v>
       </c>
-      <c r="J2" s="79"/>
+      <c r="J2" s="69"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="64" t="str">
+      <c r="B3" s="53"/>
+      <c r="C3" s="54" t="str">
         <f>'August '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="64"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="66" t="s">
+      <c r="D3" s="54"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="67"/>
+      <c r="G3" s="57"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="68">
+      <c r="I3" s="58">
         <v>2026</v>
       </c>
-      <c r="J3" s="69"/>
+      <c r="J3" s="59"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="52" t="str">
+      <c r="C4" s="70" t="str">
         <f>'August '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="53"/>
+      <c r="D4" s="70"/>
+      <c r="E4" s="71"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="54" t="str">
+      <c r="I4" s="72" t="str">
         <f>'August '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="55"/>
+      <c r="J4" s="73"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="56" t="str">
+      <c r="C5" s="74" t="str">
         <f>'August '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="56"/>
-      <c r="E5" s="57"/>
+      <c r="D5" s="74"/>
+      <c r="E5" s="75"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="58">
+      <c r="I5" s="76">
         <f>'August '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="59"/>
+      <c r="J5" s="77"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -13882,11 +13881,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="60" t="str">
+      <c r="I6" s="78" t="str">
         <f>'August '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="61"/>
+      <c r="J6" s="79"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -14621,7 +14620,7 @@
       <c r="F42" s="1"/>
       <c r="H42" s="34">
         <f>'August '!H44</f>
-        <v>3.1458333333333326</v>
+        <v>3.4374999999999991</v>
       </c>
     </row>
     <row r="43" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -14636,7 +14635,7 @@
       <c r="G43" s="15"/>
       <c r="H43" s="38">
         <f>H41-H40+H42</f>
-        <v>3.1458333333333326</v>
+        <v>3.4374999999999991</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
@@ -14654,6 +14653,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -14663,11 +14667,6 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">

</xml_diff>

<commit_message>
nachr skeleton with AA features and data scraper initial model for scraping muose mutation data
</commit_message>
<xml_diff>
--- a/HK Zeiterfassung 2026.xlsx
+++ b/HK Zeiterfassung 2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harik\Downloads\Computational Chemistry\Variant-Effect-Predictor-for-nAChRs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CA6153E-716B-457E-8D92-20952AC793AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66285D0A-43C7-4BAB-9EE3-97FB309787BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28980" yWindow="2220" windowWidth="18165" windowHeight="10290" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9720" yWindow="5190" windowWidth="18165" windowHeight="11130" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Januar " sheetId="26" r:id="rId1"/>
@@ -31,6 +31,15 @@
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -2480,6 +2489,46 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="17" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="17" fontId="0" fillId="3" borderId="17" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -2542,61 +2591,6 @@
       <alignment horizontal="right"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="3" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="17" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="17" fontId="0" fillId="3" borderId="17" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2619,6 +2613,21 @@
     <xf numFmtId="166" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2914,98 +2923,98 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="60" t="s">
+      <c r="A1" s="70" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="62"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="72"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="65" t="s">
+      <c r="A2" s="73" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="74"/>
+      <c r="C2" s="75" t="s">
         <v>408</v>
       </c>
-      <c r="D2" s="65"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="67" t="s">
+      <c r="D2" s="75"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="64"/>
+      <c r="G2" s="74"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="68" t="s">
+      <c r="I2" s="78" t="s">
         <v>407</v>
       </c>
-      <c r="J2" s="69"/>
+      <c r="J2" s="79"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="54" t="s">
+      <c r="B3" s="63"/>
+      <c r="C3" s="64" t="s">
         <v>408</v>
       </c>
-      <c r="D3" s="54"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="56" t="s">
+      <c r="D3" s="64"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="57"/>
+      <c r="G3" s="67"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="58">
+      <c r="I3" s="68">
         <v>2026</v>
       </c>
-      <c r="J3" s="59"/>
+      <c r="J3" s="69"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="70" t="s">
+      <c r="C4" s="52" t="s">
         <v>408</v>
       </c>
-      <c r="D4" s="70"/>
-      <c r="E4" s="71"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="53"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="72" t="s">
+      <c r="I4" s="54" t="s">
         <v>408</v>
       </c>
-      <c r="J4" s="73"/>
+      <c r="J4" s="55"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="74" t="s">
+      <c r="C5" s="56" t="s">
         <v>408</v>
       </c>
-      <c r="D5" s="74"/>
-      <c r="E5" s="75"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="57"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="76" t="s">
+      <c r="I5" s="58" t="s">
         <v>409</v>
       </c>
-      <c r="J5" s="77"/>
+      <c r="J5" s="59"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -3018,10 +3027,10 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="78" t="s">
+      <c r="I6" s="60" t="s">
         <v>409</v>
       </c>
-      <c r="J6" s="79"/>
+      <c r="J6" s="61"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -3810,11 +3819,6 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -3824,6 +3828,11 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -3854,104 +3863,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="60" t="s">
+      <c r="A1" s="70" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="62"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="72"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="65" t="str">
+      <c r="A2" s="73" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="74"/>
+      <c r="C2" s="75" t="str">
         <f>September!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="65"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="67" t="s">
+      <c r="D2" s="75"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="64"/>
+      <c r="G2" s="74"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="68" t="s">
+      <c r="I2" s="78" t="s">
         <v>311</v>
       </c>
-      <c r="J2" s="69"/>
+      <c r="J2" s="79"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="54" t="str">
+      <c r="B3" s="63"/>
+      <c r="C3" s="64" t="str">
         <f>September!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="54"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="56" t="s">
+      <c r="D3" s="64"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="57"/>
+      <c r="G3" s="67"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="58">
+      <c r="I3" s="68">
         <v>2026</v>
       </c>
-      <c r="J3" s="59"/>
+      <c r="J3" s="69"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="70" t="str">
+      <c r="C4" s="52" t="str">
         <f>September!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="70"/>
-      <c r="E4" s="71"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="53"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="72" t="str">
+      <c r="I4" s="54" t="str">
         <f>September!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="73"/>
+      <c r="J4" s="55"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="74" t="str">
+      <c r="C5" s="56" t="str">
         <f>September!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="74"/>
-      <c r="E5" s="75"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="57"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="76">
+      <c r="I5" s="58">
         <f>September!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="77"/>
+      <c r="J5" s="59"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -3964,11 +3973,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="78" t="str">
+      <c r="I6" s="60" t="str">
         <f>September!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="79"/>
+      <c r="J6" s="61"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -4725,7 +4734,7 @@
       <c r="F43" s="1"/>
       <c r="H43" s="34">
         <f>September!H43</f>
-        <v>3.4374999999999991</v>
+        <v>3.9999999999999991</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -4740,7 +4749,7 @@
       <c r="G44" s="15"/>
       <c r="H44" s="38">
         <f>H42-H41+H43</f>
-        <v>3.4374999999999991</v>
+        <v>3.9999999999999991</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
@@ -4758,11 +4767,6 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -4772,6 +4776,11 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -4802,104 +4811,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="60" t="s">
+      <c r="A1" s="70" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="62"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="72"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="65" t="str">
+      <c r="A2" s="73" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="74"/>
+      <c r="C2" s="75" t="str">
         <f>'Oktober '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="65"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="67" t="s">
+      <c r="D2" s="75"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="64"/>
+      <c r="G2" s="74"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="68" t="s">
+      <c r="I2" s="78" t="s">
         <v>343</v>
       </c>
-      <c r="J2" s="69"/>
+      <c r="J2" s="79"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="54" t="str">
+      <c r="B3" s="63"/>
+      <c r="C3" s="64" t="str">
         <f>'Oktober '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="54"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="56" t="s">
+      <c r="D3" s="64"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="57"/>
+      <c r="G3" s="67"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="58">
+      <c r="I3" s="68">
         <v>2026</v>
       </c>
-      <c r="J3" s="59"/>
+      <c r="J3" s="69"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="70" t="str">
+      <c r="C4" s="52" t="str">
         <f>'Oktober '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="70"/>
-      <c r="E4" s="71"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="53"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="72" t="str">
+      <c r="I4" s="54" t="str">
         <f>'Oktober '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="73"/>
+      <c r="J4" s="55"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="74" t="str">
+      <c r="C5" s="56" t="str">
         <f>'Oktober '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="74"/>
-      <c r="E5" s="75"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="57"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="76">
+      <c r="I5" s="58">
         <f>'Oktober '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="77"/>
+      <c r="J5" s="59"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -4912,11 +4921,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="78" t="str">
+      <c r="I6" s="60" t="str">
         <f>'Oktober '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="79"/>
+      <c r="J6" s="61"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -5652,7 +5661,7 @@
       <c r="F42" s="1"/>
       <c r="H42" s="34">
         <f>'Oktober '!H44</f>
-        <v>3.4374999999999991</v>
+        <v>3.9999999999999991</v>
       </c>
     </row>
     <row r="43" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -5667,7 +5676,7 @@
       <c r="G43" s="15"/>
       <c r="H43" s="38">
         <f>H41-H40+H42</f>
-        <v>3.4374999999999991</v>
+        <v>3.9999999999999991</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
@@ -5685,11 +5694,6 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -5699,6 +5703,11 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -5729,104 +5738,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="60" t="s">
+      <c r="A1" s="70" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="62"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="72"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="65" t="str">
+      <c r="A2" s="73" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="74"/>
+      <c r="C2" s="75" t="str">
         <f>'November '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="65"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="67" t="s">
+      <c r="D2" s="75"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="64"/>
+      <c r="G2" s="74"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="68" t="s">
+      <c r="I2" s="78" t="s">
         <v>374</v>
       </c>
-      <c r="J2" s="69"/>
+      <c r="J2" s="79"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="54" t="str">
+      <c r="B3" s="63"/>
+      <c r="C3" s="64" t="str">
         <f>'November '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="54"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="56" t="s">
+      <c r="D3" s="64"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="57"/>
+      <c r="G3" s="67"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="58">
+      <c r="I3" s="68">
         <v>2026</v>
       </c>
-      <c r="J3" s="59"/>
+      <c r="J3" s="69"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="70" t="str">
+      <c r="C4" s="52" t="str">
         <f>'November '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="70"/>
-      <c r="E4" s="71"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="53"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="72" t="str">
+      <c r="I4" s="54" t="str">
         <f>'November '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="73"/>
+      <c r="J4" s="55"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="74" t="str">
+      <c r="C5" s="56" t="str">
         <f>'November '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="74"/>
-      <c r="E5" s="75"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="57"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="76">
+      <c r="I5" s="58">
         <f>'November '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="77"/>
+      <c r="J5" s="59"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -5839,11 +5848,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="78" t="str">
+      <c r="I6" s="60" t="str">
         <f>'November '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="79"/>
+      <c r="J6" s="61"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -6600,7 +6609,7 @@
       <c r="F43" s="1"/>
       <c r="H43" s="34">
         <f>'November '!H43</f>
-        <v>3.4374999999999991</v>
+        <v>3.9999999999999991</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -6615,7 +6624,7 @@
       <c r="G44" s="15"/>
       <c r="H44" s="38">
         <f>H42-H41+H43</f>
-        <v>3.4374999999999991</v>
+        <v>3.9999999999999991</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
@@ -6633,11 +6642,6 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -6647,6 +6651,11 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -6678,22 +6687,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="85" t="s">
+      <c r="A1" s="80" t="s">
         <v>416</v>
       </c>
-      <c r="B1" s="86"/>
-      <c r="C1" s="86"/>
-      <c r="D1" s="86"/>
-      <c r="E1" s="86"/>
-      <c r="F1" s="86"/>
-      <c r="G1" s="86"/>
-      <c r="H1" s="87"/>
+      <c r="B1" s="81"/>
+      <c r="C1" s="81"/>
+      <c r="D1" s="81"/>
+      <c r="E1" s="81"/>
+      <c r="F1" s="81"/>
+      <c r="G1" s="81"/>
+      <c r="H1" s="82"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="52" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="53"/>
+      <c r="A2" s="62" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="63"/>
       <c r="C2" s="47" t="str">
         <f>'November '!C2:E2</f>
         <v>Hari Krishna</v>
@@ -6702,15 +6711,15 @@
       <c r="E2" s="22" t="s">
         <v>418</v>
       </c>
-      <c r="F2" s="91"/>
-      <c r="G2" s="91"/>
+      <c r="F2" s="86"/>
+      <c r="G2" s="86"/>
       <c r="H2" s="48"/>
     </row>
     <row r="3" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="82" t="s">
+      <c r="A3" s="89" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="57"/>
+      <c r="B3" s="67"/>
       <c r="C3" s="49" t="str">
         <f>'November '!C3:E3</f>
         <v>Mohan Raj</v>
@@ -6719,8 +6728,8 @@
       <c r="E3" s="18" t="s">
         <v>122</v>
       </c>
-      <c r="F3" s="58"/>
-      <c r="G3" s="58"/>
+      <c r="F3" s="68"/>
+      <c r="G3" s="68"/>
       <c r="H3" s="50"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
@@ -6734,17 +6743,17 @@
       </c>
     </row>
     <row r="6" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="89" t="s">
+      <c r="A6" s="84" t="s">
         <v>417</v>
       </c>
-      <c r="B6" s="90"/>
-      <c r="C6" s="88" t="s">
+      <c r="B6" s="85"/>
+      <c r="C6" s="83" t="s">
         <v>419</v>
       </c>
-      <c r="D6" s="88"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="88"/>
-      <c r="G6" s="88"/>
+      <c r="D6" s="83"/>
+      <c r="E6" s="83"/>
+      <c r="F6" s="83"/>
+      <c r="G6" s="83"/>
       <c r="H6" s="51"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
@@ -6756,10 +6765,10 @@
       <c r="D8" s="3"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A9" s="80" t="s">
+      <c r="A9" s="87" t="s">
         <v>410</v>
       </c>
-      <c r="B9" s="81"/>
+      <c r="B9" s="88"/>
       <c r="C9" s="44" t="s">
         <v>411</v>
       </c>
@@ -6775,10 +6784,10 @@
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A10" s="83" t="s">
+      <c r="A10" s="90" t="s">
         <v>407</v>
       </c>
-      <c r="B10" s="84"/>
+      <c r="B10" s="91"/>
       <c r="C10" s="46">
         <f>'Januar '!H41</f>
         <v>0</v>
@@ -6797,10 +6806,10 @@
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A11" s="83" t="s">
+      <c r="A11" s="90" t="s">
         <v>406</v>
       </c>
-      <c r="B11" s="84"/>
+      <c r="B11" s="91"/>
       <c r="C11" s="46">
         <f>'Februar '!H39</f>
         <v>0</v>
@@ -6820,10 +6829,10 @@
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A12" s="83" t="s">
+      <c r="A12" s="90" t="s">
         <v>89</v>
       </c>
-      <c r="B12" s="84"/>
+      <c r="B12" s="91"/>
       <c r="C12" s="46">
         <f>'März '!H41</f>
         <v>0</v>
@@ -6844,10 +6853,10 @@
       <c r="M12" s="28"/>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A13" s="83" t="s">
+      <c r="A13" s="90" t="s">
         <v>121</v>
       </c>
-      <c r="B13" s="84"/>
+      <c r="B13" s="91"/>
       <c r="C13" s="46">
         <f>'April '!H40</f>
         <v>0</v>
@@ -6867,17 +6876,17 @@
       </c>
     </row>
     <row r="14" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="83" t="s">
+      <c r="A14" s="90" t="s">
         <v>185</v>
       </c>
-      <c r="B14" s="84"/>
+      <c r="B14" s="91"/>
       <c r="C14" s="46">
         <f>'Mai '!H41</f>
         <v>0</v>
       </c>
       <c r="D14" s="46">
         <f>'Mai '!H42</f>
-        <v>0.77083333333333326</v>
+        <v>1.333333333333333</v>
       </c>
       <c r="E14" s="46">
         <f>'Mai '!H43</f>
@@ -6886,14 +6895,14 @@
       <c r="F14" s="46"/>
       <c r="G14" s="46">
         <f>'Mai '!H44</f>
-        <v>3.4374999999999991</v>
+        <v>3.9999999999999991</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A15" s="83" t="s">
+      <c r="A15" s="90" t="s">
         <v>184</v>
       </c>
-      <c r="B15" s="84"/>
+      <c r="B15" s="91"/>
       <c r="C15" s="46">
         <f>'Juni '!H40</f>
         <v>0</v>
@@ -6904,19 +6913,19 @@
       </c>
       <c r="E15" s="46">
         <f>'Juni '!H42</f>
-        <v>3.4374999999999991</v>
+        <v>3.9999999999999991</v>
       </c>
       <c r="F15" s="46"/>
       <c r="G15" s="46">
         <f>'Juni '!H43</f>
-        <v>3.4374999999999991</v>
+        <v>3.9999999999999991</v>
       </c>
     </row>
     <row r="16" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="83" t="s">
+      <c r="A16" s="90" t="s">
         <v>247</v>
       </c>
-      <c r="B16" s="84"/>
+      <c r="B16" s="91"/>
       <c r="C16" s="46">
         <f>'Juli '!H41</f>
         <v>0</v>
@@ -6927,19 +6936,19 @@
       </c>
       <c r="E16" s="46">
         <f>'Juli '!H43</f>
-        <v>3.4374999999999991</v>
+        <v>3.9999999999999991</v>
       </c>
       <c r="F16" s="46"/>
       <c r="G16" s="46">
         <f>'Juli '!H44</f>
-        <v>3.4374999999999991</v>
+        <v>3.9999999999999991</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="83" t="s">
+      <c r="A17" s="90" t="s">
         <v>248</v>
       </c>
-      <c r="B17" s="84"/>
+      <c r="B17" s="91"/>
       <c r="C17" s="46">
         <f>'August '!H41</f>
         <v>0</v>
@@ -6950,19 +6959,19 @@
       </c>
       <c r="E17" s="46">
         <f>'August '!H43</f>
-        <v>3.4374999999999991</v>
+        <v>3.9999999999999991</v>
       </c>
       <c r="F17" s="46"/>
       <c r="G17" s="46">
         <f>'August '!H44</f>
-        <v>3.4374999999999991</v>
+        <v>3.9999999999999991</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="83" t="s">
+      <c r="A18" s="90" t="s">
         <v>280</v>
       </c>
-      <c r="B18" s="84"/>
+      <c r="B18" s="91"/>
       <c r="C18" s="46">
         <f>September!H40</f>
         <v>0</v>
@@ -6973,19 +6982,19 @@
       </c>
       <c r="E18" s="46">
         <f>September!H42</f>
-        <v>3.4374999999999991</v>
+        <v>3.9999999999999991</v>
       </c>
       <c r="F18" s="46"/>
       <c r="G18" s="46">
         <f>September!H43</f>
-        <v>3.4374999999999991</v>
+        <v>3.9999999999999991</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="83" t="s">
+      <c r="A19" s="90" t="s">
         <v>311</v>
       </c>
-      <c r="B19" s="84"/>
+      <c r="B19" s="91"/>
       <c r="C19" s="46">
         <f>'Oktober '!H41</f>
         <v>0</v>
@@ -6996,19 +7005,19 @@
       </c>
       <c r="E19" s="46">
         <f>'Oktober '!H43</f>
-        <v>3.4374999999999991</v>
+        <v>3.9999999999999991</v>
       </c>
       <c r="F19" s="46"/>
       <c r="G19" s="46">
         <f>'Oktober '!H44</f>
-        <v>3.4374999999999991</v>
+        <v>3.9999999999999991</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="83" t="s">
+      <c r="A20" s="90" t="s">
         <v>343</v>
       </c>
-      <c r="B20" s="84"/>
+      <c r="B20" s="91"/>
       <c r="C20" s="46">
         <f>'November '!H40</f>
         <v>0</v>
@@ -7019,19 +7028,19 @@
       </c>
       <c r="E20" s="46">
         <f>'November '!H42</f>
-        <v>3.4374999999999991</v>
+        <v>3.9999999999999991</v>
       </c>
       <c r="F20" s="46"/>
       <c r="G20" s="46">
         <f>'November '!H43</f>
-        <v>3.4374999999999991</v>
+        <v>3.9999999999999991</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="83" t="s">
+      <c r="A21" s="90" t="s">
         <v>374</v>
       </c>
-      <c r="B21" s="84"/>
+      <c r="B21" s="91"/>
       <c r="C21" s="46">
         <f>'Dezember '!H41</f>
         <v>0</v>
@@ -7042,12 +7051,12 @@
       </c>
       <c r="E21" s="46">
         <f>'Dezember '!H43</f>
-        <v>3.4374999999999991</v>
+        <v>3.9999999999999991</v>
       </c>
       <c r="F21" s="46"/>
       <c r="G21" s="46">
         <f>'Dezember '!H44</f>
-        <v>3.4374999999999991</v>
+        <v>3.9999999999999991</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
@@ -7084,11 +7093,6 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="20">
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="C6:G6"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="F3:G3"/>
     <mergeCell ref="A9:B9"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A3:B3"/>
@@ -7104,6 +7108,11 @@
     <mergeCell ref="A17:B17"/>
     <mergeCell ref="A18:B18"/>
     <mergeCell ref="A19:B19"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="C6:G6"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="F3:G3"/>
   </mergeCells>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.39370078740157483" bottom="0.39370078740157483" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -7126,104 +7135,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="60" t="s">
+      <c r="A1" s="70" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="62"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="72"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="65" t="str">
+      <c r="A2" s="73" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="74"/>
+      <c r="C2" s="75" t="str">
         <f>'Januar '!C2:E2</f>
         <v>XXX</v>
       </c>
-      <c r="D2" s="65"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="67" t="s">
+      <c r="D2" s="75"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="64"/>
+      <c r="G2" s="74"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="68" t="s">
+      <c r="I2" s="78" t="s">
         <v>406</v>
       </c>
-      <c r="J2" s="69"/>
+      <c r="J2" s="79"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="54" t="str">
+      <c r="B3" s="63"/>
+      <c r="C3" s="64" t="str">
         <f>'Januar '!C3:E3</f>
         <v>XXX</v>
       </c>
-      <c r="D3" s="54"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="56" t="s">
+      <c r="D3" s="64"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="57"/>
+      <c r="G3" s="67"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="58">
+      <c r="I3" s="68">
         <v>2026</v>
       </c>
-      <c r="J3" s="59"/>
+      <c r="J3" s="69"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="70" t="str">
+      <c r="C4" s="52" t="str">
         <f>'Januar '!C4:E4</f>
         <v>XXX</v>
       </c>
-      <c r="D4" s="70"/>
-      <c r="E4" s="71"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="53"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="72" t="str">
+      <c r="I4" s="54" t="str">
         <f>'Januar '!I4:J4</f>
         <v>XXX</v>
       </c>
-      <c r="J4" s="73"/>
+      <c r="J4" s="55"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="74" t="str">
+      <c r="C5" s="56" t="str">
         <f>'Januar '!C5:E5</f>
         <v>XXX</v>
       </c>
-      <c r="D5" s="74"/>
-      <c r="E5" s="75"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="57"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="76" t="str">
+      <c r="I5" s="58" t="str">
         <f>'Januar '!I5:J5</f>
         <v>XX</v>
       </c>
-      <c r="J5" s="77"/>
+      <c r="J5" s="59"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -7236,11 +7245,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="78" t="str">
+      <c r="I6" s="60" t="str">
         <f>'Januar '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="79"/>
+      <c r="J6" s="61"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -7976,11 +7985,6 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -7990,6 +7994,11 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -8020,98 +8029,98 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="60" t="s">
+      <c r="A1" s="70" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="62"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="72"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="65" t="s">
+      <c r="A2" s="73" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="74"/>
+      <c r="C2" s="75" t="s">
         <v>420</v>
       </c>
-      <c r="D2" s="65"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="67" t="s">
+      <c r="D2" s="75"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="64"/>
+      <c r="G2" s="74"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="68" t="s">
+      <c r="I2" s="78" t="s">
         <v>89</v>
       </c>
-      <c r="J2" s="69"/>
+      <c r="J2" s="79"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="54" t="s">
+      <c r="B3" s="63"/>
+      <c r="C3" s="64" t="s">
         <v>421</v>
       </c>
-      <c r="D3" s="54"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="56" t="s">
+      <c r="D3" s="64"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="57"/>
+      <c r="G3" s="67"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="58">
+      <c r="I3" s="68">
         <v>2026</v>
       </c>
-      <c r="J3" s="59"/>
+      <c r="J3" s="69"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="70" t="s">
+      <c r="C4" s="52" t="s">
         <v>422</v>
       </c>
-      <c r="D4" s="70"/>
-      <c r="E4" s="71"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="53"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="72" t="s">
+      <c r="I4" s="54" t="s">
         <v>424</v>
       </c>
-      <c r="J4" s="73"/>
+      <c r="J4" s="55"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="74" t="s">
+      <c r="C5" s="56" t="s">
         <v>423</v>
       </c>
-      <c r="D5" s="74"/>
-      <c r="E5" s="75"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="57"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="76">
+      <c r="I5" s="58">
         <v>8</v>
       </c>
-      <c r="J5" s="77"/>
+      <c r="J5" s="59"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -8124,11 +8133,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="78" t="str">
+      <c r="I6" s="60" t="str">
         <f>'Februar '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="79"/>
+      <c r="J6" s="61"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -8967,11 +8976,6 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -8981,6 +8985,11 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -9011,104 +9020,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="60" t="s">
+      <c r="A1" s="70" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="62"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="72"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="65" t="str">
+      <c r="A2" s="73" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="74"/>
+      <c r="C2" s="75" t="str">
         <f>'März '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="65"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="67" t="s">
+      <c r="D2" s="75"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="64"/>
+      <c r="G2" s="74"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="68" t="s">
+      <c r="I2" s="78" t="s">
         <v>121</v>
       </c>
-      <c r="J2" s="69"/>
+      <c r="J2" s="79"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="54" t="str">
+      <c r="B3" s="63"/>
+      <c r="C3" s="64" t="str">
         <f>'März '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="54"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="56" t="s">
+      <c r="D3" s="64"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="57"/>
+      <c r="G3" s="67"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="58">
+      <c r="I3" s="68">
         <v>2026</v>
       </c>
-      <c r="J3" s="59"/>
+      <c r="J3" s="69"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="70" t="str">
+      <c r="C4" s="52" t="str">
         <f>'März '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="70"/>
-      <c r="E4" s="71"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="53"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="72" t="str">
+      <c r="I4" s="54" t="str">
         <f>'März '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="73"/>
+      <c r="J4" s="55"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="74" t="str">
+      <c r="C5" s="56" t="str">
         <f>'März '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="74"/>
-      <c r="E5" s="75"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="57"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="76">
+      <c r="I5" s="58">
         <f>'März '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="77"/>
+      <c r="J5" s="59"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -9121,11 +9130,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="78" t="str">
+      <c r="I6" s="60" t="str">
         <f>'März '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="79"/>
+      <c r="J6" s="61"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -9935,11 +9944,6 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -9949,6 +9953,11 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -9979,104 +9988,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="60" t="s">
+      <c r="A1" s="70" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="62"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="72"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="65" t="str">
+      <c r="A2" s="73" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="74"/>
+      <c r="C2" s="75" t="str">
         <f>'April '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="65"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="67" t="s">
+      <c r="D2" s="75"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="64"/>
+      <c r="G2" s="74"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="68" t="s">
+      <c r="I2" s="78" t="s">
         <v>185</v>
       </c>
-      <c r="J2" s="69"/>
+      <c r="J2" s="79"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="54" t="str">
+      <c r="B3" s="63"/>
+      <c r="C3" s="64" t="str">
         <f>'April '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="54"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="56" t="s">
+      <c r="D3" s="64"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="57"/>
+      <c r="G3" s="67"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="58">
+      <c r="I3" s="68">
         <v>2026</v>
       </c>
-      <c r="J3" s="59"/>
+      <c r="J3" s="69"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="70" t="str">
+      <c r="C4" s="52" t="str">
         <f>'April '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="70"/>
-      <c r="E4" s="71"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="53"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="72" t="str">
+      <c r="I4" s="54" t="str">
         <f>'April '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="73"/>
+      <c r="J4" s="55"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="74" t="str">
+      <c r="C5" s="56" t="str">
         <f>'April '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="74"/>
-      <c r="E5" s="75"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="57"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="76">
+      <c r="I5" s="58">
         <f>'April '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="77"/>
+      <c r="J5" s="59"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -10089,11 +10098,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="78" t="str">
+      <c r="I6" s="60" t="str">
         <f>'April '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="79"/>
+      <c r="J6" s="61"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -10443,16 +10452,16 @@
         <v>0.625</v>
       </c>
       <c r="E22" s="29">
-        <v>0.6875</v>
+        <v>0.75</v>
       </c>
       <c r="F22" s="29"/>
       <c r="G22" s="6">
         <f>IF(OR(I22="U",I22="F",I22="K"),C22,E22-D22-F22)</f>
-        <v>6.25E-2</v>
+        <v>0.125</v>
       </c>
       <c r="H22" s="26">
         <f t="shared" si="1"/>
-        <v>6.25E-2</v>
+        <v>0.125</v>
       </c>
       <c r="I22" s="30"/>
       <c r="J22" s="31"/>
@@ -10575,16 +10584,20 @@
         <v>14</v>
       </c>
       <c r="C28" s="32"/>
-      <c r="D28" s="29"/>
-      <c r="E28" s="29"/>
+      <c r="D28" s="29">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="E28" s="29">
+        <v>0.75</v>
+      </c>
       <c r="F28" s="29"/>
       <c r="G28" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.16666666666666663</v>
       </c>
       <c r="H28" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.16666666666666663</v>
       </c>
       <c r="I28" s="30"/>
       <c r="J28" s="31"/>
@@ -10733,16 +10746,20 @@
         <v>14</v>
       </c>
       <c r="C35" s="32"/>
-      <c r="D35" s="29"/>
-      <c r="E35" s="29"/>
+      <c r="D35" s="29">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="E35" s="29">
+        <v>0.75</v>
+      </c>
       <c r="F35" s="29"/>
       <c r="G35" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.16666666666666663</v>
       </c>
       <c r="H35" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.16666666666666663</v>
       </c>
       <c r="I35" s="30"/>
       <c r="J35" s="31"/>
@@ -10777,16 +10794,20 @@
         <v>16</v>
       </c>
       <c r="C37" s="32"/>
-      <c r="D37" s="29"/>
-      <c r="E37" s="29"/>
+      <c r="D37" s="29">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="E37" s="29">
+        <v>0.75</v>
+      </c>
       <c r="F37" s="29"/>
       <c r="G37" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.16666666666666663</v>
       </c>
       <c r="H37" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.16666666666666663</v>
       </c>
       <c r="I37" s="30"/>
       <c r="J37" s="31"/>
@@ -10861,7 +10882,7 @@
       <c r="F42" s="1"/>
       <c r="H42" s="34">
         <f>SUM(H9:H39)</f>
-        <v>0.77083333333333326</v>
+        <v>1.333333333333333</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
@@ -10887,7 +10908,7 @@
       <c r="G44" s="15"/>
       <c r="H44" s="38">
         <f>H42-H41+H43</f>
-        <v>3.4374999999999991</v>
+        <v>3.9999999999999991</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
@@ -10905,11 +10926,6 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -10919,6 +10935,11 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -10949,104 +10970,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="60" t="s">
+      <c r="A1" s="70" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="62"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="72"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="65" t="str">
+      <c r="A2" s="73" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="74"/>
+      <c r="C2" s="75" t="str">
         <f>'Mai '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="65"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="67" t="s">
+      <c r="D2" s="75"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="64"/>
+      <c r="G2" s="74"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="68" t="s">
+      <c r="I2" s="78" t="s">
         <v>184</v>
       </c>
-      <c r="J2" s="69"/>
+      <c r="J2" s="79"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="54" t="str">
+      <c r="B3" s="63"/>
+      <c r="C3" s="64" t="str">
         <f>'Mai '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="54"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="56" t="s">
+      <c r="D3" s="64"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="57"/>
+      <c r="G3" s="67"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="58">
+      <c r="I3" s="68">
         <v>2026</v>
       </c>
-      <c r="J3" s="59"/>
+      <c r="J3" s="69"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="70" t="str">
+      <c r="C4" s="52" t="str">
         <f>'Mai '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="70"/>
-      <c r="E4" s="71"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="53"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="72" t="str">
+      <c r="I4" s="54" t="str">
         <f>'Mai '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="73"/>
+      <c r="J4" s="55"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="74" t="str">
+      <c r="C5" s="56" t="str">
         <f>'Mai '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="74"/>
-      <c r="E5" s="75"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="57"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="76">
+      <c r="I5" s="58">
         <f>'Mai '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="77"/>
+      <c r="J5" s="59"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -11059,11 +11080,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="78" t="str">
+      <c r="I6" s="60" t="str">
         <f>'Mai '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="79"/>
+      <c r="J6" s="61"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -11798,7 +11819,7 @@
       <c r="F42" s="1"/>
       <c r="H42" s="34">
         <f>'Mai '!H44</f>
-        <v>3.4374999999999991</v>
+        <v>3.9999999999999991</v>
       </c>
     </row>
     <row r="43" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -11813,7 +11834,7 @@
       <c r="G43" s="15"/>
       <c r="H43" s="38">
         <f>H41-H40+H42</f>
-        <v>3.4374999999999991</v>
+        <v>3.9999999999999991</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
@@ -11831,11 +11852,6 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -11845,6 +11861,11 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -11875,104 +11896,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="60" t="s">
+      <c r="A1" s="70" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="62"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="72"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="65" t="str">
+      <c r="A2" s="73" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="74"/>
+      <c r="C2" s="75" t="str">
         <f>'Juni '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="65"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="67" t="s">
+      <c r="D2" s="75"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="64"/>
+      <c r="G2" s="74"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="68" t="s">
+      <c r="I2" s="78" t="s">
         <v>247</v>
       </c>
-      <c r="J2" s="69"/>
+      <c r="J2" s="79"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="54" t="str">
+      <c r="B3" s="63"/>
+      <c r="C3" s="64" t="str">
         <f>'Juni '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="54"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="56" t="s">
+      <c r="D3" s="64"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="57"/>
+      <c r="G3" s="67"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="58">
+      <c r="I3" s="68">
         <v>2026</v>
       </c>
-      <c r="J3" s="59"/>
+      <c r="J3" s="69"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="70" t="str">
+      <c r="C4" s="52" t="str">
         <f>'Juni '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="70"/>
-      <c r="E4" s="71"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="53"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="72" t="str">
+      <c r="I4" s="54" t="str">
         <f>'Juni '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="73"/>
+      <c r="J4" s="55"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="74" t="str">
+      <c r="C5" s="56" t="str">
         <f>'Juni '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="74"/>
-      <c r="E5" s="75"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="57"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="76">
+      <c r="I5" s="58">
         <f>'Juni '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="77"/>
+      <c r="J5" s="59"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -11985,11 +12006,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="78" t="str">
+      <c r="I6" s="60" t="str">
         <f>'Juni '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="79"/>
+      <c r="J6" s="61"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -12746,7 +12767,7 @@
       <c r="F43" s="1"/>
       <c r="H43" s="34">
         <f>'Juni '!H43</f>
-        <v>3.4374999999999991</v>
+        <v>3.9999999999999991</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -12761,7 +12782,7 @@
       <c r="G44" s="15"/>
       <c r="H44" s="38">
         <f>H42-H41+H43</f>
-        <v>3.4374999999999991</v>
+        <v>3.9999999999999991</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
@@ -12779,11 +12800,6 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -12793,6 +12809,11 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -12823,104 +12844,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="60" t="s">
+      <c r="A1" s="70" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="62"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="72"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="65" t="str">
+      <c r="A2" s="73" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="74"/>
+      <c r="C2" s="75" t="str">
         <f>'Juli '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="65"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="67" t="s">
+      <c r="D2" s="75"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="64"/>
+      <c r="G2" s="74"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="68" t="s">
+      <c r="I2" s="78" t="s">
         <v>248</v>
       </c>
-      <c r="J2" s="69"/>
+      <c r="J2" s="79"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="54" t="str">
+      <c r="B3" s="63"/>
+      <c r="C3" s="64" t="str">
         <f>'Juli '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="54"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="56" t="s">
+      <c r="D3" s="64"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="57"/>
+      <c r="G3" s="67"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="58">
+      <c r="I3" s="68">
         <v>2026</v>
       </c>
-      <c r="J3" s="59"/>
+      <c r="J3" s="69"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="70" t="str">
+      <c r="C4" s="52" t="str">
         <f>'Juli '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="70"/>
-      <c r="E4" s="71"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="53"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="72" t="str">
+      <c r="I4" s="54" t="str">
         <f>'Juli '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="73"/>
+      <c r="J4" s="55"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="74" t="str">
+      <c r="C5" s="56" t="str">
         <f>'Juli '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="74"/>
-      <c r="E5" s="75"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="57"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="76">
+      <c r="I5" s="58">
         <f>'Juli '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="77"/>
+      <c r="J5" s="59"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -12933,11 +12954,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="78" t="str">
+      <c r="I6" s="60" t="str">
         <f>'Juli '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="79"/>
+      <c r="J6" s="61"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -13694,7 +13715,7 @@
       <c r="F43" s="1"/>
       <c r="H43" s="34">
         <f>'Juli '!H44</f>
-        <v>3.4374999999999991</v>
+        <v>3.9999999999999991</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -13709,7 +13730,7 @@
       <c r="G44" s="15"/>
       <c r="H44" s="38">
         <f>H42-H41+H43</f>
-        <v>3.4374999999999991</v>
+        <v>3.9999999999999991</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
@@ -13727,11 +13748,6 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -13741,6 +13757,11 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -13771,104 +13792,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="60" t="s">
+      <c r="A1" s="70" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="62"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="72"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="65" t="str">
+      <c r="A2" s="73" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="74"/>
+      <c r="C2" s="75" t="str">
         <f>'August '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="65"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="67" t="s">
+      <c r="D2" s="75"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="64"/>
+      <c r="G2" s="74"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="68" t="s">
+      <c r="I2" s="78" t="s">
         <v>280</v>
       </c>
-      <c r="J2" s="69"/>
+      <c r="J2" s="79"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="54" t="str">
+      <c r="B3" s="63"/>
+      <c r="C3" s="64" t="str">
         <f>'August '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="54"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="56" t="s">
+      <c r="D3" s="64"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="57"/>
+      <c r="G3" s="67"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="58">
+      <c r="I3" s="68">
         <v>2026</v>
       </c>
-      <c r="J3" s="59"/>
+      <c r="J3" s="69"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="70" t="str">
+      <c r="C4" s="52" t="str">
         <f>'August '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="70"/>
-      <c r="E4" s="71"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="53"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="72" t="str">
+      <c r="I4" s="54" t="str">
         <f>'August '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="73"/>
+      <c r="J4" s="55"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="74" t="str">
+      <c r="C5" s="56" t="str">
         <f>'August '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="74"/>
-      <c r="E5" s="75"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="57"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="76">
+      <c r="I5" s="58">
         <f>'August '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="77"/>
+      <c r="J5" s="59"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -13881,11 +13902,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="78" t="str">
+      <c r="I6" s="60" t="str">
         <f>'August '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="79"/>
+      <c r="J6" s="61"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -14620,7 +14641,7 @@
       <c r="F42" s="1"/>
       <c r="H42" s="34">
         <f>'August '!H44</f>
-        <v>3.4374999999999991</v>
+        <v>3.9999999999999991</v>
       </c>
     </row>
     <row r="43" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -14635,7 +14656,7 @@
       <c r="G43" s="15"/>
       <c r="H43" s="38">
         <f>H41-H40+H42</f>
-        <v>3.4374999999999991</v>
+        <v>3.9999999999999991</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
@@ -14653,11 +14674,6 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -14667,6 +14683,11 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">

</xml_diff>

<commit_message>
presentation, data of mouse rat and human extras, pdf structures
</commit_message>
<xml_diff>
--- a/HK Zeiterfassung 2026.xlsx
+++ b/HK Zeiterfassung 2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harik\Downloads\Computational Chemistry\Variant-Effect-Predictor-for-nAChRs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66285D0A-43C7-4BAB-9EE3-97FB309787BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60E9E903-105A-4B81-A6F3-37FC99A1E7B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9720" yWindow="5190" windowWidth="18165" windowHeight="11130" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6810" yWindow="5550" windowWidth="16695" windowHeight="10680" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Januar " sheetId="26" r:id="rId1"/>
@@ -2489,46 +2489,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="3" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="17" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="17" fontId="0" fillId="3" borderId="17" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -2591,6 +2551,61 @@
       <alignment horizontal="right"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="17" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="17" fontId="0" fillId="3" borderId="17" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2613,21 +2628,6 @@
     <xf numFmtId="166" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2923,98 +2923,98 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="72"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="62"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="73" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="74"/>
-      <c r="C2" s="75" t="s">
+      <c r="A2" s="63" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="64"/>
+      <c r="C2" s="65" t="s">
         <v>408</v>
       </c>
-      <c r="D2" s="75"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="77" t="s">
+      <c r="D2" s="65"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="74"/>
+      <c r="G2" s="64"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="78" t="s">
+      <c r="I2" s="68" t="s">
         <v>407</v>
       </c>
-      <c r="J2" s="79"/>
+      <c r="J2" s="69"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="64" t="s">
+      <c r="B3" s="53"/>
+      <c r="C3" s="54" t="s">
         <v>408</v>
       </c>
-      <c r="D3" s="64"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="66" t="s">
+      <c r="D3" s="54"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="67"/>
+      <c r="G3" s="57"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="68">
+      <c r="I3" s="58">
         <v>2026</v>
       </c>
-      <c r="J3" s="69"/>
+      <c r="J3" s="59"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="52" t="s">
+      <c r="C4" s="70" t="s">
         <v>408</v>
       </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="53"/>
+      <c r="D4" s="70"/>
+      <c r="E4" s="71"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="54" t="s">
+      <c r="I4" s="72" t="s">
         <v>408</v>
       </c>
-      <c r="J4" s="55"/>
+      <c r="J4" s="73"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="56" t="s">
+      <c r="C5" s="74" t="s">
         <v>408</v>
       </c>
-      <c r="D5" s="56"/>
-      <c r="E5" s="57"/>
+      <c r="D5" s="74"/>
+      <c r="E5" s="75"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="58" t="s">
+      <c r="I5" s="76" t="s">
         <v>409</v>
       </c>
-      <c r="J5" s="59"/>
+      <c r="J5" s="77"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -3027,10 +3027,10 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="60" t="s">
+      <c r="I6" s="78" t="s">
         <v>409</v>
       </c>
-      <c r="J6" s="61"/>
+      <c r="J6" s="79"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -3819,6 +3819,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -3828,11 +3833,6 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -3863,104 +3863,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="72"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="62"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="73" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="74"/>
-      <c r="C2" s="75" t="str">
+      <c r="A2" s="63" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="64"/>
+      <c r="C2" s="65" t="str">
         <f>September!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="75"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="77" t="s">
+      <c r="D2" s="65"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="74"/>
+      <c r="G2" s="64"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="78" t="s">
+      <c r="I2" s="68" t="s">
         <v>311</v>
       </c>
-      <c r="J2" s="79"/>
+      <c r="J2" s="69"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="64" t="str">
+      <c r="B3" s="53"/>
+      <c r="C3" s="54" t="str">
         <f>September!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="64"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="66" t="s">
+      <c r="D3" s="54"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="67"/>
+      <c r="G3" s="57"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="68">
+      <c r="I3" s="58">
         <v>2026</v>
       </c>
-      <c r="J3" s="69"/>
+      <c r="J3" s="59"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="52" t="str">
+      <c r="C4" s="70" t="str">
         <f>September!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="53"/>
+      <c r="D4" s="70"/>
+      <c r="E4" s="71"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="54" t="str">
+      <c r="I4" s="72" t="str">
         <f>September!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="55"/>
+      <c r="J4" s="73"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="56" t="str">
+      <c r="C5" s="74" t="str">
         <f>September!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="56"/>
-      <c r="E5" s="57"/>
+      <c r="D5" s="74"/>
+      <c r="E5" s="75"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="58">
+      <c r="I5" s="76">
         <f>September!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="59"/>
+      <c r="J5" s="77"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -3973,11 +3973,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="60" t="str">
+      <c r="I6" s="78" t="str">
         <f>September!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="61"/>
+      <c r="J6" s="79"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -4734,7 +4734,7 @@
       <c r="F43" s="1"/>
       <c r="H43" s="34">
         <f>September!H43</f>
-        <v>3.9999999999999991</v>
+        <v>5.3333333333333321</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -4749,7 +4749,7 @@
       <c r="G44" s="15"/>
       <c r="H44" s="38">
         <f>H42-H41+H43</f>
-        <v>3.9999999999999991</v>
+        <v>5.3333333333333321</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
@@ -4767,6 +4767,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -4776,11 +4781,6 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -4811,104 +4811,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="72"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="62"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="73" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="74"/>
-      <c r="C2" s="75" t="str">
+      <c r="A2" s="63" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="64"/>
+      <c r="C2" s="65" t="str">
         <f>'Oktober '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="75"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="77" t="s">
+      <c r="D2" s="65"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="74"/>
+      <c r="G2" s="64"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="78" t="s">
+      <c r="I2" s="68" t="s">
         <v>343</v>
       </c>
-      <c r="J2" s="79"/>
+      <c r="J2" s="69"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="64" t="str">
+      <c r="B3" s="53"/>
+      <c r="C3" s="54" t="str">
         <f>'Oktober '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="64"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="66" t="s">
+      <c r="D3" s="54"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="67"/>
+      <c r="G3" s="57"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="68">
+      <c r="I3" s="58">
         <v>2026</v>
       </c>
-      <c r="J3" s="69"/>
+      <c r="J3" s="59"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="52" t="str">
+      <c r="C4" s="70" t="str">
         <f>'Oktober '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="53"/>
+      <c r="D4" s="70"/>
+      <c r="E4" s="71"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="54" t="str">
+      <c r="I4" s="72" t="str">
         <f>'Oktober '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="55"/>
+      <c r="J4" s="73"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="56" t="str">
+      <c r="C5" s="74" t="str">
         <f>'Oktober '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="56"/>
-      <c r="E5" s="57"/>
+      <c r="D5" s="74"/>
+      <c r="E5" s="75"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="58">
+      <c r="I5" s="76">
         <f>'Oktober '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="59"/>
+      <c r="J5" s="77"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -4921,11 +4921,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="60" t="str">
+      <c r="I6" s="78" t="str">
         <f>'Oktober '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="61"/>
+      <c r="J6" s="79"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -5661,7 +5661,7 @@
       <c r="F42" s="1"/>
       <c r="H42" s="34">
         <f>'Oktober '!H44</f>
-        <v>3.9999999999999991</v>
+        <v>5.3333333333333321</v>
       </c>
     </row>
     <row r="43" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -5676,7 +5676,7 @@
       <c r="G43" s="15"/>
       <c r="H43" s="38">
         <f>H41-H40+H42</f>
-        <v>3.9999999999999991</v>
+        <v>5.3333333333333321</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
@@ -5694,6 +5694,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -5703,11 +5708,6 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -5738,104 +5738,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="72"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="62"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="73" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="74"/>
-      <c r="C2" s="75" t="str">
+      <c r="A2" s="63" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="64"/>
+      <c r="C2" s="65" t="str">
         <f>'November '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="75"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="77" t="s">
+      <c r="D2" s="65"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="74"/>
+      <c r="G2" s="64"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="78" t="s">
+      <c r="I2" s="68" t="s">
         <v>374</v>
       </c>
-      <c r="J2" s="79"/>
+      <c r="J2" s="69"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="64" t="str">
+      <c r="B3" s="53"/>
+      <c r="C3" s="54" t="str">
         <f>'November '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="64"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="66" t="s">
+      <c r="D3" s="54"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="67"/>
+      <c r="G3" s="57"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="68">
+      <c r="I3" s="58">
         <v>2026</v>
       </c>
-      <c r="J3" s="69"/>
+      <c r="J3" s="59"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="52" t="str">
+      <c r="C4" s="70" t="str">
         <f>'November '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="53"/>
+      <c r="D4" s="70"/>
+      <c r="E4" s="71"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="54" t="str">
+      <c r="I4" s="72" t="str">
         <f>'November '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="55"/>
+      <c r="J4" s="73"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="56" t="str">
+      <c r="C5" s="74" t="str">
         <f>'November '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="56"/>
-      <c r="E5" s="57"/>
+      <c r="D5" s="74"/>
+      <c r="E5" s="75"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="58">
+      <c r="I5" s="76">
         <f>'November '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="59"/>
+      <c r="J5" s="77"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -5848,11 +5848,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="60" t="str">
+      <c r="I6" s="78" t="str">
         <f>'November '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="61"/>
+      <c r="J6" s="79"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -6609,7 +6609,7 @@
       <c r="F43" s="1"/>
       <c r="H43" s="34">
         <f>'November '!H43</f>
-        <v>3.9999999999999991</v>
+        <v>5.3333333333333321</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -6624,7 +6624,7 @@
       <c r="G44" s="15"/>
       <c r="H44" s="38">
         <f>H42-H41+H43</f>
-        <v>3.9999999999999991</v>
+        <v>5.3333333333333321</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
@@ -6642,6 +6642,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -6651,11 +6656,6 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -6687,22 +6687,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="80" t="s">
+      <c r="A1" s="85" t="s">
         <v>416</v>
       </c>
-      <c r="B1" s="81"/>
-      <c r="C1" s="81"/>
-      <c r="D1" s="81"/>
-      <c r="E1" s="81"/>
-      <c r="F1" s="81"/>
-      <c r="G1" s="81"/>
-      <c r="H1" s="82"/>
+      <c r="B1" s="86"/>
+      <c r="C1" s="86"/>
+      <c r="D1" s="86"/>
+      <c r="E1" s="86"/>
+      <c r="F1" s="86"/>
+      <c r="G1" s="86"/>
+      <c r="H1" s="87"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="62" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="63"/>
+      <c r="A2" s="52" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="53"/>
       <c r="C2" s="47" t="str">
         <f>'November '!C2:E2</f>
         <v>Hari Krishna</v>
@@ -6711,15 +6711,15 @@
       <c r="E2" s="22" t="s">
         <v>418</v>
       </c>
-      <c r="F2" s="86"/>
-      <c r="G2" s="86"/>
+      <c r="F2" s="91"/>
+      <c r="G2" s="91"/>
       <c r="H2" s="48"/>
     </row>
     <row r="3" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="89" t="s">
+      <c r="A3" s="82" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="67"/>
+      <c r="B3" s="57"/>
       <c r="C3" s="49" t="str">
         <f>'November '!C3:E3</f>
         <v>Mohan Raj</v>
@@ -6728,8 +6728,8 @@
       <c r="E3" s="18" t="s">
         <v>122</v>
       </c>
-      <c r="F3" s="68"/>
-      <c r="G3" s="68"/>
+      <c r="F3" s="58"/>
+      <c r="G3" s="58"/>
       <c r="H3" s="50"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
@@ -6743,17 +6743,17 @@
       </c>
     </row>
     <row r="6" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="84" t="s">
+      <c r="A6" s="89" t="s">
         <v>417</v>
       </c>
-      <c r="B6" s="85"/>
-      <c r="C6" s="83" t="s">
+      <c r="B6" s="90"/>
+      <c r="C6" s="88" t="s">
         <v>419</v>
       </c>
-      <c r="D6" s="83"/>
-      <c r="E6" s="83"/>
-      <c r="F6" s="83"/>
-      <c r="G6" s="83"/>
+      <c r="D6" s="88"/>
+      <c r="E6" s="88"/>
+      <c r="F6" s="88"/>
+      <c r="G6" s="88"/>
       <c r="H6" s="51"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
@@ -6765,10 +6765,10 @@
       <c r="D8" s="3"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A9" s="87" t="s">
+      <c r="A9" s="80" t="s">
         <v>410</v>
       </c>
-      <c r="B9" s="88"/>
+      <c r="B9" s="81"/>
       <c r="C9" s="44" t="s">
         <v>411</v>
       </c>
@@ -6784,10 +6784,10 @@
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A10" s="90" t="s">
+      <c r="A10" s="83" t="s">
         <v>407</v>
       </c>
-      <c r="B10" s="91"/>
+      <c r="B10" s="84"/>
       <c r="C10" s="46">
         <f>'Januar '!H41</f>
         <v>0</v>
@@ -6806,10 +6806,10 @@
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A11" s="90" t="s">
+      <c r="A11" s="83" t="s">
         <v>406</v>
       </c>
-      <c r="B11" s="91"/>
+      <c r="B11" s="84"/>
       <c r="C11" s="46">
         <f>'Februar '!H39</f>
         <v>0</v>
@@ -6829,10 +6829,10 @@
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A12" s="90" t="s">
+      <c r="A12" s="83" t="s">
         <v>89</v>
       </c>
-      <c r="B12" s="91"/>
+      <c r="B12" s="84"/>
       <c r="C12" s="46">
         <f>'März '!H41</f>
         <v>0</v>
@@ -6853,10 +6853,10 @@
       <c r="M12" s="28"/>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A13" s="90" t="s">
+      <c r="A13" s="83" t="s">
         <v>121</v>
       </c>
-      <c r="B13" s="91"/>
+      <c r="B13" s="84"/>
       <c r="C13" s="46">
         <f>'April '!H40</f>
         <v>0</v>
@@ -6876,10 +6876,10 @@
       </c>
     </row>
     <row r="14" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="90" t="s">
+      <c r="A14" s="83" t="s">
         <v>185</v>
       </c>
-      <c r="B14" s="91"/>
+      <c r="B14" s="84"/>
       <c r="C14" s="46">
         <f>'Mai '!H41</f>
         <v>0</v>
@@ -6899,17 +6899,17 @@
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A15" s="90" t="s">
+      <c r="A15" s="83" t="s">
         <v>184</v>
       </c>
-      <c r="B15" s="91"/>
+      <c r="B15" s="84"/>
       <c r="C15" s="46">
         <f>'Juni '!H40</f>
         <v>0</v>
       </c>
       <c r="D15" s="46">
         <f>'Juni '!H41</f>
-        <v>0</v>
+        <v>1.333333333333333</v>
       </c>
       <c r="E15" s="46">
         <f>'Juni '!H42</f>
@@ -6918,14 +6918,14 @@
       <c r="F15" s="46"/>
       <c r="G15" s="46">
         <f>'Juni '!H43</f>
-        <v>3.9999999999999991</v>
+        <v>5.3333333333333321</v>
       </c>
     </row>
     <row r="16" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="90" t="s">
+      <c r="A16" s="83" t="s">
         <v>247</v>
       </c>
-      <c r="B16" s="91"/>
+      <c r="B16" s="84"/>
       <c r="C16" s="46">
         <f>'Juli '!H41</f>
         <v>0</v>
@@ -6936,19 +6936,19 @@
       </c>
       <c r="E16" s="46">
         <f>'Juli '!H43</f>
-        <v>3.9999999999999991</v>
+        <v>5.3333333333333321</v>
       </c>
       <c r="F16" s="46"/>
       <c r="G16" s="46">
         <f>'Juli '!H44</f>
-        <v>3.9999999999999991</v>
+        <v>5.3333333333333321</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="90" t="s">
+      <c r="A17" s="83" t="s">
         <v>248</v>
       </c>
-      <c r="B17" s="91"/>
+      <c r="B17" s="84"/>
       <c r="C17" s="46">
         <f>'August '!H41</f>
         <v>0</v>
@@ -6959,19 +6959,19 @@
       </c>
       <c r="E17" s="46">
         <f>'August '!H43</f>
-        <v>3.9999999999999991</v>
+        <v>5.3333333333333321</v>
       </c>
       <c r="F17" s="46"/>
       <c r="G17" s="46">
         <f>'August '!H44</f>
-        <v>3.9999999999999991</v>
+        <v>5.3333333333333321</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="90" t="s">
+      <c r="A18" s="83" t="s">
         <v>280</v>
       </c>
-      <c r="B18" s="91"/>
+      <c r="B18" s="84"/>
       <c r="C18" s="46">
         <f>September!H40</f>
         <v>0</v>
@@ -6982,19 +6982,19 @@
       </c>
       <c r="E18" s="46">
         <f>September!H42</f>
-        <v>3.9999999999999991</v>
+        <v>5.3333333333333321</v>
       </c>
       <c r="F18" s="46"/>
       <c r="G18" s="46">
         <f>September!H43</f>
-        <v>3.9999999999999991</v>
+        <v>5.3333333333333321</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="90" t="s">
+      <c r="A19" s="83" t="s">
         <v>311</v>
       </c>
-      <c r="B19" s="91"/>
+      <c r="B19" s="84"/>
       <c r="C19" s="46">
         <f>'Oktober '!H41</f>
         <v>0</v>
@@ -7005,19 +7005,19 @@
       </c>
       <c r="E19" s="46">
         <f>'Oktober '!H43</f>
-        <v>3.9999999999999991</v>
+        <v>5.3333333333333321</v>
       </c>
       <c r="F19" s="46"/>
       <c r="G19" s="46">
         <f>'Oktober '!H44</f>
-        <v>3.9999999999999991</v>
+        <v>5.3333333333333321</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="90" t="s">
+      <c r="A20" s="83" t="s">
         <v>343</v>
       </c>
-      <c r="B20" s="91"/>
+      <c r="B20" s="84"/>
       <c r="C20" s="46">
         <f>'November '!H40</f>
         <v>0</v>
@@ -7028,19 +7028,19 @@
       </c>
       <c r="E20" s="46">
         <f>'November '!H42</f>
-        <v>3.9999999999999991</v>
+        <v>5.3333333333333321</v>
       </c>
       <c r="F20" s="46"/>
       <c r="G20" s="46">
         <f>'November '!H43</f>
-        <v>3.9999999999999991</v>
+        <v>5.3333333333333321</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="90" t="s">
+      <c r="A21" s="83" t="s">
         <v>374</v>
       </c>
-      <c r="B21" s="91"/>
+      <c r="B21" s="84"/>
       <c r="C21" s="46">
         <f>'Dezember '!H41</f>
         <v>0</v>
@@ -7051,12 +7051,12 @@
       </c>
       <c r="E21" s="46">
         <f>'Dezember '!H43</f>
-        <v>3.9999999999999991</v>
+        <v>5.3333333333333321</v>
       </c>
       <c r="F21" s="46"/>
       <c r="G21" s="46">
         <f>'Dezember '!H44</f>
-        <v>3.9999999999999991</v>
+        <v>5.3333333333333321</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
@@ -7093,6 +7093,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="20">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="C6:G6"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="F3:G3"/>
     <mergeCell ref="A9:B9"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A3:B3"/>
@@ -7108,11 +7113,6 @@
     <mergeCell ref="A17:B17"/>
     <mergeCell ref="A18:B18"/>
     <mergeCell ref="A19:B19"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="C6:G6"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="F3:G3"/>
   </mergeCells>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.39370078740157483" bottom="0.39370078740157483" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -7135,104 +7135,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="72"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="62"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="73" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="74"/>
-      <c r="C2" s="75" t="str">
+      <c r="A2" s="63" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="64"/>
+      <c r="C2" s="65" t="str">
         <f>'Januar '!C2:E2</f>
         <v>XXX</v>
       </c>
-      <c r="D2" s="75"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="77" t="s">
+      <c r="D2" s="65"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="74"/>
+      <c r="G2" s="64"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="78" t="s">
+      <c r="I2" s="68" t="s">
         <v>406</v>
       </c>
-      <c r="J2" s="79"/>
+      <c r="J2" s="69"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="64" t="str">
+      <c r="B3" s="53"/>
+      <c r="C3" s="54" t="str">
         <f>'Januar '!C3:E3</f>
         <v>XXX</v>
       </c>
-      <c r="D3" s="64"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="66" t="s">
+      <c r="D3" s="54"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="67"/>
+      <c r="G3" s="57"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="68">
+      <c r="I3" s="58">
         <v>2026</v>
       </c>
-      <c r="J3" s="69"/>
+      <c r="J3" s="59"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="52" t="str">
+      <c r="C4" s="70" t="str">
         <f>'Januar '!C4:E4</f>
         <v>XXX</v>
       </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="53"/>
+      <c r="D4" s="70"/>
+      <c r="E4" s="71"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="54" t="str">
+      <c r="I4" s="72" t="str">
         <f>'Januar '!I4:J4</f>
         <v>XXX</v>
       </c>
-      <c r="J4" s="55"/>
+      <c r="J4" s="73"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="56" t="str">
+      <c r="C5" s="74" t="str">
         <f>'Januar '!C5:E5</f>
         <v>XXX</v>
       </c>
-      <c r="D5" s="56"/>
-      <c r="E5" s="57"/>
+      <c r="D5" s="74"/>
+      <c r="E5" s="75"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="58" t="str">
+      <c r="I5" s="76" t="str">
         <f>'Januar '!I5:J5</f>
         <v>XX</v>
       </c>
-      <c r="J5" s="59"/>
+      <c r="J5" s="77"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -7245,11 +7245,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="60" t="str">
+      <c r="I6" s="78" t="str">
         <f>'Januar '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="61"/>
+      <c r="J6" s="79"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -7985,6 +7985,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -7994,11 +7999,6 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -8029,98 +8029,98 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="72"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="62"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="73" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="74"/>
-      <c r="C2" s="75" t="s">
+      <c r="A2" s="63" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="64"/>
+      <c r="C2" s="65" t="s">
         <v>420</v>
       </c>
-      <c r="D2" s="75"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="77" t="s">
+      <c r="D2" s="65"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="74"/>
+      <c r="G2" s="64"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="78" t="s">
+      <c r="I2" s="68" t="s">
         <v>89</v>
       </c>
-      <c r="J2" s="79"/>
+      <c r="J2" s="69"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="64" t="s">
+      <c r="B3" s="53"/>
+      <c r="C3" s="54" t="s">
         <v>421</v>
       </c>
-      <c r="D3" s="64"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="66" t="s">
+      <c r="D3" s="54"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="67"/>
+      <c r="G3" s="57"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="68">
+      <c r="I3" s="58">
         <v>2026</v>
       </c>
-      <c r="J3" s="69"/>
+      <c r="J3" s="59"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="52" t="s">
+      <c r="C4" s="70" t="s">
         <v>422</v>
       </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="53"/>
+      <c r="D4" s="70"/>
+      <c r="E4" s="71"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="54" t="s">
+      <c r="I4" s="72" t="s">
         <v>424</v>
       </c>
-      <c r="J4" s="55"/>
+      <c r="J4" s="73"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="56" t="s">
+      <c r="C5" s="74" t="s">
         <v>423</v>
       </c>
-      <c r="D5" s="56"/>
-      <c r="E5" s="57"/>
+      <c r="D5" s="74"/>
+      <c r="E5" s="75"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="58">
+      <c r="I5" s="76">
         <v>8</v>
       </c>
-      <c r="J5" s="59"/>
+      <c r="J5" s="77"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -8133,11 +8133,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="60" t="str">
+      <c r="I6" s="78" t="str">
         <f>'Februar '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="61"/>
+      <c r="J6" s="79"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -8976,6 +8976,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -8985,11 +8990,6 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -9020,104 +9020,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="72"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="62"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="73" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="74"/>
-      <c r="C2" s="75" t="str">
+      <c r="A2" s="63" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="64"/>
+      <c r="C2" s="65" t="str">
         <f>'März '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="75"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="77" t="s">
+      <c r="D2" s="65"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="74"/>
+      <c r="G2" s="64"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="78" t="s">
+      <c r="I2" s="68" t="s">
         <v>121</v>
       </c>
-      <c r="J2" s="79"/>
+      <c r="J2" s="69"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="64" t="str">
+      <c r="B3" s="53"/>
+      <c r="C3" s="54" t="str">
         <f>'März '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="64"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="66" t="s">
+      <c r="D3" s="54"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="67"/>
+      <c r="G3" s="57"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="68">
+      <c r="I3" s="58">
         <v>2026</v>
       </c>
-      <c r="J3" s="69"/>
+      <c r="J3" s="59"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="52" t="str">
+      <c r="C4" s="70" t="str">
         <f>'März '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="53"/>
+      <c r="D4" s="70"/>
+      <c r="E4" s="71"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="54" t="str">
+      <c r="I4" s="72" t="str">
         <f>'März '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="55"/>
+      <c r="J4" s="73"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="56" t="str">
+      <c r="C5" s="74" t="str">
         <f>'März '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="56"/>
-      <c r="E5" s="57"/>
+      <c r="D5" s="74"/>
+      <c r="E5" s="75"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="58">
+      <c r="I5" s="76">
         <f>'März '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="59"/>
+      <c r="J5" s="77"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -9130,11 +9130,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="60" t="str">
+      <c r="I6" s="78" t="str">
         <f>'März '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="61"/>
+      <c r="J6" s="79"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -9944,6 +9944,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -9953,11 +9958,6 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -9988,104 +9988,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="72"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="62"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="73" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="74"/>
-      <c r="C2" s="75" t="str">
+      <c r="A2" s="63" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="64"/>
+      <c r="C2" s="65" t="str">
         <f>'April '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="75"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="77" t="s">
+      <c r="D2" s="65"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="74"/>
+      <c r="G2" s="64"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="78" t="s">
+      <c r="I2" s="68" t="s">
         <v>185</v>
       </c>
-      <c r="J2" s="79"/>
+      <c r="J2" s="69"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="64" t="str">
+      <c r="B3" s="53"/>
+      <c r="C3" s="54" t="str">
         <f>'April '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="64"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="66" t="s">
+      <c r="D3" s="54"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="67"/>
+      <c r="G3" s="57"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="68">
+      <c r="I3" s="58">
         <v>2026</v>
       </c>
-      <c r="J3" s="69"/>
+      <c r="J3" s="59"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="52" t="str">
+      <c r="C4" s="70" t="str">
         <f>'April '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="53"/>
+      <c r="D4" s="70"/>
+      <c r="E4" s="71"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="54" t="str">
+      <c r="I4" s="72" t="str">
         <f>'April '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="55"/>
+      <c r="J4" s="73"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="56" t="str">
+      <c r="C5" s="74" t="str">
         <f>'April '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="56"/>
-      <c r="E5" s="57"/>
+      <c r="D5" s="74"/>
+      <c r="E5" s="75"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="58">
+      <c r="I5" s="76">
         <f>'April '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="59"/>
+      <c r="J5" s="77"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -10098,11 +10098,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="60" t="str">
+      <c r="I6" s="78" t="str">
         <f>'April '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="61"/>
+      <c r="J6" s="79"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -10926,6 +10926,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -10935,11 +10940,6 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -10970,104 +10970,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="72"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="62"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="73" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="74"/>
-      <c r="C2" s="75" t="str">
+      <c r="A2" s="63" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="64"/>
+      <c r="C2" s="65" t="str">
         <f>'Mai '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="75"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="77" t="s">
+      <c r="D2" s="65"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="74"/>
+      <c r="G2" s="64"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="78" t="s">
+      <c r="I2" s="68" t="s">
         <v>184</v>
       </c>
-      <c r="J2" s="79"/>
+      <c r="J2" s="69"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="64" t="str">
+      <c r="B3" s="53"/>
+      <c r="C3" s="54" t="str">
         <f>'Mai '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="64"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="66" t="s">
+      <c r="D3" s="54"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="67"/>
+      <c r="G3" s="57"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="68">
+      <c r="I3" s="58">
         <v>2026</v>
       </c>
-      <c r="J3" s="69"/>
+      <c r="J3" s="59"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="52" t="str">
+      <c r="C4" s="70" t="str">
         <f>'Mai '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="53"/>
+      <c r="D4" s="70"/>
+      <c r="E4" s="71"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="54" t="str">
+      <c r="I4" s="72" t="str">
         <f>'Mai '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="55"/>
+      <c r="J4" s="73"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="56" t="str">
+      <c r="C5" s="74" t="str">
         <f>'Mai '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="56"/>
-      <c r="E5" s="57"/>
+      <c r="D5" s="74"/>
+      <c r="E5" s="75"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="58">
+      <c r="I5" s="76">
         <f>'Mai '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="59"/>
+      <c r="J5" s="77"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -11080,11 +11080,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="60" t="str">
+      <c r="I6" s="78" t="str">
         <f>'Mai '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="61"/>
+      <c r="J6" s="79"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -11173,16 +11173,20 @@
         <v>14</v>
       </c>
       <c r="C11" s="32"/>
-      <c r="D11" s="29"/>
-      <c r="E11" s="29"/>
+      <c r="D11" s="29">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="E11" s="29">
+        <v>0.79166666666666663</v>
+      </c>
       <c r="F11" s="29"/>
       <c r="G11" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.20833333333333326</v>
       </c>
       <c r="H11" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.20833333333333326</v>
       </c>
       <c r="I11" s="30"/>
       <c r="J11" s="31"/>
@@ -11218,16 +11222,20 @@
         <v>16</v>
       </c>
       <c r="C13" s="32"/>
-      <c r="D13" s="29"/>
-      <c r="E13" s="29"/>
+      <c r="D13" s="29">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="E13" s="29">
+        <v>0.70833333333333337</v>
+      </c>
       <c r="F13" s="29"/>
       <c r="G13" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="H13" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="I13" s="30"/>
       <c r="J13" s="31"/>
@@ -11328,16 +11336,20 @@
         <v>14</v>
       </c>
       <c r="C18" s="32"/>
-      <c r="D18" s="29"/>
-      <c r="E18" s="29"/>
+      <c r="D18" s="29">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="E18" s="29">
+        <v>0.79166666666666663</v>
+      </c>
       <c r="F18" s="29"/>
       <c r="G18" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.20833333333333326</v>
       </c>
       <c r="H18" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.20833333333333326</v>
       </c>
       <c r="I18" s="30"/>
       <c r="J18" s="31"/>
@@ -11372,16 +11384,20 @@
         <v>16</v>
       </c>
       <c r="C20" s="32"/>
-      <c r="D20" s="29"/>
-      <c r="E20" s="29"/>
+      <c r="D20" s="29">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="E20" s="29">
+        <v>0.70833333333333337</v>
+      </c>
       <c r="F20" s="29"/>
       <c r="G20" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="H20" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="I20" s="30"/>
       <c r="J20" s="31"/>
@@ -11482,16 +11498,20 @@
         <v>14</v>
       </c>
       <c r="C25" s="32"/>
-      <c r="D25" s="29"/>
-      <c r="E25" s="29"/>
+      <c r="D25" s="29">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="E25" s="29">
+        <v>0.79166666666666663</v>
+      </c>
       <c r="F25" s="29"/>
       <c r="G25" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.20833333333333326</v>
       </c>
       <c r="H25" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.20833333333333326</v>
       </c>
       <c r="I25" s="30"/>
       <c r="J25" s="31"/>
@@ -11526,16 +11546,20 @@
         <v>16</v>
       </c>
       <c r="C27" s="32"/>
-      <c r="D27" s="29"/>
-      <c r="E27" s="29"/>
+      <c r="D27" s="29">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="E27" s="29">
+        <v>0.70833333333333337</v>
+      </c>
       <c r="F27" s="29"/>
       <c r="G27" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="H27" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="I27" s="30"/>
       <c r="J27" s="31"/>
@@ -11636,16 +11660,20 @@
         <v>14</v>
       </c>
       <c r="C32" s="32"/>
-      <c r="D32" s="29"/>
-      <c r="E32" s="29"/>
+      <c r="D32" s="29">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="E32" s="29">
+        <v>0.79166666666666663</v>
+      </c>
       <c r="F32" s="29"/>
       <c r="G32" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.20833333333333326</v>
       </c>
       <c r="H32" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.20833333333333326</v>
       </c>
       <c r="I32" s="30"/>
       <c r="J32" s="31"/>
@@ -11680,16 +11708,20 @@
         <v>16</v>
       </c>
       <c r="C34" s="32"/>
-      <c r="D34" s="29"/>
-      <c r="E34" s="29"/>
+      <c r="D34" s="29">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="E34" s="29">
+        <v>0.70833333333333337</v>
+      </c>
       <c r="F34" s="29"/>
       <c r="G34" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="H34" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="I34" s="30"/>
       <c r="J34" s="31"/>
@@ -11808,7 +11840,7 @@
       <c r="F41" s="1"/>
       <c r="H41" s="34">
         <f>SUM(H9:H38)</f>
-        <v>0</v>
+        <v>1.333333333333333</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
@@ -11834,7 +11866,7 @@
       <c r="G43" s="15"/>
       <c r="H43" s="38">
         <f>H41-H40+H42</f>
-        <v>3.9999999999999991</v>
+        <v>5.3333333333333321</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
@@ -11852,6 +11884,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -11861,11 +11898,6 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -11896,104 +11928,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="72"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="62"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="73" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="74"/>
-      <c r="C2" s="75" t="str">
+      <c r="A2" s="63" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="64"/>
+      <c r="C2" s="65" t="str">
         <f>'Juni '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="75"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="77" t="s">
+      <c r="D2" s="65"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="74"/>
+      <c r="G2" s="64"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="78" t="s">
+      <c r="I2" s="68" t="s">
         <v>247</v>
       </c>
-      <c r="J2" s="79"/>
+      <c r="J2" s="69"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="64" t="str">
+      <c r="B3" s="53"/>
+      <c r="C3" s="54" t="str">
         <f>'Juni '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="64"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="66" t="s">
+      <c r="D3" s="54"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="67"/>
+      <c r="G3" s="57"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="68">
+      <c r="I3" s="58">
         <v>2026</v>
       </c>
-      <c r="J3" s="69"/>
+      <c r="J3" s="59"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="52" t="str">
+      <c r="C4" s="70" t="str">
         <f>'Juni '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="53"/>
+      <c r="D4" s="70"/>
+      <c r="E4" s="71"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="54" t="str">
+      <c r="I4" s="72" t="str">
         <f>'Juni '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="55"/>
+      <c r="J4" s="73"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="56" t="str">
+      <c r="C5" s="74" t="str">
         <f>'Juni '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="56"/>
-      <c r="E5" s="57"/>
+      <c r="D5" s="74"/>
+      <c r="E5" s="75"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="58">
+      <c r="I5" s="76">
         <f>'Juni '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="59"/>
+      <c r="J5" s="77"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -12006,11 +12038,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="60" t="str">
+      <c r="I6" s="78" t="str">
         <f>'Juni '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="61"/>
+      <c r="J6" s="79"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -12767,7 +12799,7 @@
       <c r="F43" s="1"/>
       <c r="H43" s="34">
         <f>'Juni '!H43</f>
-        <v>3.9999999999999991</v>
+        <v>5.3333333333333321</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -12782,7 +12814,7 @@
       <c r="G44" s="15"/>
       <c r="H44" s="38">
         <f>H42-H41+H43</f>
-        <v>3.9999999999999991</v>
+        <v>5.3333333333333321</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
@@ -12800,6 +12832,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -12809,11 +12846,6 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -12844,104 +12876,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="72"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="62"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="73" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="74"/>
-      <c r="C2" s="75" t="str">
+      <c r="A2" s="63" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="64"/>
+      <c r="C2" s="65" t="str">
         <f>'Juli '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="75"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="77" t="s">
+      <c r="D2" s="65"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="74"/>
+      <c r="G2" s="64"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="78" t="s">
+      <c r="I2" s="68" t="s">
         <v>248</v>
       </c>
-      <c r="J2" s="79"/>
+      <c r="J2" s="69"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="64" t="str">
+      <c r="B3" s="53"/>
+      <c r="C3" s="54" t="str">
         <f>'Juli '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="64"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="66" t="s">
+      <c r="D3" s="54"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="67"/>
+      <c r="G3" s="57"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="68">
+      <c r="I3" s="58">
         <v>2026</v>
       </c>
-      <c r="J3" s="69"/>
+      <c r="J3" s="59"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="52" t="str">
+      <c r="C4" s="70" t="str">
         <f>'Juli '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="53"/>
+      <c r="D4" s="70"/>
+      <c r="E4" s="71"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="54" t="str">
+      <c r="I4" s="72" t="str">
         <f>'Juli '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="55"/>
+      <c r="J4" s="73"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="56" t="str">
+      <c r="C5" s="74" t="str">
         <f>'Juli '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="56"/>
-      <c r="E5" s="57"/>
+      <c r="D5" s="74"/>
+      <c r="E5" s="75"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="58">
+      <c r="I5" s="76">
         <f>'Juli '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="59"/>
+      <c r="J5" s="77"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -12954,11 +12986,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="60" t="str">
+      <c r="I6" s="78" t="str">
         <f>'Juli '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="61"/>
+      <c r="J6" s="79"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -13715,7 +13747,7 @@
       <c r="F43" s="1"/>
       <c r="H43" s="34">
         <f>'Juli '!H44</f>
-        <v>3.9999999999999991</v>
+        <v>5.3333333333333321</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -13730,7 +13762,7 @@
       <c r="G44" s="15"/>
       <c r="H44" s="38">
         <f>H42-H41+H43</f>
-        <v>3.9999999999999991</v>
+        <v>5.3333333333333321</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
@@ -13748,6 +13780,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -13757,11 +13794,6 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -13792,104 +13824,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="72"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="62"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="73" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="74"/>
-      <c r="C2" s="75" t="str">
+      <c r="A2" s="63" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="64"/>
+      <c r="C2" s="65" t="str">
         <f>'August '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="75"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="77" t="s">
+      <c r="D2" s="65"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="74"/>
+      <c r="G2" s="64"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="78" t="s">
+      <c r="I2" s="68" t="s">
         <v>280</v>
       </c>
-      <c r="J2" s="79"/>
+      <c r="J2" s="69"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="64" t="str">
+      <c r="B3" s="53"/>
+      <c r="C3" s="54" t="str">
         <f>'August '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="64"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="66" t="s">
+      <c r="D3" s="54"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="67"/>
+      <c r="G3" s="57"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="68">
+      <c r="I3" s="58">
         <v>2026</v>
       </c>
-      <c r="J3" s="69"/>
+      <c r="J3" s="59"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="52" t="str">
+      <c r="C4" s="70" t="str">
         <f>'August '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="53"/>
+      <c r="D4" s="70"/>
+      <c r="E4" s="71"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="54" t="str">
+      <c r="I4" s="72" t="str">
         <f>'August '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="55"/>
+      <c r="J4" s="73"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="56" t="str">
+      <c r="C5" s="74" t="str">
         <f>'August '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="56"/>
-      <c r="E5" s="57"/>
+      <c r="D5" s="74"/>
+      <c r="E5" s="75"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="58">
+      <c r="I5" s="76">
         <f>'August '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="59"/>
+      <c r="J5" s="77"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -13902,11 +13934,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="60" t="str">
+      <c r="I6" s="78" t="str">
         <f>'August '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="61"/>
+      <c r="J6" s="79"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -14641,7 +14673,7 @@
       <c r="F42" s="1"/>
       <c r="H42" s="34">
         <f>'August '!H44</f>
-        <v>3.9999999999999991</v>
+        <v>5.3333333333333321</v>
       </c>
     </row>
     <row r="43" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -14656,7 +14688,7 @@
       <c r="G43" s="15"/>
       <c r="H43" s="38">
         <f>H41-H40+H42</f>
-        <v>3.9999999999999991</v>
+        <v>5.3333333333333321</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
@@ -14674,6 +14706,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -14683,11 +14720,6 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">

</xml_diff>

<commit_message>
initial run with the F1 score of 0.5 and ablation results
</commit_message>
<xml_diff>
--- a/HK Zeiterfassung 2026.xlsx
+++ b/HK Zeiterfassung 2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr date1904="1" codeName="DieseArbeitsmappe"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harik\Downloads\Computational Chemistry\Variant-Effect-Predictor-for-nAChRs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60E9E903-105A-4B81-A6F3-37FC99A1E7B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29E21B5B-DE80-41EE-9E69-EE7AFC07FCB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6810" yWindow="5550" windowWidth="16695" windowHeight="10680" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11205" yWindow="4410" windowWidth="16845" windowHeight="11070" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Januar " sheetId="26" r:id="rId1"/>
@@ -2489,6 +2489,46 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="17" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="17" fontId="0" fillId="3" borderId="17" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -2551,61 +2591,6 @@
       <alignment horizontal="right"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="3" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="17" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="17" fontId="0" fillId="3" borderId="17" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2628,6 +2613,21 @@
     <xf numFmtId="166" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2923,98 +2923,98 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="60" t="s">
+      <c r="A1" s="70" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="62"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="72"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="65" t="s">
+      <c r="A2" s="73" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="74"/>
+      <c r="C2" s="75" t="s">
         <v>408</v>
       </c>
-      <c r="D2" s="65"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="67" t="s">
+      <c r="D2" s="75"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="64"/>
+      <c r="G2" s="74"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="68" t="s">
+      <c r="I2" s="78" t="s">
         <v>407</v>
       </c>
-      <c r="J2" s="69"/>
+      <c r="J2" s="79"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="54" t="s">
+      <c r="B3" s="63"/>
+      <c r="C3" s="64" t="s">
         <v>408</v>
       </c>
-      <c r="D3" s="54"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="56" t="s">
+      <c r="D3" s="64"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="57"/>
+      <c r="G3" s="67"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="58">
+      <c r="I3" s="68">
         <v>2026</v>
       </c>
-      <c r="J3" s="59"/>
+      <c r="J3" s="69"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="70" t="s">
+      <c r="C4" s="52" t="s">
         <v>408</v>
       </c>
-      <c r="D4" s="70"/>
-      <c r="E4" s="71"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="53"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="72" t="s">
+      <c r="I4" s="54" t="s">
         <v>408</v>
       </c>
-      <c r="J4" s="73"/>
+      <c r="J4" s="55"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="74" t="s">
+      <c r="C5" s="56" t="s">
         <v>408</v>
       </c>
-      <c r="D5" s="74"/>
-      <c r="E5" s="75"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="57"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="76" t="s">
+      <c r="I5" s="58" t="s">
         <v>409</v>
       </c>
-      <c r="J5" s="77"/>
+      <c r="J5" s="59"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -3027,10 +3027,10 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="78" t="s">
+      <c r="I6" s="60" t="s">
         <v>409</v>
       </c>
-      <c r="J6" s="79"/>
+      <c r="J6" s="61"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -3819,11 +3819,6 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -3833,6 +3828,11 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -3863,104 +3863,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="60" t="s">
+      <c r="A1" s="70" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="62"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="72"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="65" t="str">
+      <c r="A2" s="73" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="74"/>
+      <c r="C2" s="75" t="str">
         <f>September!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="65"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="67" t="s">
+      <c r="D2" s="75"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="64"/>
+      <c r="G2" s="74"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="68" t="s">
+      <c r="I2" s="78" t="s">
         <v>311</v>
       </c>
-      <c r="J2" s="69"/>
+      <c r="J2" s="79"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="54" t="str">
+      <c r="B3" s="63"/>
+      <c r="C3" s="64" t="str">
         <f>September!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="54"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="56" t="s">
+      <c r="D3" s="64"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="57"/>
+      <c r="G3" s="67"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="58">
+      <c r="I3" s="68">
         <v>2026</v>
       </c>
-      <c r="J3" s="59"/>
+      <c r="J3" s="69"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="70" t="str">
+      <c r="C4" s="52" t="str">
         <f>September!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="70"/>
-      <c r="E4" s="71"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="53"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="72" t="str">
+      <c r="I4" s="54" t="str">
         <f>September!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="73"/>
+      <c r="J4" s="55"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="74" t="str">
+      <c r="C5" s="56" t="str">
         <f>September!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="74"/>
-      <c r="E5" s="75"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="57"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="76">
+      <c r="I5" s="58">
         <f>September!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="77"/>
+      <c r="J5" s="59"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -3973,11 +3973,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="78" t="str">
+      <c r="I6" s="60" t="str">
         <f>September!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="79"/>
+      <c r="J6" s="61"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -4734,7 +4734,7 @@
       <c r="F43" s="1"/>
       <c r="H43" s="34">
         <f>September!H43</f>
-        <v>5.3333333333333321</v>
+        <v>6.6666666666666652</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -4749,7 +4749,7 @@
       <c r="G44" s="15"/>
       <c r="H44" s="38">
         <f>H42-H41+H43</f>
-        <v>5.3333333333333321</v>
+        <v>6.6666666666666652</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
@@ -4767,11 +4767,6 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -4781,6 +4776,11 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -4811,104 +4811,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="60" t="s">
+      <c r="A1" s="70" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="62"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="72"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="65" t="str">
+      <c r="A2" s="73" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="74"/>
+      <c r="C2" s="75" t="str">
         <f>'Oktober '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="65"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="67" t="s">
+      <c r="D2" s="75"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="64"/>
+      <c r="G2" s="74"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="68" t="s">
+      <c r="I2" s="78" t="s">
         <v>343</v>
       </c>
-      <c r="J2" s="69"/>
+      <c r="J2" s="79"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="54" t="str">
+      <c r="B3" s="63"/>
+      <c r="C3" s="64" t="str">
         <f>'Oktober '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="54"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="56" t="s">
+      <c r="D3" s="64"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="57"/>
+      <c r="G3" s="67"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="58">
+      <c r="I3" s="68">
         <v>2026</v>
       </c>
-      <c r="J3" s="59"/>
+      <c r="J3" s="69"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="70" t="str">
+      <c r="C4" s="52" t="str">
         <f>'Oktober '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="70"/>
-      <c r="E4" s="71"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="53"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="72" t="str">
+      <c r="I4" s="54" t="str">
         <f>'Oktober '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="73"/>
+      <c r="J4" s="55"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="74" t="str">
+      <c r="C5" s="56" t="str">
         <f>'Oktober '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="74"/>
-      <c r="E5" s="75"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="57"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="76">
+      <c r="I5" s="58">
         <f>'Oktober '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="77"/>
+      <c r="J5" s="59"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -4921,11 +4921,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="78" t="str">
+      <c r="I6" s="60" t="str">
         <f>'Oktober '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="79"/>
+      <c r="J6" s="61"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -5661,7 +5661,7 @@
       <c r="F42" s="1"/>
       <c r="H42" s="34">
         <f>'Oktober '!H44</f>
-        <v>5.3333333333333321</v>
+        <v>6.6666666666666652</v>
       </c>
     </row>
     <row r="43" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -5676,7 +5676,7 @@
       <c r="G43" s="15"/>
       <c r="H43" s="38">
         <f>H41-H40+H42</f>
-        <v>5.3333333333333321</v>
+        <v>6.6666666666666652</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
@@ -5694,11 +5694,6 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -5708,6 +5703,11 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -5738,104 +5738,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="60" t="s">
+      <c r="A1" s="70" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="62"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="72"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="65" t="str">
+      <c r="A2" s="73" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="74"/>
+      <c r="C2" s="75" t="str">
         <f>'November '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="65"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="67" t="s">
+      <c r="D2" s="75"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="64"/>
+      <c r="G2" s="74"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="68" t="s">
+      <c r="I2" s="78" t="s">
         <v>374</v>
       </c>
-      <c r="J2" s="69"/>
+      <c r="J2" s="79"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="54" t="str">
+      <c r="B3" s="63"/>
+      <c r="C3" s="64" t="str">
         <f>'November '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="54"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="56" t="s">
+      <c r="D3" s="64"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="57"/>
+      <c r="G3" s="67"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="58">
+      <c r="I3" s="68">
         <v>2026</v>
       </c>
-      <c r="J3" s="59"/>
+      <c r="J3" s="69"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="70" t="str">
+      <c r="C4" s="52" t="str">
         <f>'November '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="70"/>
-      <c r="E4" s="71"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="53"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="72" t="str">
+      <c r="I4" s="54" t="str">
         <f>'November '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="73"/>
+      <c r="J4" s="55"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="74" t="str">
+      <c r="C5" s="56" t="str">
         <f>'November '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="74"/>
-      <c r="E5" s="75"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="57"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="76">
+      <c r="I5" s="58">
         <f>'November '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="77"/>
+      <c r="J5" s="59"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -5848,11 +5848,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="78" t="str">
+      <c r="I6" s="60" t="str">
         <f>'November '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="79"/>
+      <c r="J6" s="61"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -6609,7 +6609,7 @@
       <c r="F43" s="1"/>
       <c r="H43" s="34">
         <f>'November '!H43</f>
-        <v>5.3333333333333321</v>
+        <v>6.6666666666666652</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -6624,7 +6624,7 @@
       <c r="G44" s="15"/>
       <c r="H44" s="38">
         <f>H42-H41+H43</f>
-        <v>5.3333333333333321</v>
+        <v>6.6666666666666652</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
@@ -6642,11 +6642,6 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -6656,6 +6651,11 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -6687,22 +6687,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="85" t="s">
+      <c r="A1" s="80" t="s">
         <v>416</v>
       </c>
-      <c r="B1" s="86"/>
-      <c r="C1" s="86"/>
-      <c r="D1" s="86"/>
-      <c r="E1" s="86"/>
-      <c r="F1" s="86"/>
-      <c r="G1" s="86"/>
-      <c r="H1" s="87"/>
+      <c r="B1" s="81"/>
+      <c r="C1" s="81"/>
+      <c r="D1" s="81"/>
+      <c r="E1" s="81"/>
+      <c r="F1" s="81"/>
+      <c r="G1" s="81"/>
+      <c r="H1" s="82"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="52" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="53"/>
+      <c r="A2" s="62" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="63"/>
       <c r="C2" s="47" t="str">
         <f>'November '!C2:E2</f>
         <v>Hari Krishna</v>
@@ -6711,15 +6711,15 @@
       <c r="E2" s="22" t="s">
         <v>418</v>
       </c>
-      <c r="F2" s="91"/>
-      <c r="G2" s="91"/>
+      <c r="F2" s="86"/>
+      <c r="G2" s="86"/>
       <c r="H2" s="48"/>
     </row>
     <row r="3" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="82" t="s">
+      <c r="A3" s="89" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="57"/>
+      <c r="B3" s="67"/>
       <c r="C3" s="49" t="str">
         <f>'November '!C3:E3</f>
         <v>Mohan Raj</v>
@@ -6728,8 +6728,8 @@
       <c r="E3" s="18" t="s">
         <v>122</v>
       </c>
-      <c r="F3" s="58"/>
-      <c r="G3" s="58"/>
+      <c r="F3" s="68"/>
+      <c r="G3" s="68"/>
       <c r="H3" s="50"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
@@ -6743,17 +6743,17 @@
       </c>
     </row>
     <row r="6" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="89" t="s">
+      <c r="A6" s="84" t="s">
         <v>417</v>
       </c>
-      <c r="B6" s="90"/>
-      <c r="C6" s="88" t="s">
+      <c r="B6" s="85"/>
+      <c r="C6" s="83" t="s">
         <v>419</v>
       </c>
-      <c r="D6" s="88"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="88"/>
-      <c r="G6" s="88"/>
+      <c r="D6" s="83"/>
+      <c r="E6" s="83"/>
+      <c r="F6" s="83"/>
+      <c r="G6" s="83"/>
       <c r="H6" s="51"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
@@ -6765,10 +6765,10 @@
       <c r="D8" s="3"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A9" s="80" t="s">
+      <c r="A9" s="87" t="s">
         <v>410</v>
       </c>
-      <c r="B9" s="81"/>
+      <c r="B9" s="88"/>
       <c r="C9" s="44" t="s">
         <v>411</v>
       </c>
@@ -6784,10 +6784,10 @@
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A10" s="83" t="s">
+      <c r="A10" s="90" t="s">
         <v>407</v>
       </c>
-      <c r="B10" s="84"/>
+      <c r="B10" s="91"/>
       <c r="C10" s="46">
         <f>'Januar '!H41</f>
         <v>0</v>
@@ -6806,10 +6806,10 @@
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A11" s="83" t="s">
+      <c r="A11" s="90" t="s">
         <v>406</v>
       </c>
-      <c r="B11" s="84"/>
+      <c r="B11" s="91"/>
       <c r="C11" s="46">
         <f>'Februar '!H39</f>
         <v>0</v>
@@ -6829,10 +6829,10 @@
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A12" s="83" t="s">
+      <c r="A12" s="90" t="s">
         <v>89</v>
       </c>
-      <c r="B12" s="84"/>
+      <c r="B12" s="91"/>
       <c r="C12" s="46">
         <f>'März '!H41</f>
         <v>0</v>
@@ -6853,10 +6853,10 @@
       <c r="M12" s="28"/>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A13" s="83" t="s">
+      <c r="A13" s="90" t="s">
         <v>121</v>
       </c>
-      <c r="B13" s="84"/>
+      <c r="B13" s="91"/>
       <c r="C13" s="46">
         <f>'April '!H40</f>
         <v>0</v>
@@ -6876,10 +6876,10 @@
       </c>
     </row>
     <row r="14" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="83" t="s">
+      <c r="A14" s="90" t="s">
         <v>185</v>
       </c>
-      <c r="B14" s="84"/>
+      <c r="B14" s="91"/>
       <c r="C14" s="46">
         <f>'Mai '!H41</f>
         <v>0</v>
@@ -6899,10 +6899,10 @@
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A15" s="83" t="s">
+      <c r="A15" s="90" t="s">
         <v>184</v>
       </c>
-      <c r="B15" s="84"/>
+      <c r="B15" s="91"/>
       <c r="C15" s="46">
         <f>'Juni '!H40</f>
         <v>0</v>
@@ -6922,17 +6922,17 @@
       </c>
     </row>
     <row r="16" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="83" t="s">
+      <c r="A16" s="90" t="s">
         <v>247</v>
       </c>
-      <c r="B16" s="84"/>
+      <c r="B16" s="91"/>
       <c r="C16" s="46">
         <f>'Juli '!H41</f>
         <v>0</v>
       </c>
       <c r="D16" s="46">
         <f>'Juli '!H42</f>
-        <v>0</v>
+        <v>1.333333333333333</v>
       </c>
       <c r="E16" s="46">
         <f>'Juli '!H43</f>
@@ -6941,14 +6941,14 @@
       <c r="F16" s="46"/>
       <c r="G16" s="46">
         <f>'Juli '!H44</f>
-        <v>5.3333333333333321</v>
+        <v>6.6666666666666652</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="83" t="s">
+      <c r="A17" s="90" t="s">
         <v>248</v>
       </c>
-      <c r="B17" s="84"/>
+      <c r="B17" s="91"/>
       <c r="C17" s="46">
         <f>'August '!H41</f>
         <v>0</v>
@@ -6959,19 +6959,19 @@
       </c>
       <c r="E17" s="46">
         <f>'August '!H43</f>
-        <v>5.3333333333333321</v>
+        <v>6.6666666666666652</v>
       </c>
       <c r="F17" s="46"/>
       <c r="G17" s="46">
         <f>'August '!H44</f>
-        <v>5.3333333333333321</v>
+        <v>6.6666666666666652</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="83" t="s">
+      <c r="A18" s="90" t="s">
         <v>280</v>
       </c>
-      <c r="B18" s="84"/>
+      <c r="B18" s="91"/>
       <c r="C18" s="46">
         <f>September!H40</f>
         <v>0</v>
@@ -6982,19 +6982,19 @@
       </c>
       <c r="E18" s="46">
         <f>September!H42</f>
-        <v>5.3333333333333321</v>
+        <v>6.6666666666666652</v>
       </c>
       <c r="F18" s="46"/>
       <c r="G18" s="46">
         <f>September!H43</f>
-        <v>5.3333333333333321</v>
+        <v>6.6666666666666652</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="83" t="s">
+      <c r="A19" s="90" t="s">
         <v>311</v>
       </c>
-      <c r="B19" s="84"/>
+      <c r="B19" s="91"/>
       <c r="C19" s="46">
         <f>'Oktober '!H41</f>
         <v>0</v>
@@ -7005,19 +7005,19 @@
       </c>
       <c r="E19" s="46">
         <f>'Oktober '!H43</f>
-        <v>5.3333333333333321</v>
+        <v>6.6666666666666652</v>
       </c>
       <c r="F19" s="46"/>
       <c r="G19" s="46">
         <f>'Oktober '!H44</f>
-        <v>5.3333333333333321</v>
+        <v>6.6666666666666652</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="83" t="s">
+      <c r="A20" s="90" t="s">
         <v>343</v>
       </c>
-      <c r="B20" s="84"/>
+      <c r="B20" s="91"/>
       <c r="C20" s="46">
         <f>'November '!H40</f>
         <v>0</v>
@@ -7028,19 +7028,19 @@
       </c>
       <c r="E20" s="46">
         <f>'November '!H42</f>
-        <v>5.3333333333333321</v>
+        <v>6.6666666666666652</v>
       </c>
       <c r="F20" s="46"/>
       <c r="G20" s="46">
         <f>'November '!H43</f>
-        <v>5.3333333333333321</v>
+        <v>6.6666666666666652</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="83" t="s">
+      <c r="A21" s="90" t="s">
         <v>374</v>
       </c>
-      <c r="B21" s="84"/>
+      <c r="B21" s="91"/>
       <c r="C21" s="46">
         <f>'Dezember '!H41</f>
         <v>0</v>
@@ -7051,12 +7051,12 @@
       </c>
       <c r="E21" s="46">
         <f>'Dezember '!H43</f>
-        <v>5.3333333333333321</v>
+        <v>6.6666666666666652</v>
       </c>
       <c r="F21" s="46"/>
       <c r="G21" s="46">
         <f>'Dezember '!H44</f>
-        <v>5.3333333333333321</v>
+        <v>6.6666666666666652</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
@@ -7093,11 +7093,6 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="20">
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="C6:G6"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="F3:G3"/>
     <mergeCell ref="A9:B9"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A3:B3"/>
@@ -7113,6 +7108,11 @@
     <mergeCell ref="A17:B17"/>
     <mergeCell ref="A18:B18"/>
     <mergeCell ref="A19:B19"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="C6:G6"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="F3:G3"/>
   </mergeCells>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.39370078740157483" bottom="0.39370078740157483" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -7135,104 +7135,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="60" t="s">
+      <c r="A1" s="70" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="62"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="72"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="65" t="str">
+      <c r="A2" s="73" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="74"/>
+      <c r="C2" s="75" t="str">
         <f>'Januar '!C2:E2</f>
         <v>XXX</v>
       </c>
-      <c r="D2" s="65"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="67" t="s">
+      <c r="D2" s="75"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="64"/>
+      <c r="G2" s="74"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="68" t="s">
+      <c r="I2" s="78" t="s">
         <v>406</v>
       </c>
-      <c r="J2" s="69"/>
+      <c r="J2" s="79"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="54" t="str">
+      <c r="B3" s="63"/>
+      <c r="C3" s="64" t="str">
         <f>'Januar '!C3:E3</f>
         <v>XXX</v>
       </c>
-      <c r="D3" s="54"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="56" t="s">
+      <c r="D3" s="64"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="57"/>
+      <c r="G3" s="67"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="58">
+      <c r="I3" s="68">
         <v>2026</v>
       </c>
-      <c r="J3" s="59"/>
+      <c r="J3" s="69"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="70" t="str">
+      <c r="C4" s="52" t="str">
         <f>'Januar '!C4:E4</f>
         <v>XXX</v>
       </c>
-      <c r="D4" s="70"/>
-      <c r="E4" s="71"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="53"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="72" t="str">
+      <c r="I4" s="54" t="str">
         <f>'Januar '!I4:J4</f>
         <v>XXX</v>
       </c>
-      <c r="J4" s="73"/>
+      <c r="J4" s="55"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="74" t="str">
+      <c r="C5" s="56" t="str">
         <f>'Januar '!C5:E5</f>
         <v>XXX</v>
       </c>
-      <c r="D5" s="74"/>
-      <c r="E5" s="75"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="57"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="76" t="str">
+      <c r="I5" s="58" t="str">
         <f>'Januar '!I5:J5</f>
         <v>XX</v>
       </c>
-      <c r="J5" s="77"/>
+      <c r="J5" s="59"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -7245,11 +7245,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="78" t="str">
+      <c r="I6" s="60" t="str">
         <f>'Januar '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="79"/>
+      <c r="J6" s="61"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -7985,11 +7985,6 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -7999,6 +7994,11 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -8029,98 +8029,98 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="60" t="s">
+      <c r="A1" s="70" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="62"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="72"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="65" t="s">
+      <c r="A2" s="73" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="74"/>
+      <c r="C2" s="75" t="s">
         <v>420</v>
       </c>
-      <c r="D2" s="65"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="67" t="s">
+      <c r="D2" s="75"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="64"/>
+      <c r="G2" s="74"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="68" t="s">
+      <c r="I2" s="78" t="s">
         <v>89</v>
       </c>
-      <c r="J2" s="69"/>
+      <c r="J2" s="79"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="54" t="s">
+      <c r="B3" s="63"/>
+      <c r="C3" s="64" t="s">
         <v>421</v>
       </c>
-      <c r="D3" s="54"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="56" t="s">
+      <c r="D3" s="64"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="57"/>
+      <c r="G3" s="67"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="58">
+      <c r="I3" s="68">
         <v>2026</v>
       </c>
-      <c r="J3" s="59"/>
+      <c r="J3" s="69"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="70" t="s">
+      <c r="C4" s="52" t="s">
         <v>422</v>
       </c>
-      <c r="D4" s="70"/>
-      <c r="E4" s="71"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="53"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="72" t="s">
+      <c r="I4" s="54" t="s">
         <v>424</v>
       </c>
-      <c r="J4" s="73"/>
+      <c r="J4" s="55"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="74" t="s">
+      <c r="C5" s="56" t="s">
         <v>423</v>
       </c>
-      <c r="D5" s="74"/>
-      <c r="E5" s="75"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="57"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="76">
+      <c r="I5" s="58">
         <v>8</v>
       </c>
-      <c r="J5" s="77"/>
+      <c r="J5" s="59"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -8133,11 +8133,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="78" t="str">
+      <c r="I6" s="60" t="str">
         <f>'Februar '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="79"/>
+      <c r="J6" s="61"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -8976,11 +8976,6 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -8990,6 +8985,11 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -9020,104 +9020,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="60" t="s">
+      <c r="A1" s="70" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="62"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="72"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="65" t="str">
+      <c r="A2" s="73" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="74"/>
+      <c r="C2" s="75" t="str">
         <f>'März '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="65"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="67" t="s">
+      <c r="D2" s="75"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="64"/>
+      <c r="G2" s="74"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="68" t="s">
+      <c r="I2" s="78" t="s">
         <v>121</v>
       </c>
-      <c r="J2" s="69"/>
+      <c r="J2" s="79"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="54" t="str">
+      <c r="B3" s="63"/>
+      <c r="C3" s="64" t="str">
         <f>'März '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="54"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="56" t="s">
+      <c r="D3" s="64"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="57"/>
+      <c r="G3" s="67"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="58">
+      <c r="I3" s="68">
         <v>2026</v>
       </c>
-      <c r="J3" s="59"/>
+      <c r="J3" s="69"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="70" t="str">
+      <c r="C4" s="52" t="str">
         <f>'März '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="70"/>
-      <c r="E4" s="71"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="53"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="72" t="str">
+      <c r="I4" s="54" t="str">
         <f>'März '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="73"/>
+      <c r="J4" s="55"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="74" t="str">
+      <c r="C5" s="56" t="str">
         <f>'März '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="74"/>
-      <c r="E5" s="75"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="57"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="76">
+      <c r="I5" s="58">
         <f>'März '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="77"/>
+      <c r="J5" s="59"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -9130,11 +9130,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="78" t="str">
+      <c r="I6" s="60" t="str">
         <f>'März '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="79"/>
+      <c r="J6" s="61"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -9944,11 +9944,6 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -9958,6 +9953,11 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -9988,104 +9988,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="60" t="s">
+      <c r="A1" s="70" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="62"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="72"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="65" t="str">
+      <c r="A2" s="73" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="74"/>
+      <c r="C2" s="75" t="str">
         <f>'April '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="65"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="67" t="s">
+      <c r="D2" s="75"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="64"/>
+      <c r="G2" s="74"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="68" t="s">
+      <c r="I2" s="78" t="s">
         <v>185</v>
       </c>
-      <c r="J2" s="69"/>
+      <c r="J2" s="79"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="54" t="str">
+      <c r="B3" s="63"/>
+      <c r="C3" s="64" t="str">
         <f>'April '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="54"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="56" t="s">
+      <c r="D3" s="64"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="57"/>
+      <c r="G3" s="67"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="58">
+      <c r="I3" s="68">
         <v>2026</v>
       </c>
-      <c r="J3" s="59"/>
+      <c r="J3" s="69"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="70" t="str">
+      <c r="C4" s="52" t="str">
         <f>'April '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="70"/>
-      <c r="E4" s="71"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="53"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="72" t="str">
+      <c r="I4" s="54" t="str">
         <f>'April '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="73"/>
+      <c r="J4" s="55"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="74" t="str">
+      <c r="C5" s="56" t="str">
         <f>'April '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="74"/>
-      <c r="E5" s="75"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="57"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="76">
+      <c r="I5" s="58">
         <f>'April '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="77"/>
+      <c r="J5" s="59"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -10098,11 +10098,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="78" t="str">
+      <c r="I6" s="60" t="str">
         <f>'April '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="79"/>
+      <c r="J6" s="61"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -10926,11 +10926,6 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -10940,6 +10935,11 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -10970,104 +10970,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="60" t="s">
+      <c r="A1" s="70" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="62"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="72"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="65" t="str">
+      <c r="A2" s="73" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="74"/>
+      <c r="C2" s="75" t="str">
         <f>'Mai '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="65"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="67" t="s">
+      <c r="D2" s="75"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="64"/>
+      <c r="G2" s="74"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="68" t="s">
+      <c r="I2" s="78" t="s">
         <v>184</v>
       </c>
-      <c r="J2" s="69"/>
+      <c r="J2" s="79"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="54" t="str">
+      <c r="B3" s="63"/>
+      <c r="C3" s="64" t="str">
         <f>'Mai '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="54"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="56" t="s">
+      <c r="D3" s="64"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="57"/>
+      <c r="G3" s="67"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="58">
+      <c r="I3" s="68">
         <v>2026</v>
       </c>
-      <c r="J3" s="59"/>
+      <c r="J3" s="69"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="70" t="str">
+      <c r="C4" s="52" t="str">
         <f>'Mai '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="70"/>
-      <c r="E4" s="71"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="53"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="72" t="str">
+      <c r="I4" s="54" t="str">
         <f>'Mai '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="73"/>
+      <c r="J4" s="55"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="74" t="str">
+      <c r="C5" s="56" t="str">
         <f>'Mai '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="74"/>
-      <c r="E5" s="75"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="57"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="76">
+      <c r="I5" s="58">
         <f>'Mai '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="77"/>
+      <c r="J5" s="59"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -11080,11 +11080,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="78" t="str">
+      <c r="I6" s="60" t="str">
         <f>'Mai '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="79"/>
+      <c r="J6" s="61"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -11884,11 +11884,6 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -11898,6 +11893,11 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -11928,104 +11928,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="60" t="s">
+      <c r="A1" s="70" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="62"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="72"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="65" t="str">
+      <c r="A2" s="73" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="74"/>
+      <c r="C2" s="75" t="str">
         <f>'Juni '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="65"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="67" t="s">
+      <c r="D2" s="75"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="64"/>
+      <c r="G2" s="74"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="68" t="s">
+      <c r="I2" s="78" t="s">
         <v>247</v>
       </c>
-      <c r="J2" s="69"/>
+      <c r="J2" s="79"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="54" t="str">
+      <c r="B3" s="63"/>
+      <c r="C3" s="64" t="str">
         <f>'Juni '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="54"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="56" t="s">
+      <c r="D3" s="64"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="57"/>
+      <c r="G3" s="67"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="58">
+      <c r="I3" s="68">
         <v>2026</v>
       </c>
-      <c r="J3" s="59"/>
+      <c r="J3" s="69"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="70" t="str">
+      <c r="C4" s="52" t="str">
         <f>'Juni '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="70"/>
-      <c r="E4" s="71"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="53"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="72" t="str">
+      <c r="I4" s="54" t="str">
         <f>'Juni '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="73"/>
+      <c r="J4" s="55"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="74" t="str">
+      <c r="C5" s="56" t="str">
         <f>'Juni '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="74"/>
-      <c r="E5" s="75"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="57"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="76">
+      <c r="I5" s="58">
         <f>'Juni '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="77"/>
+      <c r="J5" s="59"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -12038,11 +12038,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="78" t="str">
+      <c r="I6" s="60" t="str">
         <f>'Juni '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="79"/>
+      <c r="J6" s="61"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -12087,16 +12087,20 @@
         <v>14</v>
       </c>
       <c r="C9" s="32"/>
-      <c r="D9" s="29"/>
-      <c r="E9" s="29"/>
+      <c r="D9" s="29">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="E9" s="29">
+        <v>0.79166666666666663</v>
+      </c>
       <c r="F9" s="29"/>
       <c r="G9" s="6">
         <f t="shared" ref="G9:G39" si="0">IF(OR(I9="U",I9="F",I9="K"),C9,E9-D9-F9)</f>
-        <v>0</v>
+        <v>0.20833333333333326</v>
       </c>
       <c r="H9" s="26">
         <f>IF(G9&gt;TIME(10,0,0),"10:00",G9)</f>
-        <v>0</v>
+        <v>0.20833333333333326</v>
       </c>
       <c r="I9" s="30"/>
       <c r="J9" s="31"/>
@@ -12131,16 +12135,20 @@
         <v>16</v>
       </c>
       <c r="C11" s="32"/>
-      <c r="D11" s="29"/>
-      <c r="E11" s="29"/>
+      <c r="D11" s="29">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="E11" s="29">
+        <v>0.70833333333333337</v>
+      </c>
       <c r="F11" s="29"/>
       <c r="G11" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="H11" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="I11" s="30"/>
       <c r="J11" s="31"/>
@@ -12198,16 +12206,20 @@
         <v>12</v>
       </c>
       <c r="C14" s="32"/>
-      <c r="D14" s="29"/>
-      <c r="E14" s="29"/>
+      <c r="D14" s="29">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="E14" s="29">
+        <v>0.70833333333333337</v>
+      </c>
       <c r="F14" s="29"/>
       <c r="G14" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="H14" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="I14" s="30"/>
       <c r="J14" s="31"/>
@@ -12242,16 +12254,20 @@
         <v>14</v>
       </c>
       <c r="C16" s="32"/>
-      <c r="D16" s="29"/>
-      <c r="E16" s="29"/>
+      <c r="D16" s="29">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="E16" s="29">
+        <v>0.79166666666666663</v>
+      </c>
       <c r="F16" s="29"/>
       <c r="G16" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.20833333333333326</v>
       </c>
       <c r="H16" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.20833333333333326</v>
       </c>
       <c r="I16" s="30"/>
       <c r="J16" s="31"/>
@@ -12396,16 +12412,20 @@
         <v>14</v>
       </c>
       <c r="C23" s="32"/>
-      <c r="D23" s="29"/>
-      <c r="E23" s="29"/>
+      <c r="D23" s="29">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="E23" s="29">
+        <v>0.79166666666666663</v>
+      </c>
       <c r="F23" s="29"/>
       <c r="G23" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.20833333333333326</v>
       </c>
       <c r="H23" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.20833333333333326</v>
       </c>
       <c r="I23" s="30"/>
       <c r="J23" s="31"/>
@@ -12440,16 +12460,20 @@
         <v>16</v>
       </c>
       <c r="C25" s="32"/>
-      <c r="D25" s="29"/>
-      <c r="E25" s="29"/>
+      <c r="D25" s="29">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="E25" s="29">
+        <v>0.70833333333333337</v>
+      </c>
       <c r="F25" s="29"/>
       <c r="G25" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="H25" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="I25" s="30"/>
       <c r="J25" s="31"/>
@@ -12554,7 +12578,7 @@
       <c r="E30" s="29"/>
       <c r="F30" s="29"/>
       <c r="G30" s="6">
-        <f t="shared" si="0"/>
+        <f>IF(OR(I30="U",I30="F",I30="K"),C30,E30-D30-F30)</f>
         <v>0</v>
       </c>
       <c r="H30" s="26">
@@ -12642,7 +12666,7 @@
       <c r="E34" s="29"/>
       <c r="F34" s="29"/>
       <c r="G34" s="6">
-        <f t="shared" si="0"/>
+        <f>IF(OR(I34="U",I34="F",I34="K"),C34,E34-D34-F34)</f>
         <v>0</v>
       </c>
       <c r="H34" s="26">
@@ -12704,16 +12728,20 @@
         <v>14</v>
       </c>
       <c r="C37" s="32"/>
-      <c r="D37" s="29"/>
-      <c r="E37" s="29"/>
+      <c r="D37" s="29">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="E37" s="29">
+        <v>0.79166666666666663</v>
+      </c>
       <c r="F37" s="29"/>
       <c r="G37" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.20833333333333326</v>
       </c>
       <c r="H37" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.20833333333333326</v>
       </c>
       <c r="I37" s="30"/>
       <c r="J37" s="31"/>
@@ -12748,16 +12776,20 @@
         <v>16</v>
       </c>
       <c r="C39" s="32"/>
-      <c r="D39" s="29"/>
-      <c r="E39" s="29"/>
+      <c r="D39" s="29">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="E39" s="29">
+        <v>0.70833333333333337</v>
+      </c>
       <c r="F39" s="29"/>
       <c r="G39" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="H39" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="I39" s="30"/>
       <c r="J39" s="31"/>
@@ -12788,7 +12820,7 @@
       <c r="F42" s="1"/>
       <c r="H42" s="34">
         <f>SUM(H9:H39)</f>
-        <v>0</v>
+        <v>1.333333333333333</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
@@ -12814,7 +12846,7 @@
       <c r="G44" s="15"/>
       <c r="H44" s="38">
         <f>H42-H41+H43</f>
-        <v>5.3333333333333321</v>
+        <v>6.6666666666666652</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
@@ -12832,11 +12864,6 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -12846,14 +12873,13 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
-  <dataValidations count="1">
-    <dataValidation type="time" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D9:E9" xr:uid="{00000000-0002-0000-0600-000000000000}">
-      <formula1>0.25</formula1>
-      <formula2>0.833333333333333</formula2>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.39370078740157483" bottom="0.39370078740157483" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
@@ -12876,104 +12902,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="60" t="s">
+      <c r="A1" s="70" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="62"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="72"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="65" t="str">
+      <c r="A2" s="73" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="74"/>
+      <c r="C2" s="75" t="str">
         <f>'Juli '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="65"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="67" t="s">
+      <c r="D2" s="75"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="64"/>
+      <c r="G2" s="74"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="68" t="s">
+      <c r="I2" s="78" t="s">
         <v>248</v>
       </c>
-      <c r="J2" s="69"/>
+      <c r="J2" s="79"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="54" t="str">
+      <c r="B3" s="63"/>
+      <c r="C3" s="64" t="str">
         <f>'Juli '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="54"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="56" t="s">
+      <c r="D3" s="64"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="57"/>
+      <c r="G3" s="67"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="58">
+      <c r="I3" s="68">
         <v>2026</v>
       </c>
-      <c r="J3" s="59"/>
+      <c r="J3" s="69"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="70" t="str">
+      <c r="C4" s="52" t="str">
         <f>'Juli '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="70"/>
-      <c r="E4" s="71"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="53"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="72" t="str">
+      <c r="I4" s="54" t="str">
         <f>'Juli '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="73"/>
+      <c r="J4" s="55"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="74" t="str">
+      <c r="C5" s="56" t="str">
         <f>'Juli '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="74"/>
-      <c r="E5" s="75"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="57"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="76">
+      <c r="I5" s="58">
         <f>'Juli '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="77"/>
+      <c r="J5" s="59"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -12986,11 +13012,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="78" t="str">
+      <c r="I6" s="60" t="str">
         <f>'Juli '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="79"/>
+      <c r="J6" s="61"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -13747,7 +13773,7 @@
       <c r="F43" s="1"/>
       <c r="H43" s="34">
         <f>'Juli '!H44</f>
-        <v>5.3333333333333321</v>
+        <v>6.6666666666666652</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -13762,7 +13788,7 @@
       <c r="G44" s="15"/>
       <c r="H44" s="38">
         <f>H42-H41+H43</f>
-        <v>5.3333333333333321</v>
+        <v>6.6666666666666652</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
@@ -13780,11 +13806,6 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -13794,6 +13815,11 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
@@ -13824,104 +13850,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="60" t="s">
+      <c r="A1" s="70" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="62"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="72"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="65" t="str">
+      <c r="A2" s="73" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="74"/>
+      <c r="C2" s="75" t="str">
         <f>'August '!C2:E2</f>
         <v>Hari Krishna</v>
       </c>
-      <c r="D2" s="65"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="67" t="s">
+      <c r="D2" s="75"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="64"/>
+      <c r="G2" s="74"/>
       <c r="H2" s="35"/>
-      <c r="I2" s="68" t="s">
+      <c r="I2" s="78" t="s">
         <v>280</v>
       </c>
-      <c r="J2" s="69"/>
+      <c r="J2" s="79"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="54" t="str">
+      <c r="B3" s="63"/>
+      <c r="C3" s="64" t="str">
         <f>'August '!C3:E3</f>
         <v>Mohan Raj</v>
       </c>
-      <c r="D3" s="54"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="56" t="s">
+      <c r="D3" s="64"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="57"/>
+      <c r="G3" s="67"/>
       <c r="H3" s="36"/>
-      <c r="I3" s="58">
+      <c r="I3" s="68">
         <v>2026</v>
       </c>
-      <c r="J3" s="59"/>
+      <c r="J3" s="69"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="70" t="str">
+      <c r="C4" s="52" t="str">
         <f>'August '!C4:E4</f>
         <v>07.11.2001</v>
       </c>
-      <c r="D4" s="70"/>
-      <c r="E4" s="71"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="53"/>
       <c r="F4" s="17" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="I4" s="72" t="str">
+      <c r="I4" s="54" t="str">
         <f>'August '!I4:J4</f>
         <v>01.03.2026</v>
       </c>
-      <c r="J4" s="73"/>
+      <c r="J4" s="55"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="74" t="str">
+      <c r="C5" s="56" t="str">
         <f>'August '!C5:E5</f>
         <v>Hochschule Bonn  Rhein Sieg</v>
       </c>
-      <c r="D5" s="74"/>
-      <c r="E5" s="75"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="57"/>
       <c r="F5" s="22" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
-      <c r="I5" s="76">
+      <c r="I5" s="58">
         <f>'August '!I5:J5</f>
         <v>8</v>
       </c>
-      <c r="J5" s="77"/>
+      <c r="J5" s="59"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
@@ -13934,11 +13960,11 @@
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="78" t="str">
+      <c r="I6" s="60" t="str">
         <f>'August '!I6:J6</f>
         <v>XX</v>
       </c>
-      <c r="J6" s="79"/>
+      <c r="J6" s="61"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="3"/>
@@ -14673,7 +14699,7 @@
       <c r="F42" s="1"/>
       <c r="H42" s="34">
         <f>'August '!H44</f>
-        <v>5.3333333333333321</v>
+        <v>6.6666666666666652</v>
       </c>
     </row>
     <row r="43" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -14688,7 +14714,7 @@
       <c r="G43" s="15"/>
       <c r="H43" s="38">
         <f>H41-H40+H42</f>
-        <v>5.3333333333333321</v>
+        <v>6.6666666666666652</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
@@ -14706,11 +14732,6 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="14">
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -14720,6 +14741,11 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:J2"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">

</xml_diff>